<commit_message>
state: heartbeat 2026-09-06 (no upstream changes)
</commit_message>
<xml_diff>
--- a/out/programs.xlsx
+++ b/out/programs.xlsx
@@ -7777,7 +7777,7 @@
       </c>
       <c r="J142" s="2" t="inlineStr">
         <is>
-          <t>2026-09-06T01:53:19+00:00</t>
+          <t>2026-09-06T01:58:05+00:00</t>
         </is>
       </c>
       <c r="K142" s="2" t="inlineStr"/>
@@ -7841,7 +7841,7 @@
       </c>
       <c r="J143" s="2" t="inlineStr">
         <is>
-          <t>2026-09-06T01:53:19+00:00</t>
+          <t>2026-09-06T01:58:05+00:00</t>
         </is>
       </c>
       <c r="K143" s="2" t="inlineStr">
@@ -7909,7 +7909,7 @@
       </c>
       <c r="J144" s="2" t="inlineStr">
         <is>
-          <t>2026-09-06T01:53:19+00:00</t>
+          <t>2026-09-06T01:58:05+00:00</t>
         </is>
       </c>
       <c r="K144" s="2" t="inlineStr"/>
@@ -7973,7 +7973,7 @@
       </c>
       <c r="J145" s="2" t="inlineStr">
         <is>
-          <t>2026-09-06T01:53:19+00:00</t>
+          <t>2026-09-06T01:58:05+00:00</t>
         </is>
       </c>
       <c r="K145" s="2" t="inlineStr"/>
@@ -8033,7 +8033,7 @@
       </c>
       <c r="J146" s="2" t="inlineStr">
         <is>
-          <t>2026-09-06T01:53:19+00:00</t>
+          <t>2026-09-06T01:58:05+00:00</t>
         </is>
       </c>
       <c r="K146" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
Correct the Harvard competition URL to huqt.com
The article's link (harvarduqt.com/competition) 301-redirects to
www.huqt.com/competition, which 404s -- the organisation rebranded to Harvard
Undergraduate Quantitative Traders. The live site is huqt.com: 200, 1,654 chars
over plain HTTP, no robots.txt, with an Apply link.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/out/programs.xlsx
+++ b/out/programs.xlsx
@@ -8334,7 +8334,7 @@
       </c>
       <c r="C152" s="3" t="inlineStr">
         <is>
-          <t>https://harvarduqt.com/</t>
+          <t>https://www.huqt.com/</t>
         </is>
       </c>
       <c r="D152" s="2" t="inlineStr">
@@ -8354,7 +8354,7 @@
       </c>
       <c r="G152" s="2" t="inlineStr">
         <is>
-          <t>Undergraduate intercollegiate trading competition. Christina Qi's 2026 quant competitions &amp; events list (LinkedIn Pulse), read 2026-09-06. NOTE: the article's link (harvarduqt.com/competition) is a 404; the root domain works. Class year and team format not published - verify before planning.</t>
+          <t>Undergraduate intercollegiate trading competition run by Harvard Undergraduate Quantitative Traders. The organisation rebranded: the article's link harvarduqt.com/competition 301-redirects to www.huqt.com/competition, which 404s. The live site is huqt.com and it has an Apply link. Christina Qi's 2026 quant competitions &amp; events list (LinkedIn Pulse), read 2026-09-06. Class year and team format not published - verify before planning.</t>
         </is>
       </c>
       <c r="H152" s="2" t="inlineStr">
@@ -13679,7 +13679,7 @@
       </c>
       <c r="J32" s="3" t="inlineStr">
         <is>
-          <t>https://harvarduqt.com/</t>
+          <t>https://www.huqt.com/</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix source_id generation and the Harvard source URL
The slug generator sliced at 40 characters regardless of word boundaries,
producing ids like harvard-undergraduate-trading-competitio and
open-source-quantitative-finance-confere. Truncation now happens on word
boundaries, with a numeric suffix on collision.

Renames the three affected ids and updates the programs.csv references. Also
repairs the Harvard source row's URL, which the previous commit missed because
it guessed the untruncated id.

Verified: no dangling source_id references from programs.csv.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/out/programs.xlsx
+++ b/out/programs.xlsx
@@ -8359,7 +8359,7 @@
       </c>
       <c r="H152" s="2" t="inlineStr">
         <is>
-          <t>harvard-undergraduate-trading-competitio</t>
+          <t>harvard-undergraduate-trading</t>
         </is>
       </c>
       <c r="I152" s="2" t="inlineStr">
@@ -8419,7 +8419,7 @@
       </c>
       <c r="H153" s="2" t="inlineStr">
         <is>
-          <t>stevens-high-frequency-trading-competiti</t>
+          <t>stevens-high-frequency-trading</t>
         </is>
       </c>
       <c r="I153" s="2" t="inlineStr">
@@ -8719,7 +8719,7 @@
       </c>
       <c r="H158" s="2" t="inlineStr">
         <is>
-          <t>open-source-quantitative-finance-confere</t>
+          <t>open-source-quantitative-finance</t>
         </is>
       </c>
       <c r="I158" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Add MIT Battlecode 2027 (Competition)
From https://battlecode.org/ - MIT's January AI/RTS competition, $20k+ prizes.

Placement:
- programs.csv: eligible=CHECK
- sources.csv: tier 3, page_text, render_js=false (probe: HTTP 200,
  1,627 chars plain HTML, no robots.txt). Home page carries the live
  season banner, so a text diff should catch the 2027 announcement.
- priority.csv: band C - open entry, participation is the only gate

Eligibility read from battlecode.org/about.html: "Anyone can write a bot,
create a team, and participate in scrimmage matches/rankings." US Qualifier
requires "teams ... entirely of US college students studying full-time" -
no MIT affiliation needed, unlike MIT Pokerbots. MIT Newbie and High School
tournaments are gated to MIT / high school students respectively.

Site still shows "Battlecode 2026 ended on January 31st, 2026!" as of
Sep 2026; no 2027 registration date posted yet.
</commit_message>
<xml_diff>
--- a/out/programs.xlsx
+++ b/out/programs.xlsx
@@ -13,9 +13,9 @@
     <sheet name="Priority" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Programs'!$A$1:$N$187</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Programs'!$A$1:$N$188</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Manual Watch'!$A$1:$G$32</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Priority'!$A$1:$J$35</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Priority'!$A$1:$J$36</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -514,7 +514,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N187"/>
+  <dimension ref="A1:N188"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -10365,8 +10365,68 @@
       </c>
       <c r="N187" s="2" t="inlineStr"/>
     </row>
+    <row r="188">
+      <c r="A188" s="2" t="inlineStr">
+        <is>
+          <t>Competition</t>
+        </is>
+      </c>
+      <c r="B188" s="2" t="inlineStr">
+        <is>
+          <t>MIT Battlecode 2027</t>
+        </is>
+      </c>
+      <c r="C188" s="3" t="inlineStr">
+        <is>
+          <t>https://battlecode.org/</t>
+        </is>
+      </c>
+      <c r="D188" s="2" t="inlineStr">
+        <is>
+          <t>Register ~early Jan 2027; season runs all January, ends ~Jan 31</t>
+        </is>
+      </c>
+      <c r="E188" s="2" t="inlineStr">
+        <is>
+          <t>Any undergrad year</t>
+        </is>
+      </c>
+      <c r="F188" s="5" t="inlineStr">
+        <is>
+          <t>CHECK</t>
+        </is>
+      </c>
+      <c r="G188" s="2" t="inlineStr">
+        <is>
+          <t>MIT's real-time strategy AI competition: you write an autonomous player that commands a robot army, then compete in scrimmages and bracketed tournaments over January. Over $20,000 in total prize money. Open beyond MIT - 'Anyone can write a bot, create a team, and participate in scrimmage matches/rankings.' Prize-tournament gates from the Full Eligibility Rules (battlecode.org/about.html): Sprint Tournaments - 'All teams are eligible.' US Qualifier - 'Teams must consist entirely of US college students studying full-time, or in a transition phase.' Final Tournament - 'Teams must have qualified via the US or International Qualifier.' MIT Newbie Tournament is MIT-only and High School Tournament is high-school-only, so neither applies. Unlike MIT Pokerbots, no MIT-affiliated teammate or MIT certificate is needed for the track you would enter. As of Sep 2026 the site still reads 'Battlecode 2026 ended on January 31st, 2026!' - no 2027 registration date posted yet, though the page already references Battlecode 2027 sponsorships. No team size limit, age limit, or citizenship rule beyond 'US college student' was stated on the pages read. Source: battlecode.org home page and about.html.</t>
+        </is>
+      </c>
+      <c r="H188" s="2" t="inlineStr">
+        <is>
+          <t>mit-battlecode-2027</t>
+        </is>
+      </c>
+      <c r="I188" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="J188" s="2" t="inlineStr"/>
+      <c r="K188" s="2" t="inlineStr"/>
+      <c r="L188" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="M188" s="2" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="N188" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N187"/>
+  <autoFilter ref="A1:N188"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C3" r:id="rId2"/>
@@ -10549,6 +10609,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C185" r:id="rId179"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C186" r:id="rId180"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C187" r:id="rId181"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C188" r:id="rId182"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -12070,7 +12131,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J35"/>
+  <dimension ref="A1:J36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -13833,8 +13894,58 @@
         </is>
       </c>
     </row>
+    <row r="36">
+      <c r="A36" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>C - open entry, participation is the only gate</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>MIT Battlecode 2027</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>Competition</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>Dec-Jan</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>Yes - plain HTML, pollable</t>
+        </is>
+      </c>
+      <c r="I36" s="2" t="inlineStr">
+        <is>
+          <t>No application and no MIT affiliation required - registering is the only gate, so probability is entirely up to you. The catch is timing: the whole season runs during January, which overlaps Stanford winter quarter rather than a break, so treat it as a time commitment decision and not a deadline to hit.</t>
+        </is>
+      </c>
+      <c r="J36" s="3" t="inlineStr">
+        <is>
+          <t>https://battlecode.org/</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J35"/>
+  <autoFilter ref="A1:J36"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J3" r:id="rId2"/>
@@ -13869,6 +13980,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J33" r:id="rId31"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J34" r:id="rId32"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J35" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J36" r:id="rId34"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
state: 2026-09-07 upstream changes detected
</commit_message>
<xml_diff>
--- a/out/programs.xlsx
+++ b/out/programs.xlsx
@@ -7777,7 +7777,7 @@
       </c>
       <c r="J142" s="2" t="inlineStr">
         <is>
-          <t>2026-09-06T01:58:05+00:00</t>
+          <t>2026-09-07T16:42:35+00:00</t>
         </is>
       </c>
       <c r="K142" s="2" t="inlineStr"/>
@@ -7841,12 +7841,12 @@
       </c>
       <c r="J143" s="2" t="inlineStr">
         <is>
-          <t>2026-09-06T01:58:05+00:00</t>
+          <t>2026-09-07T16:42:35+00:00</t>
         </is>
       </c>
       <c r="K143" s="2" t="inlineStr">
         <is>
-          <t>2026-09-06T01:51:27+00:00</t>
+          <t>2026-09-07T16:42:35+00:00</t>
         </is>
       </c>
       <c r="L143" s="2" t="inlineStr"/>
@@ -7857,7 +7857,7 @@
       </c>
       <c r="N143" s="2" t="inlineStr">
         <is>
-          <t>fe9b38f4209ae69a95e44eeb72d10595ac9a7e74cddb9920098ec2d3a8c05dd7</t>
+          <t>7fc143ceb98ac92883eb38c3019bae500ce8ff47db54414363f16c941d4eb4a0</t>
         </is>
       </c>
     </row>
@@ -7909,10 +7909,14 @@
       </c>
       <c r="J144" s="2" t="inlineStr">
         <is>
-          <t>2026-09-06T01:58:05+00:00</t>
-        </is>
-      </c>
-      <c r="K144" s="2" t="inlineStr"/>
+          <t>2026-09-07T16:42:35+00:00</t>
+        </is>
+      </c>
+      <c r="K144" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-07T16:42:35+00:00</t>
+        </is>
+      </c>
       <c r="L144" s="2" t="inlineStr"/>
       <c r="M144" s="2" t="inlineStr">
         <is>
@@ -7921,7 +7925,7 @@
       </c>
       <c r="N144" s="2" t="inlineStr">
         <is>
-          <t>fa7a84502fd1334e1fadab7feaee57579968a3d92af6b4c1c15b35f7810b3e4f</t>
+          <t>bca8dbaaeab258f990b8a51c80a016985792548fec897f4e2d7f54c215dc4867</t>
         </is>
       </c>
     </row>
@@ -7973,10 +7977,14 @@
       </c>
       <c r="J145" s="2" t="inlineStr">
         <is>
-          <t>2026-09-06T01:58:05+00:00</t>
-        </is>
-      </c>
-      <c r="K145" s="2" t="inlineStr"/>
+          <t>2026-09-07T16:42:35+00:00</t>
+        </is>
+      </c>
+      <c r="K145" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-07T16:42:35+00:00</t>
+        </is>
+      </c>
       <c r="L145" s="2" t="inlineStr"/>
       <c r="M145" s="2" t="inlineStr">
         <is>
@@ -7985,7 +7993,7 @@
       </c>
       <c r="N145" s="2" t="inlineStr">
         <is>
-          <t>c65c8da3aee53cb04884715418e7a0f636544ae6093687a1a0bc56ac58df227b</t>
+          <t>770702cb19ea8d996aed49851c54d2d3a4bc930f4c445257f7e6626ae1b193e8</t>
         </is>
       </c>
     </row>
@@ -8033,7 +8041,7 @@
       </c>
       <c r="J146" s="2" t="inlineStr">
         <is>
-          <t>2026-09-06T01:58:05+00:00</t>
+          <t>2026-09-07T16:42:35+00:00</t>
         </is>
       </c>
       <c r="K146" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
state: 2026-09-08 upstream changes detected
</commit_message>
<xml_diff>
--- a/out/programs.xlsx
+++ b/out/programs.xlsx
@@ -7777,7 +7777,7 @@
       </c>
       <c r="J142" s="2" t="inlineStr">
         <is>
-          <t>2026-09-07T18:18:32+00:00</t>
+          <t>2026-09-08T17:18:46+00:00</t>
         </is>
       </c>
       <c r="K142" s="2" t="inlineStr"/>
@@ -7841,12 +7841,12 @@
       </c>
       <c r="J143" s="2" t="inlineStr">
         <is>
-          <t>2026-09-07T18:18:32+00:00</t>
+          <t>2026-09-08T17:18:46+00:00</t>
         </is>
       </c>
       <c r="K143" s="2" t="inlineStr">
         <is>
-          <t>2026-09-07T18:18:32+00:00</t>
+          <t>2026-09-08T17:18:46+00:00</t>
         </is>
       </c>
       <c r="L143" s="2" t="inlineStr"/>
@@ -7857,7 +7857,7 @@
       </c>
       <c r="N143" s="2" t="inlineStr">
         <is>
-          <t>170fb42f2827b7d4363891200f13444b61566ea7aafc7957e1260e34de21d6c7</t>
+          <t>bb9048572570a77e92c2a6dccdc02b43c0c81ea68043dc3530cd9856848c9166</t>
         </is>
       </c>
     </row>
@@ -7909,7 +7909,7 @@
       </c>
       <c r="J144" s="2" t="inlineStr">
         <is>
-          <t>2026-09-07T18:18:32+00:00</t>
+          <t>2026-09-08T17:18:46+00:00</t>
         </is>
       </c>
       <c r="K144" s="2" t="inlineStr">
@@ -7977,7 +7977,7 @@
       </c>
       <c r="J145" s="2" t="inlineStr">
         <is>
-          <t>2026-09-07T18:18:32+00:00</t>
+          <t>2026-09-08T17:18:46+00:00</t>
         </is>
       </c>
       <c r="K145" s="2" t="inlineStr">
@@ -8041,7 +8041,7 @@
       </c>
       <c r="J146" s="2" t="inlineStr">
         <is>
-          <t>2026-09-07T18:18:32+00:00</t>
+          <t>2026-09-08T17:18:46+00:00</t>
         </is>
       </c>
       <c r="K146" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
state: heartbeat 2026-09-08 (no upstream changes)
</commit_message>
<xml_diff>
--- a/out/programs.xlsx
+++ b/out/programs.xlsx
@@ -7777,7 +7777,7 @@
       </c>
       <c r="J142" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08T17:18:46+00:00</t>
+          <t>2026-09-08T17:58:07+00:00</t>
         </is>
       </c>
       <c r="K142" s="2" t="inlineStr"/>
@@ -7841,7 +7841,7 @@
       </c>
       <c r="J143" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08T17:18:46+00:00</t>
+          <t>2026-09-08T17:58:07+00:00</t>
         </is>
       </c>
       <c r="K143" s="2" t="inlineStr">
@@ -7909,7 +7909,7 @@
       </c>
       <c r="J144" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08T17:18:46+00:00</t>
+          <t>2026-09-08T17:58:07+00:00</t>
         </is>
       </c>
       <c r="K144" s="2" t="inlineStr">
@@ -7977,7 +7977,7 @@
       </c>
       <c r="J145" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08T17:18:46+00:00</t>
+          <t>2026-09-08T17:58:07+00:00</t>
         </is>
       </c>
       <c r="K145" s="2" t="inlineStr">
@@ -8041,7 +8041,7 @@
       </c>
       <c r="J146" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08T17:18:46+00:00</t>
+          <t>2026-09-08T17:58:07+00:00</t>
         </is>
       </c>
       <c r="K146" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
state: 2026-09-09 upstream changes detected
</commit_message>
<xml_diff>
--- a/out/programs.xlsx
+++ b/out/programs.xlsx
@@ -7777,7 +7777,7 @@
       </c>
       <c r="J142" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08T19:47:04+00:00</t>
+          <t>2026-09-09T12:16:57+00:00</t>
         </is>
       </c>
       <c r="K142" s="2" t="inlineStr"/>
@@ -7841,12 +7841,12 @@
       </c>
       <c r="J143" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08T19:47:04+00:00</t>
+          <t>2026-09-09T12:16:57+00:00</t>
         </is>
       </c>
       <c r="K143" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08T17:18:46+00:00</t>
+          <t>2026-09-09T12:16:57+00:00</t>
         </is>
       </c>
       <c r="L143" s="2" t="inlineStr"/>
@@ -7857,7 +7857,7 @@
       </c>
       <c r="N143" s="2" t="inlineStr">
         <is>
-          <t>bb9048572570a77e92c2a6dccdc02b43c0c81ea68043dc3530cd9856848c9166</t>
+          <t>4ad63790373474da10fedb09d3783c590aa7ab5e6fda532a4eacd09613f2c726</t>
         </is>
       </c>
     </row>
@@ -7909,7 +7909,7 @@
       </c>
       <c r="J144" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08T19:47:04+00:00</t>
+          <t>2026-09-09T12:16:57+00:00</t>
         </is>
       </c>
       <c r="K144" s="2" t="inlineStr">
@@ -7977,7 +7977,7 @@
       </c>
       <c r="J145" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08T19:47:04+00:00</t>
+          <t>2026-09-09T12:16:57+00:00</t>
         </is>
       </c>
       <c r="K145" s="2" t="inlineStr">
@@ -8041,7 +8041,7 @@
       </c>
       <c r="J146" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08T19:47:04+00:00</t>
+          <t>2026-09-09T12:16:57+00:00</t>
         </is>
       </c>
       <c r="K146" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
state: 2026-09-10 upstream changes detected
</commit_message>
<xml_diff>
--- a/out/programs.xlsx
+++ b/out/programs.xlsx
@@ -7777,7 +7777,7 @@
       </c>
       <c r="J142" s="2" t="inlineStr">
         <is>
-          <t>2026-09-09T13:55:00+00:00</t>
+          <t>2026-09-10T12:11:00+00:00</t>
         </is>
       </c>
       <c r="K142" s="2" t="inlineStr"/>
@@ -7841,12 +7841,12 @@
       </c>
       <c r="J143" s="2" t="inlineStr">
         <is>
-          <t>2026-09-09T13:55:00+00:00</t>
+          <t>2026-09-10T12:11:00+00:00</t>
         </is>
       </c>
       <c r="K143" s="2" t="inlineStr">
         <is>
-          <t>2026-09-09T13:55:00+00:00</t>
+          <t>2026-09-10T12:11:00+00:00</t>
         </is>
       </c>
       <c r="L143" s="2" t="inlineStr"/>
@@ -7857,7 +7857,7 @@
       </c>
       <c r="N143" s="2" t="inlineStr">
         <is>
-          <t>e7b033ab2d8e9a42a94767e81740e1f38afa64a09cdd9df04cd9b1a539002b14</t>
+          <t>8f9ce6596381c64bdbb3b0e4aa51958ff46bb66b9a02cd900564a9de6eb834f9</t>
         </is>
       </c>
     </row>
@@ -7909,12 +7909,12 @@
       </c>
       <c r="J144" s="2" t="inlineStr">
         <is>
-          <t>2026-09-09T13:55:00+00:00</t>
+          <t>2026-09-10T12:11:00+00:00</t>
         </is>
       </c>
       <c r="K144" s="2" t="inlineStr">
         <is>
-          <t>2026-09-07T16:42:35+00:00</t>
+          <t>2026-09-10T12:11:00+00:00</t>
         </is>
       </c>
       <c r="L144" s="2" t="inlineStr"/>
@@ -7925,7 +7925,7 @@
       </c>
       <c r="N144" s="2" t="inlineStr">
         <is>
-          <t>bca8dbaaeab258f990b8a51c80a016985792548fec897f4e2d7f54c215dc4867</t>
+          <t>de71475901207962ca947d6f8f4202f2de5be54ec3c1592fc60d8211806d9b25</t>
         </is>
       </c>
     </row>
@@ -7977,7 +7977,7 @@
       </c>
       <c r="J145" s="2" t="inlineStr">
         <is>
-          <t>2026-09-09T13:55:00+00:00</t>
+          <t>2026-09-10T12:11:00+00:00</t>
         </is>
       </c>
       <c r="K145" s="2" t="inlineStr">
@@ -8041,7 +8041,7 @@
       </c>
       <c r="J146" s="2" t="inlineStr">
         <is>
-          <t>2026-09-09T13:55:00+00:00</t>
+          <t>2026-09-10T12:11:00+00:00</t>
         </is>
       </c>
       <c r="K146" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
state: heartbeat 2026-09-10 (no upstream changes)
</commit_message>
<xml_diff>
--- a/out/programs.xlsx
+++ b/out/programs.xlsx
@@ -7777,7 +7777,7 @@
       </c>
       <c r="J142" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10T12:11:00+00:00</t>
+          <t>2026-09-10T12:56:09+00:00</t>
         </is>
       </c>
       <c r="K142" s="2" t="inlineStr"/>
@@ -7841,7 +7841,7 @@
       </c>
       <c r="J143" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10T12:11:00+00:00</t>
+          <t>2026-09-10T12:56:09+00:00</t>
         </is>
       </c>
       <c r="K143" s="2" t="inlineStr">
@@ -7909,7 +7909,7 @@
       </c>
       <c r="J144" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10T12:11:00+00:00</t>
+          <t>2026-09-10T12:56:09+00:00</t>
         </is>
       </c>
       <c r="K144" s="2" t="inlineStr">
@@ -7977,7 +7977,7 @@
       </c>
       <c r="J145" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10T12:11:00+00:00</t>
+          <t>2026-09-10T12:56:09+00:00</t>
         </is>
       </c>
       <c r="K145" s="2" t="inlineStr">
@@ -8041,7 +8041,7 @@
       </c>
       <c r="J146" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10T12:11:00+00:00</t>
+          <t>2026-09-10T12:56:09+00:00</t>
         </is>
       </c>
       <c r="K146" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
state: 2026-09-11 upstream changes detected
</commit_message>
<xml_diff>
--- a/out/programs.xlsx
+++ b/out/programs.xlsx
@@ -7777,7 +7777,7 @@
       </c>
       <c r="J142" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10T13:49:13+00:00</t>
+          <t>2026-09-11T04:26:32+00:00</t>
         </is>
       </c>
       <c r="K142" s="2" t="inlineStr"/>
@@ -7841,12 +7841,12 @@
       </c>
       <c r="J143" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10T13:49:13+00:00</t>
+          <t>2026-09-11T04:26:32+00:00</t>
         </is>
       </c>
       <c r="K143" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10T13:49:13+00:00</t>
+          <t>2026-09-11T04:26:32+00:00</t>
         </is>
       </c>
       <c r="L143" s="2" t="inlineStr"/>
@@ -7857,7 +7857,7 @@
       </c>
       <c r="N143" s="2" t="inlineStr">
         <is>
-          <t>b5f26837f8aa9736997f79129117de740519cbc5848e258bf943fee05ef1e1c4</t>
+          <t>d2a1d6e73cc2a6e238e4d953033362e6346c235c2e5e77b389aca849d48fe70d</t>
         </is>
       </c>
     </row>
@@ -7909,7 +7909,7 @@
       </c>
       <c r="J144" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10T13:49:13+00:00</t>
+          <t>2026-09-11T04:26:32+00:00</t>
         </is>
       </c>
       <c r="K144" s="2" t="inlineStr">
@@ -7977,7 +7977,7 @@
       </c>
       <c r="J145" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10T13:49:13+00:00</t>
+          <t>2026-09-11T04:26:32+00:00</t>
         </is>
       </c>
       <c r="K145" s="2" t="inlineStr">
@@ -8041,7 +8041,7 @@
       </c>
       <c r="J146" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10T13:49:13+00:00</t>
+          <t>2026-09-11T04:26:32+00:00</t>
         </is>
       </c>
       <c r="K146" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
Write comments, docs and data notes as neutral engineering records
Comments, docstrings, docs, prompt text and CSV notes now state each decision
and its technical reason without attributing it to a person, quoting a
conversation, or addressing a particular reader. Gendered pronouns for the
user become the user, the student, or a restructured sentence, including in
the profile and prompts sent to the model, where every rule and fact is
unchanged. The workbooks are rebuilt from the edited CSVs.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/out/programs.xlsx
+++ b/out/programs.xlsx
@@ -857,7 +857,7 @@
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>Highest-signal single line you can add to a quant resume in year one. A high placement reportedly overrides GPA and non-target background. | Checked 2026-09-26: maa.org returns 403 to this client, so it cannot be watched; registration goes through Stanford's local supervisor, typically opening in September and closing before the early-December exam.</t>
+          <t>Among the highest-signal lines a first-year can add to a quant resume. A high placement reportedly overrides GPA and non-target background. | Checked 2026-09-26: maa.org returns 403 to this client, so it cannot be watched; registration goes through Stanford's local supervisor, typically opening in September and closing before the early-December exam.</t>
         </is>
       </c>
     </row>
@@ -2046,7 +2046,7 @@
       </c>
       <c r="G42" s="3" t="inlineStr">
         <is>
-          <t>Built for you: 5 weeks, discrete math, for students not yet in advanced courses. Apprentices often return to the full program. | Checked 2026-09-26: the URL is year-specific; REU2027/ returns 404 today and the parent page does not link it yet. Kept.</t>
+          <t>Built for first-years: 5 weeks, discrete math, for students not yet in advanced courses. Apprentices often return to the full program. | Checked 2026-09-26: the URL is year-specific; REU2027/ returns 404 today and the parent page does not link it yet. Kept.</t>
         </is>
       </c>
     </row>
@@ -2305,7 +2305,7 @@
       </c>
       <c r="G49" s="3" t="inlineStr">
         <is>
-          <t>THE right entry point for a freshman - a professor applies on your behalf. VPUE calls these 'good starting points'.</t>
+          <t>THE right entry point for a freshman - a professor applies on the student's behalf. VPUE calls these 'good starting points'.</t>
         </is>
       </c>
     </row>
@@ -3642,7 +3642,7 @@
       </c>
       <c r="G86" s="3" t="inlineStr">
         <is>
-          <t>Morgan Stanley's whole campus board, on Talentlink (morganstanley.tal.net) - 125 programmes, 31 in the United States, with business-unit facets including Quantitative Finance (8), Technology (12) and Investment Management (14). Found 2026-09-18 while resolving a pasted posting link. IMPORTANT, the obvious URL is the wrong one: www.morganstanley.com/careers/career-opportunities-search sits behind an Akamai WAF that resets the connection for paths.USER_AGENT and returns HTTP 200 with 134KB to a spoofed Chrome string - same machine, same IP, so the block is User-Agent based and it is the Citadel case, reachable only by misrepresenting the client. Do not re-point a source at it. Morgan Stanley's OTHER board, morganstanley.eightfold.ai, is reachable honestly via /api/pcsx/search but is deliberately NOT watched: it carries 1,327 corporate roles, caps page size at 10 (about 133 requests a day), and a query for 'Sophomore' or 'Freshman' returns zero - the campus programmes are not on it. Probed 2026-09-18: 9,660 chars of visible text, ratio 0.063, allowed by robots.txt (crawl-delay 10; the named-bot block covers ClaudeBot/GPTBot, not this tracker's own UA), no redirect. RETIRED 2026-09-21, asked for directly: this board is no longer watched. It failed on consecutive runs returning only ~350 characters because the Talentlink page renders its listings in JavaScript, and there is no honest route to the same content -- www.morganstanley.com refuses this tracker's User-Agent (the Citadel case) and morganstanley.eightfold.ai does not carry the campus programmes. source_id cleared, so this row is the owner's to check by hand.</t>
+          <t>Morgan Stanley's whole campus board, on Talentlink (morganstanley.tal.net) - 125 programmes, 31 in the United States, with business-unit facets including Quantitative Finance (8), Technology (12) and Investment Management (14). Found 2026-09-18 while resolving a pasted posting link. IMPORTANT, the obvious URL is the wrong one: www.morganstanley.com/careers/career-opportunities-search sits behind an Akamai WAF that resets the connection for paths.USER_AGENT and returns HTTP 200 with 134KB to a spoofed Chrome string - same machine, same IP, so the block is User-Agent based and it is the Citadel case, reachable only by misrepresenting the client. Do not re-point a source at it. Morgan Stanley's OTHER board, morganstanley.eightfold.ai, is reachable honestly via /api/pcsx/search but is deliberately NOT watched: it carries 1,327 corporate roles, caps page size at 10 (about 133 requests a day), and a query for 'Sophomore' or 'Freshman' returns zero - the campus programmes are not on it. Probed 2026-09-18: 9,660 chars of visible text, ratio 0.063, allowed by robots.txt (crawl-delay 10; the named-bot block covers ClaudeBot/GPTBot, not this tracker's own UA), no redirect. RETIRED 2026-09-21: this board is no longer watched. It failed on consecutive runs returning only ~350 characters because the Talentlink page renders its listings in JavaScript, and there is no honest route to the same content -- www.morganstanley.com refuses this tracker's User-Agent (the Citadel case) and morganstanley.eightfold.ai does not carry the campus programmes. source_id cleared, so this row is the owner's to check by hand.</t>
         </is>
       </c>
     </row>
@@ -3918,7 +3918,7 @@
       </c>
       <c r="G94" s="3" t="inlineStr">
         <is>
-          <t>40+ universities, RIT Market Simulator. Entry runs through Traders @ Stanford, not you directly.</t>
+          <t>40+ universities, RIT Market Simulator. Entry runs through Traders @ Stanford, not by individual application.</t>
         </is>
       </c>
     </row>
@@ -4066,7 +4066,7 @@
       </c>
       <c r="G98" s="3" t="inlineStr">
         <is>
-          <t>Open to RISING sophomores - you qualify spring 2027. Computational biochemistry entity, not the fund. | Checked 2026-09-26: now redirects to deshawresearch.com/joining.html, which mentions only summer internships. Kept: it may reopen.</t>
+          <t>Open to RISING sophomores - a first-year qualifies in spring 2027. Computational biochemistry entity, not the fund. | Checked 2026-09-26: now redirects to deshawresearch.com/joining.html, which mentions only summer internships. Kept: it may reopen.</t>
         </is>
       </c>
     </row>
@@ -4140,7 +4140,7 @@
       </c>
       <c r="G100" s="3" t="inlineStr">
         <is>
-          <t>Right programme, wrong year. The 2027 edition states applicants must 'graduate between December 2028 and June 2029', which is the class of 2029 - Jason is class of 2030, so he is a year early. The 2028 edition should target Dec 2029-Jun 2030 and is the one to apply to. Ten weeks from June 2027, New York, on the MSIM Tactical Value team; $36.06/hr. The 2027 deadline was Sep 25 2026 11:55pm ET with a HireVue due Sep 27. Added 2026-09-18 from a pasted link. The website column points at the campus board's keyword search rather than the requisition URL, which dies when the req closes; ?ftq=Sophomore returned exactly this one posting on 2026-09-18. Eligibility read from the reposted job description, not from morganstanley.com, which refuses this tracker's User-Agent - worth re-reading by hand before the 2028 cycle.</t>
+          <t>Right programme, wrong year. The 2027 edition states applicants must 'graduate between December 2028 and June 2029', which is the class of 2029 - a class of 2030 student is a year early. The 2028 edition should target Dec 2029-Jun 2030 and is the one to apply to. Ten weeks from June 2027, New York, on the MSIM Tactical Value team; $36.06/hr. The 2027 deadline was Sep 25 2026 11:55pm ET with a HireVue due Sep 27. Added 2026-09-18 from a pasted link. The website column points at the campus board's keyword search rather than the requisition URL, which dies when the req closes; ?ftq=Sophomore returned exactly this one posting on 2026-09-18. Eligibility read from the reposted job description, not from morganstanley.com, which refuses this tracker's User-Agent - worth re-reading by hand before the 2028 cycle.</t>
         </is>
       </c>
     </row>
@@ -4753,7 +4753,7 @@
       </c>
       <c r="G117" s="3" t="inlineStr">
         <is>
-          <t>You can attend; low relative value for you.</t>
+          <t>Open to attend; low relative value for a first-year.</t>
         </is>
       </c>
     </row>
@@ -5359,12 +5359,12 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>The site is pollable, but announcements go out on the club's Instagram and university listservs BEFORE the page updates. By the time a diff fires you may be late.</t>
+          <t>The site is pollable, but announcements go out on the club's Instagram and university listservs BEFORE the page updates. By the time a diff fires it may be late.</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>Club Instagram plus your Traders @ Stanford channels.</t>
+          <t>Club Instagram plus Traders @ Stanford channels.</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
@@ -5549,7 +5549,7 @@
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>Watch your Stanford email and the campus recruiting calendar.</t>
+          <t>Watch Stanford email and the campus recruiting calendar.</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
@@ -5623,7 +5623,7 @@
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>Join the mailing list and Slack/GroupMe in your first week of fall quarter.</t>
+          <t>Join the mailing list and Slack/GroupMe in the first week of fall quarter.</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
@@ -6528,7 +6528,7 @@
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>First-year only, and the single highest-value freshman program in quant. Rolling review: slots have reportedly filled by late October, so week-one applications face the most open seats. If you do one thing this fall, do this.</t>
+          <t>First-year only, and the single highest-value freshman program in quant. Rolling review: slots have reportedly filled by late October, so week-one applications face the most open seats. The single highest-value action of the fall.</t>
         </is>
       </c>
       <c r="J2" s="4" t="inlineStr">
@@ -6578,7 +6578,7 @@
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>Both are freshman-eligible and marked YES in your sheet, and they are SEPARATE applications - apply to both. Citadel's sites 403 every automated client, so this tool is structurally blind to them. This is the biggest gap in the system.</t>
+          <t>Both are freshman-eligible and marked YES in programs.csv, and they are SEPARATE applications - apply to both. Citadel's sites 403 every automated client, so this tool is structurally blind to them. This is the biggest gap in the system.</t>
         </is>
       </c>
       <c r="J3" s="4" t="inlineStr">
@@ -6628,7 +6628,7 @@
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>First-year only. Note your sheet's warning: the 'for Women' Discovery Days are a different, ineligible track - make sure you are looking at the general one.</t>
+          <t>First-year only. Note the warning in programs.csv: the 'for Women' Discovery Days are a different, ineligible track - the general one is the right track.</t>
         </is>
       </c>
       <c r="J4" s="4" t="inlineStr">
@@ -6828,7 +6828,7 @@
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>No class-year gate - open to any enrolled bachelor's student, which is unusual and makes it one of the few research-track roles a first-year can actually win. Fixed deadline, so put it in your calendar now.</t>
+          <t>No class-year gate - open to any enrolled bachelor's student, which is unusual and makes it one of the few research-track roles a first-year can actually win. Fixed deadline, so it belongs in a calendar now.</t>
         </is>
       </c>
       <c r="J8" s="4" t="inlineStr">
@@ -6878,7 +6878,7 @@
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>Early-undergrad program, marked YES. Same Cloudflare block as the rest of Citadel - you must check this one by hand.</t>
+          <t>Early-undergrad program, marked YES. Same Cloudflare block as the rest of Citadel - this one must be checked by hand.</t>
         </is>
       </c>
       <c r="J9" s="4" t="inlineStr">
@@ -6928,7 +6928,7 @@
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>First- and second-year eligible. HRT's student page is plain HTML and this tool watches it well, so a state change here should reach you.</t>
+          <t>First- and second-year eligible. HRT's student page is plain HTML and this tool watches it well, so a state change here should reach the digest.</t>
         </is>
       </c>
       <c r="J10" s="4" t="inlineStr">
@@ -7078,7 +7078,7 @@
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>Explicitly NO class-year requirement, paid, at a national lab - one of the strongest research options genuinely open to a first-year. Not mentioned in any repo this tool tracks, so it is on you until phase 3.</t>
+          <t>Explicitly NO class-year requirement, paid, at a national lab - one of the strongest research options genuinely open to a first-year. Not mentioned in any repo this tool tracks, so it is a manual check until phase 3.</t>
         </is>
       </c>
       <c r="J13" s="4" t="inlineStr">
@@ -7128,7 +7128,7 @@
       </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>Paid CS research with Stanford faculty, open to any Stanford undergrad. Competing against Stanford students only, which is a far smaller pool than any national program. The site is fully client-rendered and appears in zero tracked repos - check it yourself in January.</t>
+          <t>Paid CS research with Stanford faculty, open to any Stanford undergrad. Competing against Stanford students only, which is a far smaller pool than any national program. The site is fully client-rendered and appears in zero tracked repos - check it by hand in January.</t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr">
@@ -7228,7 +7228,7 @@
       </c>
       <c r="I16" s="3" t="inlineStr">
         <is>
-          <t>Funding, not a competition - if you have a faculty sponsor and a coherent plan, these are close to a formality. The quarterly Small Grants are the easiest money on this entire sheet. Note the Major Grant mentor letter is due Mar 8.</t>
+          <t>Funding, not a competition - given a faculty sponsor and a coherent plan, these are close to a formality. The quarterly Small Grants are the easiest money on this entire sheet. Note the Major Grant mentor letter is due Mar 8.</t>
         </is>
       </c>
       <c r="J16" s="4" t="inlineStr">
@@ -7328,7 +7328,7 @@
       </c>
       <c r="I18" s="3" t="inlineStr">
         <is>
-          <t>Paid, on-campus, repeatable, and a genuine credential on a quant/SWE resume. Available as soon as you have taken 106A/B - apply the very first quarter you are eligible.</t>
+          <t>Paid, on-campus, repeatable, and a genuine credential on a quant/SWE resume. Available after 106A/B - apply in the first eligible quarter.</t>
         </is>
       </c>
       <c r="J18" s="4" t="inlineStr">
@@ -7428,7 +7428,7 @@
       </c>
       <c r="I20" s="3" t="inlineStr">
         <is>
-          <t>Not an application, and it is the gateway to several competitions that only accept university-sponsored teams. It is also where you will hear about Cornell CTC and UChicago UTC before any website says anything.</t>
+          <t>Not an application, and it is the gateway to several competitions that only accept university-sponsored teams. It is also where announcements come for Cornell CTC and UChicago UTC before any website says anything.</t>
         </is>
       </c>
       <c r="J20" s="3" t="inlineStr"/>
@@ -7474,7 +7474,7 @@
       </c>
       <c r="I21" s="3" t="inlineStr">
         <is>
-          <t>No gate at all. A submitted solution is a real touchpoint with the firm you most want, every single month, for the price of an evening.</t>
+          <t>No gate at all. A submitted solution is a real touchpoint with the firm, every single month, for the price of an evening.</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr">
@@ -7524,7 +7524,7 @@
       </c>
       <c r="I22" s="3" t="inlineStr">
         <is>
-          <t>Open entry, no class-year or identity gate. A leaderboard placing is portable, verifiable evidence - and the Optiver and Jane Street sponsored competitions read as quant credentials specifically. Your sheet already flags these as a legitimate substitute if ETC never materialises.</t>
+          <t>Open entry, no class-year or identity gate. A leaderboard placing is portable, verifiable evidence - and the Optiver and Jane Street sponsored competitions read as quant credentials specifically. programs.csv already flags these as a legitimate substitute if ETC never materialises.</t>
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr">
@@ -7574,7 +7574,7 @@
       </c>
       <c r="I23" s="3" t="inlineStr">
         <is>
-          <t>Open to anyone 18+ and enrolled. Algorithmic trading against thousands of teams - high signal, zero admission risk. Appears in no tracked repo, so diarise mid-March yourself.</t>
+          <t>Open to anyone 18+ and enrolled. Algorithmic trading against thousands of teams - high signal, zero admission risk. Appears in no tracked repo, so it needs a mid-March calendar entry.</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
@@ -7624,7 +7624,7 @@
       </c>
       <c r="I24" s="3" t="inlineStr">
         <is>
-          <t>Team registration rather than individual selection, so getting in is mostly about hearing in time. That is exactly what this tool cannot do for you: announcements go out on Instagram and listservs first. Cornell CTC in early fall is the most time-critical item on the whole sheet.</t>
+          <t>Team registration rather than individual selection, so getting in is mostly about hearing in time. That is exactly what this tool cannot do: announcements go out on Instagram and listservs first. Cornell CTC in early fall is the most time-critical item on the whole sheet.</t>
         </is>
       </c>
       <c r="J24" s="4" t="inlineStr">
@@ -7724,7 +7724,7 @@
       </c>
       <c r="I26" s="3" t="inlineStr">
         <is>
-          <t>Quarterly, so you get four attempts a year and missing one costs almost nothing. Good backtesting practice that produces something concrete to talk about.</t>
+          <t>Quarterly, so there are four attempts a year and missing one costs almost nothing. Good backtesting practice that produces something concrete to talk about.</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">
@@ -7974,7 +7974,7 @@
       </c>
       <c r="I31" s="3" t="inlineStr">
         <is>
-          <t>No deadline, no selection, no rejection. Worth doing once each in a quiet week purely so the firm's name appears on your resume with something real behind it. Do not spend fall on these at the expense of rank 1-12.</t>
+          <t>No deadline, no selection, no rejection. Worth doing once each in a quiet week purely so the firm's name appears on a resume with something real behind it. Do not spend fall on these at the expense of rank 1-12.</t>
         </is>
       </c>
       <c r="J31" s="4" t="inlineStr">
@@ -8224,7 +8224,7 @@
       </c>
       <c r="I36" s="3" t="inlineStr">
         <is>
-          <t>No application and no MIT affiliation required - registering is the only gate, so probability is entirely up to you. The catch is timing: the whole season runs during January, which overlaps Stanford winter quarter rather than a break, so treat it as a time commitment decision and not a deadline to hit.</t>
+          <t>No application and no MIT affiliation required - registering is the only gate, so the odds rest entirely on the applicant. The catch is timing: the whole season runs during January, which overlaps Stanford winter quarter rather than a break, so treat it as a time commitment decision and not a deadline to hit.</t>
         </is>
       </c>
       <c r="J36" s="4" t="inlineStr">
@@ -8274,7 +8274,7 @@
       </c>
       <c r="I37" s="3" t="inlineStr">
         <is>
-          <t>A sophomore-specific summer analyst seat at a major firm, which is a narrower and less contested door than the junior programme. He is one year early for the 2027 cycle; the 2028 cycle is his first shot and it closed in late September for 2027, so the window opens earlier than most people expect.</t>
+          <t>A sophomore-specific summer analyst seat at a major firm, which is a narrower and less contested door than the junior programme. A class of 2030 student is one year early for the 2027 cycle; the 2028 cycle is the first realistic one, and it closed in late September for 2027, so the window opens earlier than most people expect.</t>
         </is>
       </c>
       <c r="J37" s="4" t="inlineStr">
@@ -9205,7 +9205,7 @@
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>THE one for you next year - Nexus is the all-students track. 3 days NYC, $1,500 stipend, travel + lodging. | Checked 2026-09-26: campus.deshaw.com/fellowships now redirects to the campus root, which mentions no fellowships. Kept; the root is watched as deshaw-campus.</t>
+          <t>THE one for a first-year to target the following year - Nexus is the all-students track. 3 days NYC, $1,500 stipend, travel + lodging. | Checked 2026-09-26: campus.deshaw.com/fellowships now redirects to the campus root, which mentions no fellowships. Kept; the root is watched as deshaw-campus.</t>
         </is>
       </c>
     </row>
@@ -10185,7 +10185,7 @@
       </c>
       <c r="F47" s="3" t="inlineStr">
         <is>
-          <t>Largest intercollegiate competition, $20,000+. NOT the same as Pokerbots - this one IS open to you.</t>
+          <t>Largest intercollegiate competition, $20,000+. NOT the same as Pokerbots - this one IS open to first-years.</t>
         </is>
       </c>
     </row>
@@ -11233,7 +11233,7 @@
       </c>
       <c r="F80" s="3" t="inlineStr">
         <is>
-          <t>Geographic exclusion - you are US-based.</t>
+          <t>Geographic exclusion - excludes US-based students.</t>
         </is>
       </c>
     </row>
@@ -11325,7 +11325,7 @@
       </c>
       <c r="F83" s="3" t="inlineStr">
         <is>
-          <t>That is a junior-year window. Not you.</t>
+          <t>That is a junior-year window; a first-year does not qualify.</t>
         </is>
       </c>
     </row>
@@ -11669,7 +11669,7 @@
       </c>
       <c r="F94" s="3" t="inlineStr">
         <is>
-          <t>Highest pay in the industry, but you are too early.</t>
+          <t>Highest pay in the industry, but a first-year is too early.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
sources: watch Built In's internship front pages
Three page_text watchers on builtin.com/jobs/<category>/internship for
software engineering, data and analytics, and finance. Each is a what's-new
feed of the newest ~14-25 cards; the site rate-limits after about 70 requests,
so it is not crawled in full.

Built In prints a bare relative age before each card's Saved control
("11 Hours Ago Saved", "Reposted Yesterday Saved"), which would rewrite the
page snapshot every day. parse_page now replaces it with a placeholder,
anchored on that control so prose containing "yesterday" is untouched.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/out/programs.xlsx
+++ b/out/programs.xlsx
@@ -17,7 +17,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Check By Hand'!$A$1:$G$201</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Manual Watch'!$A$1:$G$35</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Priority'!$A$1:$J$37</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Left Out'!$A$1:$F$120</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Left Out'!$A$1:$F$123</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -11688,7 +11688,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F120"/>
+  <dimension ref="A1:F123"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -11990,108 +11990,108 @@
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>Already watched by caltech-surf</t>
+          <t>Already watched by builtin-data-analytics</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Caltech SURF</t>
+          <t>Built In data and analytics internships</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>Research / math</t>
-        </is>
-      </c>
-      <c r="D10" s="5" t="inlineStr">
-        <is>
-          <t>CHECK</t>
+          <t>Tracker / resource</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>USE</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>https://sfp.caltech.edu/undergraduate-research/programs/surf/application_information</t>
+          <t>https://builtin.com/jobs/data-analytics/internship</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>Summer Undergraduate Research Fellowship. Open to non-Caltech students, though the page notes they may find it harder to secure a mentor.</t>
+          <t>Front page of Built In's data and analytics internship listings, newest first (about 14-25 cards), watched as a what's-new feed rather than a full list: the site returns HTTP 429 after roughly 70 requests at one a second, so a full crawl is not polite. Measured 2026-10-01 across a deeper crawl: most of its in-field internships were not on Simplify, but many are generic internships at large non-technology employers.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>Already watched by capitalone-early-career</t>
+          <t>Already watched by builtin-dev-engineering</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Capital One Analyst / Tech / Product Summits</t>
+          <t>Built In software engineering internships</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>Tech internship</t>
-        </is>
-      </c>
-      <c r="D11" s="5" t="inlineStr">
-        <is>
-          <t>CHECK</t>
+          <t>Tracker / resource</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>USE</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>https://www.capitalonecareers.com/get-ahead-with-early-career-programs-for-students</t>
+          <t>https://builtin.com/jobs/dev-engineering/internship</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>Verified 2026-09-26: Analyst Summit 'First-year students or sophomores pursuing a quantitative/STEM major'; Tech Summit 'Sophomores with beginner coding experience'. Separate from the Capital One TEIP row.</t>
+          <t>Front page of Built In's software engineering internship listings, newest first (about 14-25 cards), watched as a what's-new feed rather than a full list: the site returns HTTP 429 after roughly 70 requests at one a second, so a full crawl is not polite. Measured 2026-10-01 across a deeper crawl: most of its in-field internships were not on Simplify, but many are generic internships at large non-technology employers.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>Already watched by citi-pre-internships</t>
+          <t>Already watched by builtin-finance</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Citi Freshman Discovery</t>
+          <t>Built In finance internships</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>Conference / other</t>
+          <t>Tracker / resource</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>USE</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>https://jobs.citi.com/early-career-programs-pre-internships</t>
+          <t>https://builtin.com/jobs/finance/internship</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>Verified 2026-09-30: 'All first-year students in a four-year bachelor's degree program from a US accredited institution, regardless of major.' 3-day virtual introduction to financial services.</t>
+          <t>Front page of Built In's finance internship listings, newest first (about 14-25 cards), watched as a what's-new feed rather than a full list: the site returns HTTP 429 after roughly 70 requests at one a second, so a full crawl is not polite. Measured 2026-10-01 across a deeper crawl: most of its in-field internships were not on Simplify, but many are generic internships at large non-technology employers.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Already watched by cmu-riss</t>
+          <t>Already watched by caltech-surf</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>CMU Robotics Institute Summer Scholars (RISS)</t>
+          <t>Caltech SURF</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
@@ -12106,29 +12106,29 @@
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>https://riss.ri.cmu.edu/</t>
+          <t>https://sfp.caltech.edu/undergraduate-research/programs/surf/application_information</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>11-week summer research immersion for undergraduates at CMU's Robotics Institute.</t>
+          <t>Summer Undergraduate Research Fellowship. Open to non-Caltech students, though the page notes they may find it harder to secure a mentor.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>Already watched by comap-mcm</t>
+          <t>Already watched by capitalone-early-career</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>COMAP MCM/ICM</t>
+          <t>Capital One Analyst / Tech / Product Summits</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>Competition</t>
+          <t>Tech internship</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
@@ -12138,29 +12138,29 @@
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>https://www.contest.comap.com/undergraduate/contests/</t>
+          <t>https://www.capitalonecareers.com/get-ahead-with-early-career-programs-for-students</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>Verified 2026-09-26: 'high school students and college undergraduates'; 2027 contest 28 Jan - 1 Feb.</t>
+          <t>Verified 2026-09-26: Analyst Summit 'First-year students or sophomores pursuing a quantitative/STEM major'; Tech Summit 'Sophomores with beginner coding experience'. Separate from the Capital One TEIP row.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>Already watched by cornell-trading-competition</t>
+          <t>Already watched by citi-pre-internships</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Cornell Trading Competition</t>
+          <t>Citi Freshman Discovery</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>Competition</t>
+          <t>Conference / other</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
@@ -12170,24 +12170,24 @@
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>https://cornellquantfund.org/competition</t>
+          <t>https://jobs.citi.com/early-career-programs-pre-internships</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>Teams of 4, NO EXPERIENCE NECESSARY, $10k+ prizes, Cornell Tech NYC. Case packets released 2 weeks early.</t>
+          <t>Verified 2026-09-30: 'All first-year students in a four-year bachelor's degree program from a US accredited institution, regardless of major.' 3-day virtual introduction to financial services.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>Already watched by cra-dreu</t>
+          <t>Already watched by cmu-riss</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>CRA DREU</t>
+          <t>CMU Robotics Institute Summer Scholars (RISS)</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
@@ -12202,61 +12202,61 @@
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>https://cra.org/cra-wp/dreu/</t>
+          <t>https://riss.ri.cmu.edu/</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>Verified 2026-09-26: 'High school graduates who have been accepted ... are also eligible'; priority to CS majors. Large page (94K chars).</t>
+          <t>11-week summer research immersion for undergraduates at CMU's Robotics Institute.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>Already watched by cs-social-good-fellowships</t>
+          <t>Already watched by comap-mcm</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>CS+Social Good Summer Fellowships</t>
+          <t>COMAP MCM/ICM</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>Stanford-only</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="inlineStr">
-        <is>
-          <t>YES</t>
+          <t>Competition</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>CHECK</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>https://cardinalservice.stanford.edu/opportunities/cssocial-good-summer-fellowships</t>
+          <t>https://www.contest.comap.com/undergraduate/contests/</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>Verified 2026-09-30 from the 2026 SOLO listing: 'enrolled as a first-year, sophomore, or junior ... must have completed CS 106B by the end of Spring Quarter.' $7,000 base stipend, full-time summer with a tech-for-good partner. Cardinal Quarter.</t>
+          <t>Verified 2026-09-26: 'high school students and college undergraduates'; 2027 contest 28 Jan - 1 Feb.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>Already watched by curis</t>
+          <t>Already watched by cornell-trading-competition</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>Stanford CURIS</t>
+          <t>Cornell Trading Competition</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>Stanford-only</t>
+          <t>Competition</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
@@ -12266,189 +12266,189 @@
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>https://curis.stanford.edu/</t>
+          <t>https://cornellquantfund.org/competition</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>CS dept paid summer research. Project list posted late Jan. Also lists year-round projects for units or hourly pay. | Checked 2026-09-26: now watched with render_js - the page is client-rendered and yields 1,264 chars in the browser.</t>
+          <t>Teams of 4, NO EXPERIENCE NECESSARY, $10k+ prizes, Cornell Tech NYC. Case packets released 2 weeks early.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>Already watched by datasurf</t>
+          <t>Already watched by cra-dreu</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>Stanford DataSURF (formerly SURP-Stats)</t>
+          <t>CRA DREU</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>Stanford-only</t>
-        </is>
-      </c>
-      <c r="D19" s="2" t="inlineStr">
-        <is>
-          <t>YES</t>
+          <t>Research / math</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>CHECK</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>https://datasciencemajor.stanford.edu/research-impact/data-science-undergraduate-research-focus</t>
+          <t>https://cra.org/cra-wp/dreu/</t>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>Verified 2026-09-30: 'Stanford undergraduate students from any department who meet the prerequisites are encouraged to apply' (examples: STATS 60, MATH 51-53, CS 106A/B). 10 weeks, $8,500 stipend plus need-based supplement.</t>
+          <t>Verified 2026-09-26: 'High school graduates who have been accepted ... are also eligible'; priority to CS majors. Large page (94K chars).</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>Already watched by deshaw-campus</t>
+          <t>Already watched by cs-social-good-fellowships</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>D. E. Shaw Nexus Fellowship</t>
+          <t>CS+Social Good Summer Fellowships</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>Quant firm program</t>
-        </is>
-      </c>
-      <c r="D20" s="6" t="inlineStr">
-        <is>
-          <t>LATER</t>
+          <t>Stanford-only</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>https://campus.deshaw.com/fellowships</t>
+          <t>https://cardinalservice.stanford.edu/opportunities/cssocial-good-summer-fellowships</t>
         </is>
       </c>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t>THE one for a first-year to target the following year - Nexus is the all-students track. 3 days NYC, $1,500 stipend, travel + lodging. | Checked 2026-09-26: campus.deshaw.com/fellowships now redirects to the campus root, which mentions no fellowships. Kept; the root is watched as deshaw-campus.</t>
+          <t>Verified 2026-09-30 from the 2026 SOLO listing: 'enrolled as a first-year, sophomore, or junior ... must have completed CS 106B by the end of Spring Quarter.' $7,000 base stipend, full-time summer with a tech-for-good partner. Cardinal Quarter.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>Already watched by deshaw-campus</t>
+          <t>Already watched by curis</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>D. E. Shaw campus site</t>
+          <t>Stanford CURIS</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>Quant firm program</t>
-        </is>
-      </c>
-      <c r="D21" s="5" t="inlineStr">
-        <is>
-          <t>CHECK</t>
+          <t>Stanford-only</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t>https://campus.deshaw.com/</t>
+          <t>https://curis.stanford.edu/</t>
         </is>
       </c>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>Verified 2026-09-26: internships for 'undergraduate and graduate students'. The fellowship rows' campus.deshaw.com/fellowships URL now redirects here; this page is watched so a returning fellowship shows up.</t>
+          <t>CS dept paid summer research. Project list posted late Jan. Also lists year-round projects for units or hourly pay. | Checked 2026-09-26: now watched with render_js - the page is client-rendered and yields 1,264 chars in the browser.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>Already watched by dimacs-reu</t>
+          <t>Already watched by datasurf</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>DIMACS REU</t>
+          <t>Stanford DataSURF (formerly SURP-Stats)</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>Research / math</t>
-        </is>
-      </c>
-      <c r="D22" s="6" t="inlineStr">
-        <is>
-          <t>LATER</t>
+          <t>Stanford-only</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>https://dimacs.rutgers.edu/reu-main</t>
+          <t>https://datasciencemajor.stanford.edu/research-impact/data-science-undergraduate-research-focus</t>
         </is>
       </c>
       <c r="F22" s="3" t="inlineStr">
         <is>
-          <t>Verified 2026-09-26: 'We do not usually admit freshmen' - watch for sophomore year.</t>
+          <t>Verified 2026-09-30: 'Stanford undergraduate students from any department who meet the prerequisites are encouraged to apply' (examples: STATS 60, MATH 51-53, CS 106A/B). 10 weeks, $8,500 stipend plus need-based supplement.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>Already watched by dukequant-competition</t>
+          <t>Already watched by deshaw-campus</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>Duke FinTech Trading Competition</t>
+          <t>D. E. Shaw Nexus Fellowship</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>Competition</t>
-        </is>
-      </c>
-      <c r="D23" s="2" t="inlineStr">
-        <is>
-          <t>YES</t>
+          <t>Quant firm program</t>
+        </is>
+      </c>
+      <c r="D23" s="6" t="inlineStr">
+        <is>
+          <t>LATER</t>
         </is>
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t>https://www.duke.edu/</t>
+          <t>https://campus.deshaw.com/fellowships</t>
         </is>
       </c>
       <c r="F23" s="3" t="inlineStr">
         <is>
-          <t>3 months, paper trading, bracket format. Sponsors include Schonfeld. Lowest time commitment. | Checked 2026-09-26: Duke Quantitative Finance's competition page is dukequant.com/general-7 (watched with render_js); not yet confirmed to be the same event this row names. The listed duke.edu is kept.</t>
+          <t>THE one for a first-year to target the following year - Nexus is the all-students track. 3 days NYC, $1,500 stipend, travel + lodging. | Checked 2026-09-26: campus.deshaw.com/fellowships now redirects to the campus root, which mentions no fellowships. Kept; the root is watched as deshaw-campus.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>Already watched by evercore-campus</t>
+          <t>Already watched by deshaw-campus</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>Evercore student events</t>
+          <t>D. E. Shaw campus site</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>Conference / other</t>
+          <t>Quant firm program</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
@@ -12458,29 +12458,29 @@
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>https://evercore.tal.net/vx/mobile-0/candidate/jobboard/vacancy/2/feed</t>
+          <t>https://campus.deshaw.com/</t>
         </is>
       </c>
       <c r="F24" s="3" t="inlineStr">
         <is>
-          <t>Verified 2026-09-26: Oleeo Atom feed, 39 entries; vacancy/1/feed has 29 more. Some events are restricted-audience per the Simplify blog.</t>
+          <t>Verified 2026-09-26: internships for 'undergraduate and graduate students'. The fellowship rows' campus.deshaw.com/fellowships URL now redirects here; this page is watched so a returning fellowship shows up.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>Already watched by futureforce-launchpad</t>
+          <t>Already watched by dimacs-reu</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>Salesforce Futureforce Tech Launchpad (CodePath)</t>
+          <t>DIMACS REU</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>Tech internship</t>
+          <t>Research / math</t>
         </is>
       </c>
       <c r="D25" s="6" t="inlineStr">
@@ -12490,24 +12490,24 @@
       </c>
       <c r="E25" s="4" t="inlineStr">
         <is>
-          <t>https://info.codepath.org/futureforce-tech-launchpad</t>
+          <t>https://dimacs.rutgers.edu/reu-main</t>
         </is>
       </c>
       <c r="F25" s="3" t="inlineStr">
         <is>
-          <t>Verified 2026-09-26: 'Students who will complete their sophomore year in Spring 2026' - so summer 2028 for a class of 2030.</t>
+          <t>Verified 2026-09-26: 'We do not usually admit freshmen' - watch for sophomore year.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>Already watched by harvard-undergraduate-trading</t>
+          <t>Already watched by dukequant-competition</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>Harvard Undergraduate Trading Competition</t>
+          <t>Duke FinTech Trading Competition</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
@@ -12515,31 +12515,31 @@
           <t>Competition</t>
         </is>
       </c>
-      <c r="D26" s="5" t="inlineStr">
-        <is>
-          <t>CHECK</t>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>https://www.huqt.com/</t>
+          <t>https://www.duke.edu/</t>
         </is>
       </c>
       <c r="F26" s="3" t="inlineStr">
         <is>
-          <t>Undergraduate intercollegiate trading competition run by Harvard Undergraduate Quantitative Traders. The organisation rebranded: the article's link harvarduqt.com/competition 301-redirects to www.huqt.com/competition, which 404s. The live site is huqt.com and it has an Apply link. Christina Qi's 2026 quant competitions &amp; events list (LinkedIn Pulse), read 2026-09-06. Class year and team format not published - verify before planning.</t>
+          <t>3 months, paper trading, bracket format. Sponsors include Schonfeld. Lowest time commitment. | Checked 2026-09-26: Duke Quantitative Finance's competition page is dukequant.com/general-7 (watched with render_js); not yet confirmed to be the same event this row names. The listed duke.edu is kept.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>Already watched by hedgewest-sf-meetup-series</t>
+          <t>Already watched by evercore-campus</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>HedgeWest SF Meetup Series</t>
+          <t>Evercore student events</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
@@ -12554,61 +12554,61 @@
       </c>
       <c r="E27" s="4" t="inlineStr">
         <is>
-          <t>https://hedgewestsf.org/</t>
+          <t>https://evercore.tal.net/vx/mobile-0/candidate/jobboard/vacancy/2/feed</t>
         </is>
       </c>
       <c r="F27" s="3" t="inlineStr">
         <is>
-          <t>Quant/hedge-fund meetup series in San Francisco - one of the very few items in this article that is geographically local to Stanford. Christina Qi's 2026 quant competitions &amp; events list (LinkedIn Pulse), read 2026-09-06. Verify whether undergraduates may attend.</t>
+          <t>Verified 2026-09-26: Oleeo Atom feed, 39 entries; vacancy/1/feed has 29 more. Some events are restricted-audience per the Simplify blog.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>Already watched by iaqf-academic-paper-competition</t>
+          <t>Already watched by futureforce-launchpad</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>IAQF Academic Paper Competition</t>
+          <t>Salesforce Futureforce Tech Launchpad (CodePath)</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>Competition</t>
-        </is>
-      </c>
-      <c r="D28" s="5" t="inlineStr">
-        <is>
-          <t>CHECK</t>
+          <t>Tech internship</t>
+        </is>
+      </c>
+      <c r="D28" s="6" t="inlineStr">
+        <is>
+          <t>LATER</t>
         </is>
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>https://www.iaqf.org/upcoming-events</t>
+          <t>https://info.codepath.org/futureforce-tech-launchpad</t>
         </is>
       </c>
       <c r="F28" s="3" t="inlineStr">
         <is>
-          <t>International Association for Quantitative Finance paper competition. Christina Qi's 2026 quant competitions &amp; events list (LinkedIn Pulse), read 2026-09-06. A paper is a slower but more durable credential than a trading competition; verify undergraduate eligibility.</t>
+          <t>Verified 2026-09-26: 'Students who will complete their sophomore year in Spring 2026' - so summer 2028 for a class of 2030.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>Already watched by icerm-summer</t>
+          <t>Already watched by harvard-undergraduate-trading</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>Summer@ICERM</t>
+          <t>Harvard Undergraduate Trading Competition</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>Research / math</t>
+          <t>Competition</t>
         </is>
       </c>
       <c r="D29" s="5" t="inlineStr">
@@ -12618,61 +12618,61 @@
       </c>
       <c r="E29" s="4" t="inlineStr">
         <is>
-          <t>https://icerm.brown.edu/summerug/</t>
+          <t>https://www.huqt.com/</t>
         </is>
       </c>
       <c r="F29" s="3" t="inlineStr">
         <is>
-          <t>Verified 2026-09-26: 'Applicants must be matriculating undergraduate students'.</t>
+          <t>Undergraduate intercollegiate trading competition run by Harvard Undergraduate Quantitative Traders. The organisation rebranded: the article's link harvarduqt.com/competition 301-redirects to www.huqt.com/competition, which 404s. The live site is huqt.com and it has an Apply link. Christina Qi's 2026 quant competitions &amp; events list (LinkedIn Pulse), read 2026-09-06. Class year and team format not published - verify before planning.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>Already watched by icpc-pnw</t>
+          <t>Already watched by hedgewest-sf-meetup-series</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>ICPC</t>
+          <t>HedgeWest SF Meetup Series</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>Competition</t>
-        </is>
-      </c>
-      <c r="D30" s="2" t="inlineStr">
-        <is>
-          <t>YES</t>
+          <t>Conference / other</t>
+        </is>
+      </c>
+      <c r="D30" s="5" t="inlineStr">
+        <is>
+          <t>CHECK</t>
         </is>
       </c>
       <c r="E30" s="4" t="inlineStr">
         <is>
-          <t>https://icpc.global/</t>
+          <t>https://hedgewestsf.org/</t>
         </is>
       </c>
       <c r="F30" s="3" t="inlineStr">
         <is>
-          <t>Checked 2026-09-26: icpc.global is a JavaScript shell (53 chars); Stanford's regional, pnw.na.icpc.global, is what is watched.</t>
+          <t>Quant/hedge-fund meetup series in San Francisco - one of the very few items in this article that is geographically local to Stanford. Christina Qi's 2026 quant competitions &amp; events list (LinkedIn Pulse), read 2026-09-06. Verify whether undergraduates may attend.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>Already watched by imc-launchpad-us</t>
+          <t>Already watched by iaqf-academic-paper-competition</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>IMC Launchpad (US)</t>
+          <t>IAQF Academic Paper Competition</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>Quant firm program</t>
+          <t>Competition</t>
         </is>
       </c>
       <c r="D31" s="5" t="inlineStr">
@@ -12682,88 +12682,88 @@
       </c>
       <c r="E31" s="4" t="inlineStr">
         <is>
-          <t>https://www.imc.com/us/careers/students-graduates/programs/launchpad</t>
+          <t>https://www.iaqf.org/upcoming-events</t>
         </is>
       </c>
       <c r="F31" s="3" t="inlineStr">
         <is>
-          <t>IMC's US student program - distinct from the EU Business Course and UK Masterclass, which are geography-excluded. Christina Qi's 2026 quant competitions &amp; events list (LinkedIn Pulse), read 2026-09-06. Class year not published; verify.</t>
+          <t>International Association for Quantitative Finance paper competition. Christina Qi's 2026 quant competitions &amp; events list (LinkedIn Pulse), read 2026-09-06. A paper is a slower but more durable credential than a trading competition; verify undergraduate eligibility.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
         <is>
-          <t>Already watched by imc-prosperity</t>
+          <t>Already watched by icerm-summer</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>IMC Prosperity Trading Competition</t>
+          <t>Summer@ICERM</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>Quant firm program</t>
-        </is>
-      </c>
-      <c r="D32" s="2" t="inlineStr">
-        <is>
-          <t>YES</t>
+          <t>Research / math</t>
+        </is>
+      </c>
+      <c r="D32" s="5" t="inlineStr">
+        <is>
+          <t>CHECK</t>
         </is>
       </c>
       <c r="E32" s="4" t="inlineStr">
         <is>
-          <t>https://prosperity.imc.com/</t>
+          <t>https://icerm.brown.edu/summerug/</t>
         </is>
       </c>
       <c r="F32" s="3" t="inlineStr">
         <is>
-          <t>Teams up to 5, $50,000 pool, fully online. Most accessible serious quant competition. Stanford won top-US in year one.</t>
+          <t>Verified 2026-09-26: 'Applicants must be matriculating undergraduate students'.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>Already watched by ipam-rips</t>
+          <t>Already watched by icpc-pnw</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>IPAM RIPS (UCLA)</t>
+          <t>ICPC</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>Research / math</t>
-        </is>
-      </c>
-      <c r="D33" s="5" t="inlineStr">
-        <is>
-          <t>CHECK</t>
+          <t>Competition</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
       <c r="E33" s="4" t="inlineStr">
         <is>
-          <t>https://www.ipam.ucla.edu/programs/student-research-programs/</t>
+          <t>https://icpc.global/</t>
         </is>
       </c>
       <c r="F33" s="3" t="inlineStr">
         <is>
-          <t>Research in Industrial Projects for Students: teams of undergraduates on sponsored industry problems in applied mathematics.</t>
+          <t>Checked 2026-09-26: icpc.global is a JavaScript shell (53 chars); Stanford's regional, pnw.na.icpc.global, is what is watched.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>Already watched by janestreet-fttp</t>
+          <t>Already watched by imc-launchpad-us</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>Jane Street FTTP</t>
+          <t>IMC Launchpad (US)</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
@@ -12771,31 +12771,31 @@
           <t>Quant firm program</t>
         </is>
       </c>
-      <c r="D34" s="2" t="inlineStr">
-        <is>
-          <t>YES</t>
+      <c r="D34" s="5" t="inlineStr">
+        <is>
+          <t>CHECK</t>
         </is>
       </c>
       <c r="E34" s="4" t="inlineStr">
         <is>
-          <t>https://www.janestreet.com/join-jane-street/programs-and-events/fttp/</t>
+          <t>https://www.imc.com/us/careers/students-graduates/programs/launchpad</t>
         </is>
       </c>
       <c r="F34" s="3" t="inlineStr">
         <is>
-          <t>Classes + team-based mock trading. STEM majors, no finance background needed. Rolling - apply week one.</t>
+          <t>IMC's US student program - distinct from the EU Business Course and UK Masterclass, which are geography-excluded. Christina Qi's 2026 quant competitions &amp; events list (LinkedIn Pulse), read 2026-09-06. Class year not published; verify.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>Already watched by janestreet-preview</t>
+          <t>Already watched by imc-prosperity</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>Jane Street Preview</t>
+          <t>IMC Prosperity Trading Competition</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
@@ -12803,63 +12803,63 @@
           <t>Quant firm program</t>
         </is>
       </c>
-      <c r="D35" s="5" t="inlineStr">
-        <is>
-          <t>CHECK</t>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
       <c r="E35" s="4" t="inlineStr">
         <is>
-          <t>https://www.janestreet.com/join-jane-street/programs-and-events/preview/</t>
+          <t>https://prosperity.imc.com/</t>
         </is>
       </c>
       <c r="F35" s="3" t="inlineStr">
         <is>
-          <t>Verified 2026-09-26 (source research): day-long programme 'for students at any point in their academic career'. One of the 12 programmes on the watched janestreet-programs index; this watches its own page.</t>
+          <t>Teams up to 5, $50,000 pool, fully online. Most accessible serious quant competition. Stanford won top-US in year one.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>Already watched by janestreet-programs</t>
+          <t>Already watched by ipam-rips</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>Jane Street AMP - TA role</t>
+          <t>IPAM RIPS (UCLA)</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>Quant firm program</t>
-        </is>
-      </c>
-      <c r="D36" s="6" t="inlineStr">
-        <is>
-          <t>LATER</t>
+          <t>Research / math</t>
+        </is>
+      </c>
+      <c r="D36" s="5" t="inlineStr">
+        <is>
+          <t>CHECK</t>
         </is>
       </c>
       <c r="E36" s="4" t="inlineStr">
         <is>
-          <t>https://www.janestreet.com/join-jane-street/programs-and-events/amp/</t>
+          <t>https://www.ipam.ucla.edu/programs/student-research-programs/</t>
         </is>
       </c>
       <c r="F36" s="3" t="inlineStr">
         <is>
-          <t>Paid Jane Street summer on the teaching side. Housing, meals, travel covered. Eligible from spring 2027.</t>
+          <t>Research in Industrial Projects for Students: teams of undergraduates on sponsored industry problems in applied mathematics.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>Already watched by janestreet-programs</t>
+          <t>Already watched by janestreet-fttp</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>Jane Street ETC</t>
+          <t>Jane Street FTTP</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
@@ -12867,31 +12867,31 @@
           <t>Quant firm program</t>
         </is>
       </c>
-      <c r="D37" s="5" t="inlineStr">
-        <is>
-          <t>INVITE</t>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
       <c r="E37" s="4" t="inlineStr">
         <is>
-          <t>https://www.janestreet.com/join-jane-street/programs-and-events/</t>
+          <t>https://www.janestreet.com/join-jane-street/programs-and-events/fttp/</t>
         </is>
       </c>
       <c r="F37" s="3" t="inlineStr">
         <is>
-          <t>Electronic Trading Challenge. Entry via university, prior JS events, or the puzzle ecosystem.</t>
+          <t>Classes + team-based mock trading. STEM majors, no finance background needed. Rolling - apply week one.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
         <is>
-          <t>Already watched by janestreet-programs</t>
+          <t>Already watched by janestreet-preview</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>Jane Street SEE</t>
+          <t>Jane Street Preview</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
@@ -12899,19 +12899,19 @@
           <t>Quant firm program</t>
         </is>
       </c>
-      <c r="D38" s="2" t="inlineStr">
-        <is>
-          <t>YES</t>
+      <c r="D38" s="5" t="inlineStr">
+        <is>
+          <t>CHECK</t>
         </is>
       </c>
       <c r="E38" s="4" t="inlineStr">
         <is>
-          <t>https://www.janestreet.com/join-jane-street/programs-and-events/</t>
+          <t>https://www.janestreet.com/join-jane-street/programs-and-events/preview/</t>
         </is>
       </c>
       <c r="F38" s="3" t="inlineStr">
         <is>
-          <t>Software Engineering Experience - OCaml and systems design.</t>
+          <t>Verified 2026-09-26 (source research): day-long programme 'for students at any point in their academic career'. One of the 12 programmes on the watched janestreet-programs index; this watches its own page.</t>
         </is>
       </c>
     </row>
@@ -12923,7 +12923,7 @@
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>Jane Street Symposium</t>
+          <t>Jane Street AMP - TA role</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
@@ -12931,17 +12931,21 @@
           <t>Quant firm program</t>
         </is>
       </c>
-      <c r="D39" s="5" t="inlineStr">
-        <is>
-          <t>INVITE</t>
+      <c r="D39" s="6" t="inlineStr">
+        <is>
+          <t>LATER</t>
         </is>
       </c>
       <c r="E39" s="4" t="inlineStr">
         <is>
-          <t>https://www.janestreet.com/join-jane-street/programs-and-events/</t>
-        </is>
-      </c>
-      <c r="F39" s="3" t="inlineStr"/>
+          <t>https://www.janestreet.com/join-jane-street/programs-and-events/amp/</t>
+        </is>
+      </c>
+      <c r="F39" s="3" t="inlineStr">
+        <is>
+          <t>Paid Jane Street summer on the teaching side. Housing, meals, travel covered. Eligible from spring 2027.</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
@@ -12951,7 +12955,7 @@
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>Jane Street Unboxed</t>
+          <t>Jane Street ETC</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
@@ -12961,7 +12965,7 @@
       </c>
       <c r="D40" s="5" t="inlineStr">
         <is>
-          <t>CHECK</t>
+          <t>INVITE</t>
         </is>
       </c>
       <c r="E40" s="4" t="inlineStr">
@@ -12969,209 +12973,205 @@
           <t>https://www.janestreet.com/join-jane-street/programs-and-events/</t>
         </is>
       </c>
-      <c r="F40" s="3" t="inlineStr"/>
+      <c r="F40" s="3" t="inlineStr">
+        <is>
+          <t>Electronic Trading Challenge. Entry via university, prior JS events, or the puzzle ecosystem.</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>Already watched by jefferies-campus</t>
+          <t>Already watched by janestreet-programs</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>Jefferies campus opportunities</t>
+          <t>Jane Street SEE</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>Conference / other</t>
-        </is>
-      </c>
-      <c r="D41" s="5" t="inlineStr">
-        <is>
-          <t>CHECK</t>
+          <t>Quant firm program</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
       <c r="E41" s="4" t="inlineStr">
         <is>
-          <t>https://jefferies.tal.net/vx/mobile-0/candidate/jobboard/vacancy/2/feed</t>
+          <t>https://www.janestreet.com/join-jane-street/programs-and-events/</t>
         </is>
       </c>
       <c r="F41" s="3" t="inlineStr">
         <is>
-          <t>Verified 2026-09-26: Oleeo Atom feed, 60 entries. Banking is lower priority than quant.</t>
+          <t>Software Engineering Experience - OCaml and systems design.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
         <is>
-          <t>Already watched by jhuapl-internships</t>
+          <t>Already watched by janestreet-programs</t>
         </is>
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>Johns Hopkins APL internships</t>
+          <t>Jane Street Symposium</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>Research / math</t>
+          <t>Quant firm program</t>
         </is>
       </c>
       <c r="D42" s="5" t="inlineStr">
         <is>
-          <t>CHECK</t>
+          <t>INVITE</t>
         </is>
       </c>
       <c r="E42" s="4" t="inlineStr">
         <is>
-          <t>https://www.jhuapl.edu/careers/internships</t>
-        </is>
-      </c>
-      <c r="F42" s="3" t="inlineStr">
-        <is>
-          <t>Page states a minimum GPA requirement. Simplify already carries some APL postings; this watches the programme page itself.</t>
-        </is>
-      </c>
+          <t>https://www.janestreet.com/join-jane-street/programs-and-events/</t>
+        </is>
+      </c>
+      <c r="F42" s="3" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
         <is>
-          <t>Already watched by jpmc-career-edyou</t>
+          <t>Already watched by janestreet-programs</t>
         </is>
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>JPMorganChase Career.edYOU Academy</t>
+          <t>Jane Street Unboxed</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>Tech internship</t>
-        </is>
-      </c>
-      <c r="D43" s="6" t="inlineStr">
-        <is>
-          <t>LATER</t>
+          <t>Quant firm program</t>
+        </is>
+      </c>
+      <c r="D43" s="5" t="inlineStr">
+        <is>
+          <t>CHECK</t>
         </is>
       </c>
       <c r="E43" s="4" t="inlineStr">
         <is>
-          <t>https://www.jpmorganchase.com/careers/explore-opportunities/programs/career-edyou</t>
-        </is>
-      </c>
-      <c r="F43" s="3" t="inlineStr">
-        <is>
-          <t>Verified 2026-09-26: 'designed for college sophomores studying in the United States'.</t>
-        </is>
-      </c>
+          <t>https://www.janestreet.com/join-jane-street/programs-and-events/</t>
+        </is>
+      </c>
+      <c r="F43" s="3" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
         <is>
-          <t>Already watched by jpmc-fellowship</t>
+          <t>Already watched by jefferies-campus</t>
         </is>
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>JPMC Fellowship Program</t>
+          <t>Jefferies campus opportunities</t>
         </is>
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>Tech internship</t>
-        </is>
-      </c>
-      <c r="D44" s="6" t="inlineStr">
-        <is>
-          <t>LATER</t>
+          <t>Conference / other</t>
+        </is>
+      </c>
+      <c r="D44" s="5" t="inlineStr">
+        <is>
+          <t>CHECK</t>
         </is>
       </c>
       <c r="E44" s="4" t="inlineStr">
         <is>
-          <t>https://www.jpmorganchase.com/careers/explore-opportunities/programs/jpmcfellowship</t>
+          <t>https://jefferies.tal.net/vx/mobile-0/candidate/jobboard/vacancy/2/feed</t>
         </is>
       </c>
       <c r="F44" s="3" t="inlineStr">
         <is>
-          <t>Verified 2026-09-26: 'sophomore students, including, without limitation, Black, Hispanic and Latino... All sophomore students... regardless of background, are welcome'.</t>
+          <t>Verified 2026-09-26: Oleeo Atom feed, 60 entries. Banking is lower priority than quant.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
         <is>
-          <t>Already watched by jumptrading-greenhouse</t>
+          <t>Already watched by jhuapl-internships</t>
         </is>
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>Jump Trading Campus Jump Early Access</t>
+          <t>Johns Hopkins APL internships</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>Quant firm program</t>
-        </is>
-      </c>
-      <c r="D45" s="2" t="inlineStr">
-        <is>
-          <t>YES</t>
+          <t>Research / math</t>
+        </is>
+      </c>
+      <c r="D45" s="5" t="inlineStr">
+        <is>
+          <t>CHECK</t>
         </is>
       </c>
       <c r="E45" s="4" t="inlineStr">
         <is>
-          <t>https://www.jumptrading.com/hr/students-new-grads</t>
+          <t>https://www.jhuapl.edu/careers/internships</t>
         </is>
       </c>
       <c r="F45" s="3" t="inlineStr">
         <is>
-          <t>Verified 2026-09-30 from the 2026 posting: 'First-year undergraduates at US universities' in math/CS/physics/stats/engineering/econ. One-day programme in Chicago, travel/meals/lodging covered. Posts on the Greenhouse board watched by jumptrading-greenhouse; not live today.</t>
+          <t>Page states a minimum GPA requirement. Simplify already carries some APL postings; this watches the programme page itself.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="3" t="inlineStr">
         <is>
-          <t>Already watched by kkr-greenhouse</t>
+          <t>Already watched by jpmc-career-edyou</t>
         </is>
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>KKR Scholars Program</t>
+          <t>JPMorganChase Career.edYOU Academy</t>
         </is>
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>Quant firm program</t>
-        </is>
-      </c>
-      <c r="D46" s="2" t="inlineStr">
-        <is>
-          <t>YES</t>
+          <t>Tech internship</t>
+        </is>
+      </c>
+      <c r="D46" s="6" t="inlineStr">
+        <is>
+          <t>LATER</t>
         </is>
       </c>
       <c r="E46" s="4" t="inlineStr">
         <is>
-          <t>https://www.kkr.com/careers/student-careers/student-career-opportunities</t>
+          <t>https://www.jpmorganchase.com/careers/explore-opportunities/programs/career-edyou</t>
         </is>
       </c>
       <c r="F46" s="3" t="inlineStr">
         <is>
-          <t>2025 posting: 'rising sophomores graduating with a Bachelor's degree in December 2027 – June 2028'. The 2027 edition should be Dec 2029-Jun 2030, the owner's window. Late-May dates may clash with Stanford spring quarter. Posts on KKR's Greenhouse board, slug 'staged'.</t>
+          <t>Verified 2026-09-26: 'designed for college sophomores studying in the United States'.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
         <is>
-          <t>Already watched by kleinerperkins-fellows-ashby</t>
+          <t>Already watched by jpmc-fellowship</t>
         </is>
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>Kleiner Perkins Engineering Fellows</t>
+          <t>JPMC Fellowship Program</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr">
@@ -13179,123 +13179,127 @@
           <t>Tech internship</t>
         </is>
       </c>
-      <c r="D47" s="5" t="inlineStr">
-        <is>
-          <t>CHECK</t>
+      <c r="D47" s="6" t="inlineStr">
+        <is>
+          <t>LATER</t>
         </is>
       </c>
       <c r="E47" s="4" t="inlineStr">
         <is>
-          <t>https://www.kleinerperkins.com/fellows/</t>
+          <t>https://www.jpmorganchase.com/careers/explore-opportunities/programs/jpmcfellowship</t>
         </is>
       </c>
       <c r="F47" s="3" t="inlineStr">
         <is>
-          <t>Verified 2026-09-30 from the Ashby posting: no class-year gate; wants 'Degree in computer science, engineering, math, physics or other fields related to software engineering' and Bay Area availability. Summer placement at a KP portfolio startup plus speaker series. Selective, and cohorts skew upperclass.</t>
+          <t>Verified 2026-09-26: 'sophomore students, including, without limitation, Black, Hispanic and Latino... All sophomore students... regardless of background, are welcome'.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="3" t="inlineStr">
         <is>
-          <t>Already watched by lanl-students</t>
+          <t>Already watched by jumptrading-greenhouse</t>
         </is>
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>LANL student internships (Los Alamos National Laboratory)</t>
+          <t>Jump Trading Campus Jump Early Access</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>Research / math</t>
-        </is>
-      </c>
-      <c r="D48" s="5" t="inlineStr">
-        <is>
-          <t>CHECK</t>
+          <t>Quant firm program</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
       <c r="E48" s="4" t="inlineStr">
         <is>
-          <t>https://www.lanl.gov/engage/collaboration/internships</t>
+          <t>https://www.jumptrading.com/hr/students-new-grads</t>
         </is>
       </c>
       <c r="F48" s="3" t="inlineStr">
         <is>
-          <t>Lab-run undergraduate internship programme. The old /careers/career-options/student-internships URL redirects here.</t>
+          <t>Verified 2026-09-30 from the 2026 posting: 'First-year undergraduates at US universities' in math/CS/physics/stats/engineering/econ. One-day programme in Chicago, travel/meals/lodging covered. Posts on the Greenhouse board watched by jumptrading-greenhouse; not live today.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
         <is>
-          <t>Already watched by llnl-students</t>
+          <t>Already watched by kkr-greenhouse</t>
         </is>
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>LLNL student internships (Lawrence Livermore National Laboratory)</t>
+          <t>KKR Scholars Program</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>Research / math</t>
-        </is>
-      </c>
-      <c r="D49" s="5" t="inlineStr">
-        <is>
-          <t>CHECK</t>
+          <t>Quant firm program</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
       <c r="E49" s="4" t="inlineStr">
         <is>
-          <t>https://www.llnl.gov/join-our-team/careers/student-internship-veteran-programs</t>
+          <t>https://www.kkr.com/careers/student-careers/student-career-opportunities</t>
         </is>
       </c>
       <c r="F49" s="3" t="inlineStr">
         <is>
-          <t>Undergraduate summer internships plus internally and externally sponsored student programmes. Not part of DOE SULI's lab list in this file.</t>
+          <t>2025 posting: 'rising sophomores graduating with a Bachelor's degree in December 2027 – June 2028'. The 2027 edition should be Dec 2029-Jun 2030, the owner's window. Late-May dates may clash with Stanford spring quarter. Posts on KKR's Greenhouse board, slug 'staged'.</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="3" t="inlineStr">
         <is>
-          <t>Already watched by luisae</t>
+          <t>Already watched by kleinerperkins-fellows-ashby</t>
         </is>
       </c>
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t>LuisaE/opportunities</t>
+          <t>Kleiner Perkins Engineering Fellows</t>
         </is>
       </c>
       <c r="C50" s="3" t="inlineStr">
         <is>
-          <t>Tracker / resource</t>
-        </is>
-      </c>
-      <c r="D50" s="2" t="inlineStr">
-        <is>
-          <t>USE</t>
+          <t>Tech internship</t>
+        </is>
+      </c>
+      <c r="D50" s="5" t="inlineStr">
+        <is>
+          <t>CHECK</t>
         </is>
       </c>
       <c r="E50" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/LuisaE/opportunities</t>
-        </is>
-      </c>
-      <c r="F50" s="3" t="inlineStr"/>
+          <t>https://www.kleinerperkins.com/fellows/</t>
+        </is>
+      </c>
+      <c r="F50" s="3" t="inlineStr">
+        <is>
+          <t>Verified 2026-09-30 from the Ashby posting: no class-year gate; wants 'Degree in computer science, engineering, math, physics or other fields related to software engineering' and Bay Area availability. Summer placement at a KP portfolio startup plus speaker series. Selective, and cohorts skew upperclass.</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
         <is>
-          <t>Already watched by mathprograms-listing</t>
+          <t>Already watched by lanl-students</t>
         </is>
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>MathPrograms.org programme listing</t>
+          <t>LANL student internships (Los Alamos National Laboratory)</t>
         </is>
       </c>
       <c r="C51" s="3" t="inlineStr">
@@ -13310,29 +13314,29 @@
       </c>
       <c r="E51" s="4" t="inlineStr">
         <is>
-          <t>https://www.mathprograms.org/db/program</t>
+          <t>https://www.lanl.gov/engage/collaboration/internships</t>
         </is>
       </c>
       <c r="F51" s="3" t="inlineStr">
         <is>
-          <t>Verified 2026-09-26: AMS-run application portal most math REUs use (UChicago, PCMI, Polymath Jr); already lists POLYMATHREU2027 and SLMath PROOF 2027. Substitutes for the NSF REU directory (AWS WAF challenge) and the AMS REU list (403), neither readable by this client.</t>
+          <t>Lab-run undergraduate internship programme. The old /careers/career-options/student-internships URL redirects here.</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="3" t="inlineStr">
         <is>
-          <t>Already watched by meta-hacker-cup</t>
+          <t>Already watched by llnl-students</t>
         </is>
       </c>
       <c r="B52" s="3" t="inlineStr">
         <is>
-          <t>Meta Hacker Cup</t>
+          <t>LLNL student internships (Lawrence Livermore National Laboratory)</t>
         </is>
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>Competition</t>
+          <t>Research / math</t>
         </is>
       </c>
       <c r="D52" s="5" t="inlineStr">
@@ -13342,61 +13346,57 @@
       </c>
       <c r="E52" s="4" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/codingcompetitions/hacker-cup</t>
+          <t>https://www.llnl.gov/join-our-team/careers/student-internship-veteran-programs</t>
         </is>
       </c>
       <c r="F52" s="3" t="inlineStr">
         <is>
-          <t>Verified 2026-09-26: 'Open to participants around the world'. Page still shows the 2025 season. JavaScript page: 15 chars plain, 1,485 rendered.</t>
+          <t>Undergraduate summer internships plus internally and externally sponsored student programmes. Not part of DOE SULI's lab list in this file.</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="3" t="inlineStr">
         <is>
-          <t>Already watched by millennium-eightfold</t>
+          <t>Already watched by luisae</t>
         </is>
       </c>
       <c r="B53" s="3" t="inlineStr">
         <is>
-          <t>Meet Millennium</t>
+          <t>LuisaE/opportunities</t>
         </is>
       </c>
       <c r="C53" s="3" t="inlineStr">
         <is>
-          <t>Quant firm program</t>
-        </is>
-      </c>
-      <c r="D53" s="5" t="inlineStr">
-        <is>
-          <t>CHECK</t>
+          <t>Tracker / resource</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>USE</t>
         </is>
       </c>
       <c r="E53" s="4" t="inlineStr">
         <is>
-          <t>https://www.mlp.com/life-at-millennium/inside-meet-millennium/</t>
-        </is>
-      </c>
-      <c r="F53" s="3" t="inlineStr">
-        <is>
-          <t>Verified 2026-09-30: 'high-performing undergraduate and master's students ... Designed as an insight into Millennium's 2027 Summer Intern Program'. Travel to one of five offices; SWE/quant-engineering simulations. www.mlp.com is WP Engine, so not watched directly; the posting should surface via millennium-eightfold.</t>
-        </is>
-      </c>
+          <t>https://github.com/LuisaE/opportunities</t>
+        </is>
+      </c>
+      <c r="F53" s="3" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="3" t="inlineStr">
         <is>
-          <t>Already watched by mit-battlecode-2027</t>
+          <t>Already watched by mathprograms-listing</t>
         </is>
       </c>
       <c r="B54" s="3" t="inlineStr">
         <is>
-          <t>MIT Battlecode 2027</t>
+          <t>MathPrograms.org programme listing</t>
         </is>
       </c>
       <c r="C54" s="3" t="inlineStr">
         <is>
-          <t>Competition</t>
+          <t>Research / math</t>
         </is>
       </c>
       <c r="D54" s="5" t="inlineStr">
@@ -13406,24 +13406,24 @@
       </c>
       <c r="E54" s="4" t="inlineStr">
         <is>
-          <t>https://battlecode.org/</t>
+          <t>https://www.mathprograms.org/db/program</t>
         </is>
       </c>
       <c r="F54" s="3" t="inlineStr">
         <is>
-          <t>MIT's real-time strategy AI competition: you write an autonomous player that commands a robot army, then compete in scrimmages and bracketed tournaments over January. Over $20,000 in total prize money. Open beyond MIT - 'Anyone can write a bot, create a team, and participate in scrimmage matches/rankings.' Prize-tournament gates from the Full Eligibility Rules (battlecode.org/about.html): Sprint Tournaments - 'All teams are eligible.' US Qualifier - 'Teams must consist entirely of US college students studying full-time, or in a transition phase.' Final Tournament - 'Teams must have qualified via the US or International Qualifier.' MIT Newbie Tournament is MIT-only and High School Tournament is high-school-only, so neither applies. Unlike MIT Pokerbots, no MIT-affiliated teammate or MIT certificate is needed for the track you would enter. As of Sep 2026 the site still reads 'Battlecode 2026 ended on January 31st, 2026!' - no 2027 registration date posted yet, though the page already references Battlecode 2027 sponsorships. No team size limit, age limit, or citizenship rule beyond 'US college student' was stated on the pages read. Source: battlecode.org home page and about.html.</t>
+          <t>Verified 2026-09-26: AMS-run application portal most math REUs use (UChicago, PCMI, Polymath Jr); already lists POLYMATHREU2027 and SLMath PROOF 2027. Substitutes for the NSF REU directory (AWS WAF challenge) and the AMS REU list (403), neither readable by this client.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="3" t="inlineStr">
         <is>
-          <t>Already watched by mit-trading-competition</t>
+          <t>Already watched by meta-hacker-cup</t>
         </is>
       </c>
       <c r="B55" s="3" t="inlineStr">
         <is>
-          <t>Traders@MIT Trading Competition</t>
+          <t>Meta Hacker Cup</t>
         </is>
       </c>
       <c r="C55" s="3" t="inlineStr">
@@ -13431,36 +13431,36 @@
           <t>Competition</t>
         </is>
       </c>
-      <c r="D55" s="2" t="inlineStr">
-        <is>
-          <t>YES</t>
+      <c r="D55" s="5" t="inlineStr">
+        <is>
+          <t>CHECK</t>
         </is>
       </c>
       <c r="E55" s="4" t="inlineStr">
         <is>
-          <t>https://traders.mit.edu/competition</t>
+          <t>https://www.facebook.com/codingcompetitions/hacker-cup</t>
         </is>
       </c>
       <c r="F55" s="3" t="inlineStr">
         <is>
-          <t>Largest intercollegiate competition, $20,000+. NOT the same as Pokerbots - this one IS open to first-years.</t>
+          <t>Verified 2026-09-26: 'Open to participants around the world'. Page still shows the 2025 season. JavaScript page: 15 chars plain, 1,485 rendered.</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="3" t="inlineStr">
         <is>
-          <t>Already watched by mitll-students</t>
+          <t>Already watched by millennium-eightfold</t>
         </is>
       </c>
       <c r="B56" s="3" t="inlineStr">
         <is>
-          <t>MIT Lincoln Laboratory student opportunities</t>
+          <t>Meet Millennium</t>
         </is>
       </c>
       <c r="C56" s="3" t="inlineStr">
         <is>
-          <t>Research / math</t>
+          <t>Quant firm program</t>
         </is>
       </c>
       <c r="D56" s="5" t="inlineStr">
@@ -13470,157 +13470,157 @@
       </c>
       <c r="E56" s="4" t="inlineStr">
         <is>
-          <t>https://www.ll.mit.edu/careers/student-opportunities</t>
+          <t>https://www.mlp.com/life-at-millennium/inside-meet-millennium/</t>
         </is>
       </c>
       <c r="F56" s="3" t="inlineStr">
         <is>
-          <t>Several tracks. The industry-mentor programme is for students in their junior year; the Summer Research Program takes undergraduate and graduate students.</t>
+          <t>Verified 2026-09-30: 'high-performing undergraduate and master's students ... Designed as an insight into Millennium's 2027 Summer Intern Program'. Travel to one of five offices; SWE/quant-engineering simulations. www.mlp.com is WP Engine, so not watched directly; the posting should surface via millennium-eightfold.</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="3" t="inlineStr">
         <is>
-          <t>Already watched by nist-surf</t>
+          <t>Already watched by mit-battlecode-2027</t>
         </is>
       </c>
       <c r="B57" s="3" t="inlineStr">
         <is>
-          <t>NIST SURF</t>
+          <t>MIT Battlecode 2027</t>
         </is>
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t>Research / math</t>
-        </is>
-      </c>
-      <c r="D57" s="2" t="inlineStr">
-        <is>
-          <t>YES</t>
+          <t>Competition</t>
+        </is>
+      </c>
+      <c r="D57" s="5" t="inlineStr">
+        <is>
+          <t>CHECK</t>
         </is>
       </c>
       <c r="E57" s="4" t="inlineStr">
         <is>
-          <t>https://www.nist.gov/surf</t>
+          <t>https://battlecode.org/</t>
         </is>
       </c>
       <c r="F57" s="3" t="inlineStr">
         <is>
-          <t>Verified 2026-09-30: 'only open to U.S. citizens and U.S. permanent residents enrolled as undergraduate students at U.S. colleges or universities'; states no class-year minimum. 11 weeks, $710/week plus lodging/travel allowance. Information Technology Lab has math/CS/ML projects.</t>
+          <t>MIT's real-time strategy AI competition: you write an autonomous player that commands a robot army, then compete in scrimmages and bracketed tournaments over January. Over $20,000 in total prize money. Open beyond MIT - 'Anyone can write a bot, create a team, and participate in scrimmage matches/rankings.' Prize-tournament gates from the Full Eligibility Rules (battlecode.org/about.html): Sprint Tournaments - 'All teams are eligible.' US Qualifier - 'Teams must consist entirely of US college students studying full-time, or in a transition phase.' Final Tournament - 'Teams must have qualified via the US or International Qualifier.' MIT Newbie Tournament is MIT-only and High School Tournament is high-school-only, so neither applies. Unlike MIT Pokerbots, no MIT-affiliated teammate or MIT certificate is needed for the track you would enter. As of Sep 2026 the site still reads 'Battlecode 2026 ended on January 31st, 2026!' - no 2027 registration date posted yet, though the page already references Battlecode 2027 sponsorships. No team size limit, age limit, or citizenship rule beyond 'US college student' was stated on the pages read. Source: battlecode.org home page and about.html.</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="3" t="inlineStr">
         <is>
-          <t>Already watched by nsa-students</t>
+          <t>Already watched by mit-trading-competition</t>
         </is>
       </c>
       <c r="B58" s="3" t="inlineStr">
         <is>
-          <t>NSA student programs</t>
+          <t>Traders@MIT Trading Competition</t>
         </is>
       </c>
       <c r="C58" s="3" t="inlineStr">
         <is>
-          <t>Research / math</t>
-        </is>
-      </c>
-      <c r="D58" s="5" t="inlineStr">
-        <is>
-          <t>CHECK</t>
+          <t>Competition</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
       <c r="E58" s="4" t="inlineStr">
         <is>
-          <t>https://www.intelligencecareers.gov/nsa/students</t>
+          <t>https://traders.mit.edu/competition</t>
         </is>
       </c>
       <c r="F58" s="3" t="inlineStr">
         <is>
-          <t>NSA's student internship and co-op listings on intelligencecareers.gov. Security clearance means US citizens only.</t>
+          <t>Largest intercollegiate competition, $20,000+. NOT the same as Pokerbots - this one IS open to first-years.</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="3" t="inlineStr">
         <is>
-          <t>Already watched by nuft-2027</t>
+          <t>Already watched by mitll-students</t>
         </is>
       </c>
       <c r="B59" s="3" t="inlineStr">
         <is>
-          <t>NUFT 2027 Quant Internships</t>
+          <t>MIT Lincoln Laboratory student opportunities</t>
         </is>
       </c>
       <c r="C59" s="3" t="inlineStr">
         <is>
-          <t>Tracker / resource</t>
-        </is>
-      </c>
-      <c r="D59" s="2" t="inlineStr">
-        <is>
-          <t>USE WEEKLY</t>
+          <t>Research / math</t>
+        </is>
+      </c>
+      <c r="D59" s="5" t="inlineStr">
+        <is>
+          <t>CHECK</t>
         </is>
       </c>
       <c r="E59" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/northwesternfintech/2027QuantInternships</t>
+          <t>https://www.ll.mit.edu/careers/student-opportunities</t>
         </is>
       </c>
       <c r="F59" s="3" t="inlineStr">
         <is>
-          <t>47 firms. No class-year tags - use as a firm checklist and open each careers page yourself.</t>
+          <t>Several tracks. The industry-mentor programme is for students in their junior year; the Summer Research Program takes undergraduate and graduate students.</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="3" t="inlineStr">
         <is>
-          <t>Already watched by open-source-quantitative-finance</t>
+          <t>Already watched by nist-surf</t>
         </is>
       </c>
       <c r="B60" s="3" t="inlineStr">
         <is>
-          <t>Open Source Quantitative Finance Conference</t>
+          <t>NIST SURF</t>
         </is>
       </c>
       <c r="C60" s="3" t="inlineStr">
         <is>
-          <t>Conference / other</t>
-        </is>
-      </c>
-      <c r="D60" s="5" t="inlineStr">
-        <is>
-          <t>CHECK</t>
+          <t>Research / math</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
       <c r="E60" s="4" t="inlineStr">
         <is>
-          <t>https://osqf.org/</t>
+          <t>https://www.nist.gov/surf</t>
         </is>
       </c>
       <c r="F60" s="3" t="inlineStr">
         <is>
-          <t>Open-source quant finance conference, free per the article. Christina Qi's 2026 quant competitions &amp; events list (LinkedIn Pulse), read 2026-09-06. Verify format and whether students may attend.</t>
+          <t>Verified 2026-09-30: 'only open to U.S. citizens and U.S. permanent residents enrolled as undergraduate students at U.S. colleges or universities'; states no class-year minimum. 11 weeks, $710/week plus lodging/travel allowance. Information Technology Lab has math/CS/ML projects.</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="3" t="inlineStr">
         <is>
-          <t>Already watched by optiver-futurefocus</t>
+          <t>Already watched by nsa-students</t>
         </is>
       </c>
       <c r="B61" s="3" t="inlineStr">
         <is>
-          <t>Optiver FutureFocus Chicago 2026</t>
+          <t>NSA student programs</t>
         </is>
       </c>
       <c r="C61" s="3" t="inlineStr">
         <is>
-          <t>Quant firm program</t>
+          <t>Research / math</t>
         </is>
       </c>
       <c r="D61" s="5" t="inlineStr">
@@ -13630,57 +13630,61 @@
       </c>
       <c r="E61" s="4" t="inlineStr">
         <is>
-          <t>https://optiver.com/recruitment-events/futurefocus-chicago</t>
+          <t>https://www.intelligencecareers.gov/nsa/students</t>
         </is>
       </c>
       <c r="F61" s="3" t="inlineStr">
         <is>
-          <t>Optiver's US (Chicago) student recruitment event. The other FutureFocus and Career Kickstarter events are ANZ, China, Singapore, India and Europe - see the consolidated non-US row. Christina Qi's 2026 quant competitions &amp; events list (LinkedIn Pulse), read 2026-09-06.</t>
+          <t>NSA's student internship and co-op listings on intelligencecareers.gov. Security clearance means US citizens only.</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="3" t="inlineStr">
         <is>
-          <t>Already watched by optiver-ready-trader</t>
+          <t>Already watched by nuft-2027</t>
         </is>
       </c>
       <c r="B62" s="3" t="inlineStr">
         <is>
-          <t>Optiver Ready Trader Go</t>
+          <t>NUFT 2027 Quant Internships</t>
         </is>
       </c>
       <c r="C62" s="3" t="inlineStr">
         <is>
-          <t>Quant firm program</t>
-        </is>
-      </c>
-      <c r="D62" s="5" t="inlineStr">
-        <is>
-          <t>CHECK</t>
+          <t>Tracker / resource</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>USE WEEKLY</t>
         </is>
       </c>
       <c r="E62" s="4" t="inlineStr">
         <is>
-          <t>https://optiver.com/working-at-optiver/career-opportunities/</t>
-        </is>
-      </c>
-      <c r="F62" s="3" t="inlineStr"/>
+          <t>https://github.com/northwesternfintech/2027QuantInternships</t>
+        </is>
+      </c>
+      <c r="F62" s="3" t="inlineStr">
+        <is>
+          <t>47 firms. No class-year tags - use as a firm checklist and open each careers page yourself.</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="3" t="inlineStr">
         <is>
-          <t>Already watched by purdue-srop</t>
+          <t>Already watched by open-source-quantitative-finance</t>
         </is>
       </c>
       <c r="B63" s="3" t="inlineStr">
         <is>
-          <t>Purdue Summer Research Opportunities Program (SROP)</t>
+          <t>Open Source Quantitative Finance Conference</t>
         </is>
       </c>
       <c r="C63" s="3" t="inlineStr">
         <is>
-          <t>Research / math</t>
+          <t>Conference / other</t>
         </is>
       </c>
       <c r="D63" s="5" t="inlineStr">
@@ -13690,71 +13694,71 @@
       </c>
       <c r="E63" s="4" t="inlineStr">
         <is>
-          <t>https://www.purdue.edu/academics/ogsps/ogrs/summer-research-opportunity-program/</t>
+          <t>https://osqf.org/</t>
         </is>
       </c>
       <c r="F63" s="3" t="inlineStr">
         <is>
-          <t>Part of the Big Ten Academic Alliance SROP. Page states eligibility includes US citizens, permanent residents, refugees and asylees enrolled at a US institution; read the full criteria on the page.</t>
+          <t>Open-source quant finance conference, free per the article. Christina Qi's 2026 quant competitions &amp; events list (LinkedIn Pulse), read 2026-09-06. Verify format and whether students may attend.</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="3" t="inlineStr">
         <is>
-          <t>Already watched by ramp-ashby</t>
+          <t>Already watched by optiver-futurefocus</t>
         </is>
       </c>
       <c r="B64" s="3" t="inlineStr">
         <is>
-          <t>Ramp Emerging Talent</t>
+          <t>Optiver FutureFocus Chicago 2026</t>
         </is>
       </c>
       <c r="C64" s="3" t="inlineStr">
         <is>
-          <t>Tech internship</t>
-        </is>
-      </c>
-      <c r="D64" s="2" t="inlineStr">
-        <is>
-          <t>YES</t>
+          <t>Quant firm program</t>
+        </is>
+      </c>
+      <c r="D64" s="5" t="inlineStr">
+        <is>
+          <t>CHECK</t>
         </is>
       </c>
       <c r="E64" s="4" t="inlineStr">
         <is>
-          <t>https://ramp.com/emerging-talent</t>
+          <t>https://optiver.com/recruitment-events/futurefocus-chicago</t>
         </is>
       </c>
       <c r="F64" s="3" t="inlineStr">
         <is>
-          <t>Verified 2026-09-30: 'For interns: anyone who will be registered in an accredited 4 year university post-internship.' Fintech SWE internships posted on Ashby 'ramp'.</t>
+          <t>Optiver's US (Chicago) student recruitment event. The other FutureFocus and Career Kickstarter events are ANZ, China, Singapore, India and Europe - see the consolidated non-US row. Christina Qi's 2026 quant competitions &amp; events list (LinkedIn Pulse), read 2026-09-06.</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="3" t="inlineStr">
         <is>
-          <t>Already watched by reufinder-freshmen</t>
+          <t>Already watched by optiver-ready-trader</t>
         </is>
       </c>
       <c r="B65" s="3" t="inlineStr">
         <is>
-          <t>REU Finder - freshman-eligible filter</t>
+          <t>Optiver Ready Trader Go</t>
         </is>
       </c>
       <c r="C65" s="3" t="inlineStr">
         <is>
-          <t>Research / math</t>
-        </is>
-      </c>
-      <c r="D65" s="2" t="inlineStr">
-        <is>
-          <t>YES</t>
+          <t>Quant firm program</t>
+        </is>
+      </c>
+      <c r="D65" s="5" t="inlineStr">
+        <is>
+          <t>CHECK</t>
         </is>
       </c>
       <c r="E65" s="4" t="inlineStr">
         <is>
-          <t>https://reufinder.com/programs-for-freshmen/</t>
+          <t>https://optiver.com/working-at-optiver/career-opportunities/</t>
         </is>
       </c>
       <c r="F65" s="3" t="inlineStr"/>
@@ -13762,12 +13766,12 @@
     <row r="66">
       <c r="A66" s="3" t="inlineStr">
         <is>
-          <t>Already watched by sandia-students</t>
+          <t>Already watched by purdue-srop</t>
         </is>
       </c>
       <c r="B66" s="3" t="inlineStr">
         <is>
-          <t>Sandia National Laboratories student internships</t>
+          <t>Purdue Summer Research Opportunities Program (SROP)</t>
         </is>
       </c>
       <c r="C66" s="3" t="inlineStr">
@@ -13782,29 +13786,29 @@
       </c>
       <c r="E66" s="4" t="inlineStr">
         <is>
-          <t>https://www.sandia.gov/careers/careers/students-and-postdocs/</t>
+          <t>https://www.purdue.edu/academics/ogsps/ogrs/summer-research-opportunity-program/</t>
         </is>
       </c>
       <c r="F66" s="3" t="inlineStr">
         <is>
-          <t>Undergraduate and graduate internships across Sandia's sites.</t>
+          <t>Part of the Big Ten Academic Alliance SROP. Page states eligibility includes US citizens, permanent residents, refugees and asylees enrolled at a US institution; read the full criteria on the page.</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="3" t="inlineStr">
         <is>
-          <t>Already watched by scudem</t>
+          <t>Already watched by ramp-ashby</t>
         </is>
       </c>
       <c r="B67" s="3" t="inlineStr">
         <is>
-          <t>SCUDEM XI 2026</t>
+          <t>Ramp Emerging Talent</t>
         </is>
       </c>
       <c r="C67" s="3" t="inlineStr">
         <is>
-          <t>Competition</t>
+          <t>Tech internship</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr">
@@ -13814,56 +13818,52 @@
       </c>
       <c r="E67" s="4" t="inlineStr">
         <is>
-          <t>https://www.contest.comap.com/scudem/index.html</t>
+          <t>https://ramp.com/emerging-talent</t>
         </is>
       </c>
       <c r="F67" s="3" t="inlineStr">
         <is>
-          <t>Verified 2026-09-30: COMAP's differential-equations modelling challenge. FAQ: 'open to teams of 3 undergraduate or high school students. Each team must have a coach (typically a faculty member or instructor).' Ends in a 10-minute video judged by at least 3 judges. Needs a faculty coach.</t>
+          <t>Verified 2026-09-30: 'For interns: anyone who will be registered in an accredited 4 year university post-internship.' Fintech SWE internships posted on Ashby 'ramp'.</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="3" t="inlineStr">
         <is>
-          <t>Already watched by seo-tech</t>
+          <t>Already watched by reufinder-freshmen</t>
         </is>
       </c>
       <c r="B68" s="3" t="inlineStr">
         <is>
-          <t>SEO Tech Developer + First-Year Academy</t>
+          <t>REU Finder - freshman-eligible filter</t>
         </is>
       </c>
       <c r="C68" s="3" t="inlineStr">
         <is>
-          <t>Tech internship</t>
-        </is>
-      </c>
-      <c r="D68" s="5" t="inlineStr">
-        <is>
-          <t>CHECK</t>
+          <t>Research / math</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
       <c r="E68" s="4" t="inlineStr">
         <is>
-          <t>https://tech.seo-usa.org/</t>
-        </is>
-      </c>
-      <c r="F68" s="3" t="inlineStr">
-        <is>
-          <t>Verified 2026-09-26: 'Enrolled as a sophomore'; the Academy is for 'first-year college students'. Page says 'All are welcome to apply'; SEO is a diversity organisation, so confirm eligibility by hand.</t>
-        </is>
-      </c>
+          <t>https://reufinder.com/programs-for-freshmen/</t>
+        </is>
+      </c>
+      <c r="F68" s="3" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" s="3" t="inlineStr">
         <is>
-          <t>Already watched by sfi-ucr</t>
+          <t>Already watched by sandia-students</t>
         </is>
       </c>
       <c r="B69" s="3" t="inlineStr">
         <is>
-          <t>SFI Undergraduate Complexity Research</t>
+          <t>Sandia National Laboratories student internships</t>
         </is>
       </c>
       <c r="C69" s="3" t="inlineStr">
@@ -13878,61 +13878,61 @@
       </c>
       <c r="E69" s="4" t="inlineStr">
         <is>
-          <t>https://www.santafe.edu/engage/learn/programs/undergraduate-complexity-research</t>
+          <t>https://www.sandia.gov/careers/careers/students-and-postdocs/</t>
         </is>
       </c>
       <c r="F69" s="3" t="inlineStr">
         <is>
-          <t>Verified 2026-09-26: 'for current undergraduate students. Prior research experience is not required'; 'return to this page in November 2026'.</t>
+          <t>Undergraduate and graduate internships across Sandia's sites.</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="3" t="inlineStr">
         <is>
-          <t>Already watched by simplify-2027</t>
+          <t>Already watched by scudem</t>
         </is>
       </c>
       <c r="B70" s="3" t="inlineStr">
         <is>
-          <t>SimplifyJobs Summer 2027 Internships</t>
+          <t>SCUDEM XI 2026</t>
         </is>
       </c>
       <c r="C70" s="3" t="inlineStr">
         <is>
-          <t>Tracker / resource</t>
-        </is>
-      </c>
-      <c r="D70" s="6" t="inlineStr">
-        <is>
-          <t>LOW VALUE</t>
+          <t>Competition</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
       <c r="E70" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/SimplifyJobs/Summer2027-Internships</t>
+          <t>https://www.contest.comap.com/scudem/index.html</t>
         </is>
       </c>
       <c r="F70" s="3" t="inlineStr">
         <is>
-          <t>613 roles, 94 quant, but no class-year tagging and almost all target penultimate-year students.</t>
+          <t>Verified 2026-09-30: COMAP's differential-equations modelling challenge. FAQ: 'open to teams of 3 undergraduate or high school students. Each team must have a coach (typically a faculty member or instructor).' Ends in a 10-minute video judged by at least 3 judges. Needs a faculty coach.</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="3" t="inlineStr">
         <is>
-          <t>Already watched by smart-scholarship</t>
+          <t>Already watched by seo-tech</t>
         </is>
       </c>
       <c r="B71" s="3" t="inlineStr">
         <is>
-          <t>SMART Scholarship</t>
+          <t>SEO Tech Developer + First-Year Academy</t>
         </is>
       </c>
       <c r="C71" s="3" t="inlineStr">
         <is>
-          <t>Conference / other</t>
+          <t>Tech internship</t>
         </is>
       </c>
       <c r="D71" s="5" t="inlineStr">
@@ -13942,29 +13942,29 @@
       </c>
       <c r="E71" s="4" t="inlineStr">
         <is>
-          <t>https://www.smartscholarship.org/smart</t>
+          <t>https://tech.seo-usa.org/</t>
         </is>
       </c>
       <c r="F71" s="3" t="inlineStr">
         <is>
-          <t>Verified 2026-09-26: scholarship-for-service - requires civilian employment with the Department of War after graduation. 'open annually from August 1 to the first Friday in December'.</t>
+          <t>Verified 2026-09-26: 'Enrolled as a sophomore'; the Academy is for 'first-year college students'. Page says 'All are welcome to apply'; SEO is a diversity organisation, so confirm eligibility by hand.</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="3" t="inlineStr">
         <is>
-          <t>Already watched by stevens-high-frequency-trading</t>
+          <t>Already watched by sfi-ucr</t>
         </is>
       </c>
       <c r="B72" s="3" t="inlineStr">
         <is>
-          <t>Stevens High Frequency Trading Competition 2026</t>
+          <t>SFI Undergraduate Complexity Research</t>
         </is>
       </c>
       <c r="C72" s="3" t="inlineStr">
         <is>
-          <t>Competition</t>
+          <t>Research / math</t>
         </is>
       </c>
       <c r="D72" s="5" t="inlineStr">
@@ -13974,61 +13974,61 @@
       </c>
       <c r="E72" s="4" t="inlineStr">
         <is>
-          <t>https://www.stevens.edu/page-basic/2026-stevens-high-frequency-trading-competition</t>
+          <t>https://www.santafe.edu/engage/learn/programs/undergraduate-complexity-research</t>
         </is>
       </c>
       <c r="F72" s="3" t="inlineStr">
         <is>
-          <t>HFT-focused student competition at Stevens Institute (Hoboken NJ). Christina Qi's 2026 quant competitions &amp; events list (LinkedIn Pulse), read 2026-09-06. Directly relevant to quant dev; verify class-year eligibility.</t>
+          <t>Verified 2026-09-26: 'for current undergraduate students. Prior research experience is not required'; 'return to this page in November 2026'.</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="3" t="inlineStr">
         <is>
-          <t>Already watched by surim-apply</t>
+          <t>Already watched by simplify-2027</t>
         </is>
       </c>
       <c r="B73" s="3" t="inlineStr">
         <is>
-          <t>Stanford SURIM</t>
+          <t>SimplifyJobs Summer 2027 Internships</t>
         </is>
       </c>
       <c r="C73" s="3" t="inlineStr">
         <is>
-          <t>Stanford-only</t>
-        </is>
-      </c>
-      <c r="D73" s="2" t="inlineStr">
-        <is>
-          <t>YES</t>
+          <t>Tracker / resource</t>
+        </is>
+      </c>
+      <c r="D73" s="6" t="inlineStr">
+        <is>
+          <t>LOW VALUE</t>
         </is>
       </c>
       <c r="E73" s="4" t="inlineStr">
         <is>
-          <t>https://mathematics.stanford.edu/</t>
+          <t>https://github.com/SimplifyJobs/Summer2027-Internships</t>
         </is>
       </c>
       <c r="F73" s="3" t="inlineStr">
         <is>
-          <t>8 weeks, $8,500 + up to $1,500 need-based. Needs MATH 56/61CM/61DM/110/113/115 first, and 2 letters (1 from Stanford Math). | Checked 2026-09-26: SURIM has its own page at surim.stanford.edu/apply-surim, which is watched; the listed mathematics.stanford.edu is kept.</t>
+          <t>613 roles, 94 quant, but no class-year tagging and almost all target penultimate-year students.</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="3" t="inlineStr">
         <is>
-          <t>Already watched by treehacks</t>
+          <t>Already watched by smart-scholarship</t>
         </is>
       </c>
       <c r="B74" s="3" t="inlineStr">
         <is>
-          <t>TreeHacks</t>
+          <t>SMART Scholarship</t>
         </is>
       </c>
       <c r="C74" s="3" t="inlineStr">
         <is>
-          <t>Competition</t>
+          <t>Conference / other</t>
         </is>
       </c>
       <c r="D74" s="5" t="inlineStr">
@@ -14038,61 +14038,61 @@
       </c>
       <c r="E74" s="4" t="inlineStr">
         <is>
-          <t>https://treehacks.com/</t>
+          <t>https://www.smartscholarship.org/smart</t>
         </is>
       </c>
       <c r="F74" s="3" t="inlineStr">
         <is>
-          <t>Verified 2026-09-26: 'open to any enrolled college student'; Stanford students get priority by the priority deadline.</t>
+          <t>Verified 2026-09-26: scholarship-for-service - requires civilian employment with the Department of War after graduation. 'open annually from August 1 to the first Friday in December'.</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="3" t="inlineStr">
         <is>
-          <t>Already watched by twosigma-campus</t>
+          <t>Already watched by stevens-high-frequency-trading</t>
         </is>
       </c>
       <c r="B75" s="3" t="inlineStr">
         <is>
-          <t>Two Sigma New Seekers Summit</t>
+          <t>Stevens High Frequency Trading Competition 2026</t>
         </is>
       </c>
       <c r="C75" s="3" t="inlineStr">
         <is>
-          <t>Quant firm program</t>
-        </is>
-      </c>
-      <c r="D75" s="2" t="inlineStr">
-        <is>
-          <t>YES</t>
+          <t>Competition</t>
+        </is>
+      </c>
+      <c r="D75" s="5" t="inlineStr">
+        <is>
+          <t>CHECK</t>
         </is>
       </c>
       <c r="E75" s="4" t="inlineStr">
         <is>
-          <t>https://www.twosigma.com/new-seekers-summit/</t>
+          <t>https://www.stevens.edu/page-basic/2026-stevens-high-frequency-trading-competition</t>
         </is>
       </c>
       <c r="F75" s="3" t="inlineStr">
         <is>
-          <t>Verified 2026-09-30: 'gives first-and second-year undergraduates the opportunity to delve into the world of Data Scientists and Quantitative Researchers.' QR seminars, networking, interview prep. www.twosigma.com is WP Engine, which 403s the Actions runner, so it is not watched as page_text; the posting should appear on twosigma-campus (Avature).</t>
+          <t>HFT-focused student competition at Stevens Institute (Hoboken NJ). Christina Qi's 2026 quant competitions &amp; events list (LinkedIn Pulse), read 2026-09-06. Directly relevant to quant dev; verify class-year eligibility.</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="3" t="inlineStr">
         <is>
-          <t>Already watched by uchicago-trading-competition</t>
+          <t>Already watched by surim-apply</t>
         </is>
       </c>
       <c r="B76" s="3" t="inlineStr">
         <is>
-          <t>UChicago Trading Competition</t>
+          <t>Stanford SURIM</t>
         </is>
       </c>
       <c r="C76" s="3" t="inlineStr">
         <is>
-          <t>Competition</t>
+          <t>Stanford-only</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
@@ -14102,93 +14102,93 @@
       </c>
       <c r="E76" s="4" t="inlineStr">
         <is>
-          <t>https://tradingcompetition.uchicago.edu/</t>
+          <t>https://mathematics.stanford.edu/</t>
         </is>
       </c>
       <c r="F76" s="3" t="inlineStr">
         <is>
-          <t>PRIORITY TO TEAMS WITHOUT PRIOR TRADING WORK EXPERIENCE - structurally favors freshmen. April event, $15k+ prizes.</t>
+          <t>8 weeks, $8,500 + up to $1,500 need-based. Needs MATH 56/61CM/61DM/110/113/115 first, and 2 letters (1 from Stanford Math). | Checked 2026-09-26: SURIM has its own page at surim.stanford.edu/apply-surim, which is watched; the listed mathematics.stanford.edu is kept.</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="3" t="inlineStr">
         <is>
-          <t>Already watched by underclassmen-cruz</t>
+          <t>Already watched by treehacks</t>
         </is>
       </c>
       <c r="B77" s="3" t="inlineStr">
         <is>
-          <t>underclassmen-opportunities (Cruz-Lopez)</t>
+          <t>TreeHacks</t>
         </is>
       </c>
       <c r="C77" s="3" t="inlineStr">
         <is>
-          <t>Tracker / resource</t>
-        </is>
-      </c>
-      <c r="D77" s="2" t="inlineStr">
-        <is>
-          <t>USE WEEKLY</t>
+          <t>Competition</t>
+        </is>
+      </c>
+      <c r="D77" s="5" t="inlineStr">
+        <is>
+          <t>CHECK</t>
         </is>
       </c>
       <c r="E77" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/Jose-Gael-Cruz-Lopez/underclassmen-opportunities</t>
+          <t>https://treehacks.com/</t>
         </is>
       </c>
       <c r="F77" s="3" t="inlineStr">
         <is>
-          <t>Better maintained than zapplyjobs, with open/closing-soon flags. Heavy on ambassador programs - filter hard.</t>
+          <t>Verified 2026-09-26: 'open to any enrolled college student'; Stanford students get priority by the priority deadline.</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="3" t="inlineStr">
         <is>
-          <t>Already watched by usc-ict-summer</t>
+          <t>Already watched by twosigma-campus</t>
         </is>
       </c>
       <c r="B78" s="3" t="inlineStr">
         <is>
-          <t>USC ICT Summer Research Program</t>
+          <t>Two Sigma New Seekers Summit</t>
         </is>
       </c>
       <c r="C78" s="3" t="inlineStr">
         <is>
-          <t>Research / math</t>
-        </is>
-      </c>
-      <c r="D78" s="5" t="inlineStr">
-        <is>
-          <t>CHECK</t>
+          <t>Quant firm program</t>
+        </is>
+      </c>
+      <c r="D78" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
       <c r="E78" s="4" t="inlineStr">
         <is>
-          <t>https://ict.usc.edu/careers/internships/summer-research-program-application/</t>
+          <t>https://www.twosigma.com/new-seekers-summit/</t>
         </is>
       </c>
       <c r="F78" s="3" t="inlineStr">
         <is>
-          <t>USC Institute for Creative Technologies summer research programme.</t>
+          <t>Verified 2026-09-30: 'gives first-and second-year undergraduates the opportunity to delve into the world of Data Scientists and Quantitative Researchers.' QR seminars, networking, interview prep. www.twosigma.com is WP Engine, which 403s the Actions runner, so it is not watched as page_text; the posting should appear on twosigma-campus (Avature).</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="3" t="inlineStr">
         <is>
-          <t>Already watched by worldquant-iqc</t>
+          <t>Already watched by uchicago-trading-competition</t>
         </is>
       </c>
       <c r="B79" s="3" t="inlineStr">
         <is>
-          <t>WorldQuant IQC / BRAIN</t>
+          <t>UChicago Trading Competition</t>
         </is>
       </c>
       <c r="C79" s="3" t="inlineStr">
         <is>
-          <t>Quant firm program</t>
+          <t>Competition</t>
         </is>
       </c>
       <c r="D79" s="2" t="inlineStr">
@@ -14198,88 +14198,88 @@
       </c>
       <c r="E79" s="4" t="inlineStr">
         <is>
-          <t>https://www.worldquant.com/brain/iqc/</t>
+          <t>https://tradingcompetition.uchicago.edu/</t>
         </is>
       </c>
       <c r="F79" s="3" t="inlineStr">
         <is>
-          <t>Teams of 1-4 from one university. $100k pool. Solo entry allowed. Huge field (140k+ registrations) so mid-table means little.</t>
+          <t>PRIORITY TO TEAMS WITHOUT PRIOR TRADING WORK EXPERIENCE - structurally favors freshmen. April event, $15k+ prizes.</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="3" t="inlineStr">
         <is>
-          <t>Already watched by yutc</t>
+          <t>Already watched by underclassmen-cruz</t>
         </is>
       </c>
       <c r="B80" s="3" t="inlineStr">
         <is>
-          <t>Yale Undergraduate Trading Competition</t>
+          <t>underclassmen-opportunities (Cruz-Lopez)</t>
         </is>
       </c>
       <c r="C80" s="3" t="inlineStr">
         <is>
-          <t>Competition</t>
+          <t>Tracker / resource</t>
         </is>
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>USE WEEKLY</t>
         </is>
       </c>
       <c r="E80" s="4" t="inlineStr">
         <is>
-          <t>https://www.yale.edu/</t>
+          <t>https://github.com/Jose-Gael-Cruz-Lopez/underclassmen-opportunities</t>
         </is>
       </c>
       <c r="F80" s="3" t="inlineStr">
         <is>
-          <t>$10,000+ in prizes, nationwide. | Checked 2026-09-26: the competition's own site is yutc.org (a JavaScript page, watched with render_js); the listed yale.edu is kept.</t>
+          <t>Better maintained than zapplyjobs, with open/closing-soon flags. Heavy on ambassador programs - filter hard.</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="3" t="inlineStr">
         <is>
-          <t>You cannot apply (NO)</t>
+          <t>Already watched by usc-ict-summer</t>
         </is>
       </c>
       <c r="B81" s="3" t="inlineStr">
         <is>
-          <t>Bank of America APAC Quant Conference</t>
+          <t>USC ICT Summer Research Program</t>
         </is>
       </c>
       <c r="C81" s="3" t="inlineStr">
         <is>
-          <t>Conference / other</t>
-        </is>
-      </c>
-      <c r="D81" s="8" t="inlineStr">
-        <is>
-          <t>NO</t>
+          <t>Research / math</t>
+        </is>
+      </c>
+      <c r="D81" s="5" t="inlineStr">
+        <is>
+          <t>CHECK</t>
         </is>
       </c>
       <c r="E81" s="4" t="inlineStr">
         <is>
-          <t>https://www.bofa.com/</t>
+          <t>https://ict.usc.edu/careers/internships/summer-research-program-application/</t>
         </is>
       </c>
       <c r="F81" s="3" t="inlineStr">
         <is>
-          <t>Ruled out on geography - APAC, May 20 2026. Christina Qi's 2026 quant competitions &amp; events list (LinkedIn Pulse), read 2026-09-06.</t>
+          <t>USC Institute for Creative Technologies summer research programme.</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="3" t="inlineStr">
         <is>
-          <t>You cannot apply (NO)</t>
+          <t>Already watched by worldquant-iqc</t>
         </is>
       </c>
       <c r="B82" s="3" t="inlineStr">
         <is>
-          <t>Bridgewater Rising Fellows</t>
+          <t>WorldQuant IQC / BRAIN</t>
         </is>
       </c>
       <c r="C82" s="3" t="inlineStr">
@@ -14287,51 +14287,51 @@
           <t>Quant firm program</t>
         </is>
       </c>
-      <c r="D82" s="8" t="inlineStr">
-        <is>
-          <t>NO</t>
+      <c r="D82" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
       <c r="E82" s="4" t="inlineStr">
         <is>
-          <t>https://www.bridgewater.com/risingfellowsprogram</t>
+          <t>https://www.worldquant.com/brain/iqc/</t>
         </is>
       </c>
       <c r="F82" s="3" t="inlineStr">
         <is>
-          <t>CORRECTED: first-year eligible BUT targets backgrounds underrepresented in the industry, recruiting via HBCUs, O4U, BLK Capital, Prep for Prep. | Checked 2026-09-26: now redirects to the generic /working-at-bridgewater page. Kept: it may reopen.</t>
+          <t>Teams of 1-4 from one university. $100k pool. Solo entry allowed. Huge field (140k+ registrations) so mid-table means little.</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="3" t="inlineStr">
         <is>
-          <t>You cannot apply (NO)</t>
+          <t>Already watched by yutc</t>
         </is>
       </c>
       <c r="B83" s="3" t="inlineStr">
         <is>
-          <t>CQA Young Professionals Event</t>
+          <t>Yale Undergraduate Trading Competition</t>
         </is>
       </c>
       <c r="C83" s="3" t="inlineStr">
         <is>
-          <t>Conference / other</t>
-        </is>
-      </c>
-      <c r="D83" s="8" t="inlineStr">
-        <is>
-          <t>NO</t>
+          <t>Competition</t>
+        </is>
+      </c>
+      <c r="D83" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
       <c r="E83" s="4" t="inlineStr">
         <is>
-          <t>https://cqa.org/upcoming-events-cqa-young-professional</t>
+          <t>https://www.yale.edu/</t>
         </is>
       </c>
       <c r="F83" s="3" t="inlineStr">
         <is>
-          <t>Ruled out on stage - for working professionals, not undergraduates. Christina Qi's 2026 quant competitions &amp; events list (LinkedIn Pulse), read 2026-09-06.</t>
+          <t>$10,000+ in prizes, nationwide. | Checked 2026-09-26: the competition's own site is yutc.org (a JavaScript page, watched with render_js); the listed yale.edu is kept.</t>
         </is>
       </c>
     </row>
@@ -14343,12 +14343,12 @@
       </c>
       <c r="B84" s="3" t="inlineStr">
         <is>
-          <t>Citadel Securities Ignite</t>
+          <t>Bank of America APAC Quant Conference</t>
         </is>
       </c>
       <c r="C84" s="3" t="inlineStr">
         <is>
-          <t>Quant firm program</t>
+          <t>Conference / other</t>
         </is>
       </c>
       <c r="D84" s="8" t="inlineStr">
@@ -14358,12 +14358,12 @@
       </c>
       <c r="E84" s="4" t="inlineStr">
         <is>
-          <t>https://www.citadelsecurities.com/careers/programs-and-events/</t>
+          <t>https://www.bofa.com/</t>
         </is>
       </c>
       <c r="F84" s="3" t="inlineStr">
         <is>
-          <t>Invite-only weeklong program for sophomore women.</t>
+          <t>Ruled out on geography - APAC, May 20 2026. Christina Qi's 2026 quant competitions &amp; events list (LinkedIn Pulse), read 2026-09-06.</t>
         </is>
       </c>
     </row>
@@ -14375,12 +14375,12 @@
       </c>
       <c r="B85" s="3" t="inlineStr">
         <is>
-          <t>Coding it Forward - Civic Digital Fellowship</t>
+          <t>Bridgewater Rising Fellows</t>
         </is>
       </c>
       <c r="C85" s="3" t="inlineStr">
         <is>
-          <t>Tech internship</t>
+          <t>Quant firm program</t>
         </is>
       </c>
       <c r="D85" s="8" t="inlineStr">
@@ -14390,12 +14390,12 @@
       </c>
       <c r="E85" s="4" t="inlineStr">
         <is>
-          <t>https://www.codingitforward.com/fellowship</t>
+          <t>https://www.bridgewater.com/risingfellowsprogram</t>
         </is>
       </c>
       <c r="F85" s="3" t="inlineStr">
         <is>
-          <t>TRAP - appears on most underclassmen lists but 2026 required graduating May 2025-Dec 2027. Diary for junior year.</t>
+          <t>CORRECTED: first-year eligible BUT targets backgrounds underrepresented in the industry, recruiting via HBCUs, O4U, BLK Capital, Prep for Prep. | Checked 2026-09-26: now redirects to the generic /working-at-bridgewater page. Kept: it may reopen.</t>
         </is>
       </c>
     </row>
@@ -14407,12 +14407,12 @@
       </c>
       <c r="B86" s="3" t="inlineStr">
         <is>
-          <t>D. E. Shaw Discovery Fellowship</t>
+          <t>CQA Young Professionals Event</t>
         </is>
       </c>
       <c r="C86" s="3" t="inlineStr">
         <is>
-          <t>Quant firm program</t>
+          <t>Conference / other</t>
         </is>
       </c>
       <c r="D86" s="8" t="inlineStr">
@@ -14422,12 +14422,12 @@
       </c>
       <c r="E86" s="4" t="inlineStr">
         <is>
-          <t>https://campus.deshaw.com/fellowships</t>
+          <t>https://cqa.org/upcoming-events-cqa-young-professional</t>
         </is>
       </c>
       <c r="F86" s="3" t="inlineStr">
         <is>
-          <t>Checked 2026-09-26: campus.deshaw.com/fellowships now redirects to the campus root, which mentions no fellowships. Kept; the root is watched as deshaw-campus.</t>
+          <t>Ruled out on stage - for working professionals, not undergraduates. Christina Qi's 2026 quant competitions &amp; events list (LinkedIn Pulse), read 2026-09-06.</t>
         </is>
       </c>
     </row>
@@ -14439,7 +14439,7 @@
       </c>
       <c r="B87" s="3" t="inlineStr">
         <is>
-          <t>D. E. Shaw Latitude Fellowship</t>
+          <t>Citadel Securities Ignite</t>
         </is>
       </c>
       <c r="C87" s="3" t="inlineStr">
@@ -14454,12 +14454,12 @@
       </c>
       <c r="E87" s="4" t="inlineStr">
         <is>
-          <t>https://campus.deshaw.com/fellowships</t>
+          <t>https://www.citadelsecurities.com/careers/programs-and-events/</t>
         </is>
       </c>
       <c r="F87" s="3" t="inlineStr">
         <is>
-          <t>Checked 2026-09-26: campus.deshaw.com/fellowships now redirects to the campus root, which mentions no fellowships. Kept; the root is watched as deshaw-campus.</t>
+          <t>Invite-only weeklong program for sophomore women.</t>
         </is>
       </c>
     </row>
@@ -14471,12 +14471,12 @@
       </c>
       <c r="B88" s="3" t="inlineStr">
         <is>
-          <t>D. E. Shaw London Insight Programme</t>
+          <t>Coding it Forward - Civic Digital Fellowship</t>
         </is>
       </c>
       <c r="C88" s="3" t="inlineStr">
         <is>
-          <t>Quant firm program</t>
+          <t>Tech internship</t>
         </is>
       </c>
       <c r="D88" s="8" t="inlineStr">
@@ -14486,12 +14486,12 @@
       </c>
       <c r="E88" s="4" t="inlineStr">
         <is>
-          <t>https://campus.deshaw.com/additional-experiences</t>
+          <t>https://www.codingitforward.com/fellowship</t>
         </is>
       </c>
       <c r="F88" s="3" t="inlineStr">
         <is>
-          <t>Ruled out on geography - London. Christina Qi's 2026 quant competitions &amp; events list (LinkedIn Pulse), read 2026-09-06. | Checked 2026-09-26: campus.deshaw.com/additional-experiences now redirects to the campus root (which lists London Insight as closed). Kept.</t>
+          <t>TRAP - appears on most underclassmen lists but 2026 required graduating May 2025-Dec 2027. Diary for junior year.</t>
         </is>
       </c>
     </row>
@@ -14503,7 +14503,7 @@
       </c>
       <c r="B89" s="3" t="inlineStr">
         <is>
-          <t>D. E. Shaw Momentum Fellowship</t>
+          <t>D. E. Shaw Discovery Fellowship</t>
         </is>
       </c>
       <c r="C89" s="3" t="inlineStr">
@@ -14535,12 +14535,12 @@
       </c>
       <c r="B90" s="3" t="inlineStr">
         <is>
-          <t>Databento partner quant events (Shanghai, London)</t>
+          <t>D. E. Shaw Latitude Fellowship</t>
         </is>
       </c>
       <c r="C90" s="3" t="inlineStr">
         <is>
-          <t>Conference / other</t>
+          <t>Quant firm program</t>
         </is>
       </c>
       <c r="D90" s="8" t="inlineStr">
@@ -14550,12 +14550,12 @@
       </c>
       <c r="E90" s="4" t="inlineStr">
         <is>
-          <t>https://databento.com/</t>
+          <t>https://campus.deshaw.com/fellowships</t>
         </is>
       </c>
       <c r="F90" s="3" t="inlineStr">
         <is>
-          <t>Consolidated row for the Databento events with Nasdaq/Bank of America (Shanghai, May 21 2026), Google (London, June 2026) and Man Group (London, June 2026). Ruled out on geography. Christina Qi's 2026 quant competitions &amp; events list (LinkedIn Pulse), read 2026-09-06.</t>
+          <t>Checked 2026-09-26: campus.deshaw.com/fellowships now redirects to the campus root, which mentions no fellowships. Kept; the root is watched as deshaw-campus.</t>
         </is>
       </c>
     </row>
@@ -14567,12 +14567,12 @@
       </c>
       <c r="B91" s="3" t="inlineStr">
         <is>
-          <t>Global Crypto Quant Competition and Digital Asset Forum Hong Kong 2026</t>
+          <t>D. E. Shaw London Insight Programme</t>
         </is>
       </c>
       <c r="C91" s="3" t="inlineStr">
         <is>
-          <t>Competition</t>
+          <t>Quant firm program</t>
         </is>
       </c>
       <c r="D91" s="8" t="inlineStr">
@@ -14582,12 +14582,12 @@
       </c>
       <c r="E91" s="4" t="inlineStr">
         <is>
-          <t>https://en.tmtpost.com/post/7752441</t>
+          <t>https://campus.deshaw.com/additional-experiences</t>
         </is>
       </c>
       <c r="F91" s="3" t="inlineStr">
         <is>
-          <t>Ruled out on geography - Hong Kong. Christina Qi's 2026 quant competitions &amp; events list (LinkedIn Pulse), read 2026-09-06.</t>
+          <t>Ruled out on geography - London. Christina Qi's 2026 quant competitions &amp; events list (LinkedIn Pulse), read 2026-09-06. | Checked 2026-09-26: campus.deshaw.com/additional-experiences now redirects to the campus root (which lists London Insight as closed). Kept.</t>
         </is>
       </c>
     </row>
@@ -14599,7 +14599,7 @@
       </c>
       <c r="B92" s="3" t="inlineStr">
         <is>
-          <t>IMC EU Business Course</t>
+          <t>D. E. Shaw Momentum Fellowship</t>
         </is>
       </c>
       <c r="C92" s="3" t="inlineStr">
@@ -14614,12 +14614,12 @@
       </c>
       <c r="E92" s="4" t="inlineStr">
         <is>
-          <t>https://www.imc.com/eu/careers/students-graduates/programs/business-course</t>
+          <t>https://campus.deshaw.com/fellowships</t>
         </is>
       </c>
       <c r="F92" s="3" t="inlineStr">
         <is>
-          <t>Ruled out on geography - EU. The US Launchpad program is tracked separately. Christina Qi's 2026 quant competitions &amp; events list (LinkedIn Pulse), read 2026-09-06.</t>
+          <t>Checked 2026-09-26: campus.deshaw.com/fellowships now redirects to the campus root, which mentions no fellowships. Kept; the root is watched as deshaw-campus.</t>
         </is>
       </c>
     </row>
@@ -14631,12 +14631,12 @@
       </c>
       <c r="B93" s="3" t="inlineStr">
         <is>
-          <t>IMC UK Masterclass</t>
+          <t>Databento partner quant events (Shanghai, London)</t>
         </is>
       </c>
       <c r="C93" s="3" t="inlineStr">
         <is>
-          <t>Quant firm program</t>
+          <t>Conference / other</t>
         </is>
       </c>
       <c r="D93" s="8" t="inlineStr">
@@ -14646,12 +14646,12 @@
       </c>
       <c r="E93" s="4" t="inlineStr">
         <is>
-          <t>https://careers.imc.com/</t>
+          <t>https://databento.com/</t>
         </is>
       </c>
       <c r="F93" s="3" t="inlineStr">
         <is>
-          <t>Geographic exclusion - excludes US-based students.</t>
+          <t>Consolidated row for the Databento events with Nasdaq/Bank of America (Shanghai, May 21 2026), Google (London, June 2026) and Man Group (London, June 2026). Ruled out on geography. Christina Qi's 2026 quant competitions &amp; events list (LinkedIn Pulse), read 2026-09-06.</t>
         </is>
       </c>
     </row>
@@ -14663,12 +14663,12 @@
       </c>
       <c r="B94" s="3" t="inlineStr">
         <is>
-          <t>IMC WiT (Women in Technology)</t>
+          <t>Global Crypto Quant Competition and Digital Asset Forum Hong Kong 2026</t>
         </is>
       </c>
       <c r="C94" s="3" t="inlineStr">
         <is>
-          <t>Quant firm program</t>
+          <t>Competition</t>
         </is>
       </c>
       <c r="D94" s="8" t="inlineStr">
@@ -14678,10 +14678,14 @@
       </c>
       <c r="E94" s="4" t="inlineStr">
         <is>
-          <t>https://careers.imc.com/us/en/student-opportunities</t>
-        </is>
-      </c>
-      <c r="F94" s="3" t="inlineStr"/>
+          <t>https://en.tmtpost.com/post/7752441</t>
+        </is>
+      </c>
+      <c r="F94" s="3" t="inlineStr">
+        <is>
+          <t>Ruled out on geography - Hong Kong. Christina Qi's 2026 quant competitions &amp; events list (LinkedIn Pulse), read 2026-09-06.</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="3" t="inlineStr">
@@ -14691,7 +14695,7 @@
       </c>
       <c r="B95" s="3" t="inlineStr">
         <is>
-          <t>IMC Women in Trading and Engineering</t>
+          <t>IMC EU Business Course</t>
         </is>
       </c>
       <c r="C95" s="3" t="inlineStr">
@@ -14706,12 +14710,12 @@
       </c>
       <c r="E95" s="4" t="inlineStr">
         <is>
-          <t>https://www.imc.com/ap/careers/students-graduates/programs/womens-talent</t>
+          <t>https://www.imc.com/eu/careers/students-graduates/programs/business-course</t>
         </is>
       </c>
       <c r="F95" s="3" t="inlineStr">
         <is>
-          <t>Ruled out by an identity gate: this program is for women. Christina Qi's 2026 quant competitions &amp; events list (LinkedIn Pulse), read 2026-09-06. Listed here so it is not re-researched.</t>
+          <t>Ruled out on geography - EU. The US Launchpad program is tracked separately. Christina Qi's 2026 quant competitions &amp; events list (LinkedIn Pulse), read 2026-09-06.</t>
         </is>
       </c>
     </row>
@@ -14723,12 +14727,12 @@
       </c>
       <c r="B96" s="3" t="inlineStr">
         <is>
-          <t>JPMorgan Data for Good Hackathon</t>
+          <t>IMC UK Masterclass</t>
         </is>
       </c>
       <c r="C96" s="3" t="inlineStr">
         <is>
-          <t>Conference / other</t>
+          <t>Quant firm program</t>
         </is>
       </c>
       <c r="D96" s="8" t="inlineStr">
@@ -14738,12 +14742,12 @@
       </c>
       <c r="E96" s="4" t="inlineStr">
         <is>
-          <t>https://careers.jpmorgan.com/</t>
+          <t>https://careers.imc.com/</t>
         </is>
       </c>
       <c r="F96" s="3" t="inlineStr">
         <is>
-          <t>That is a junior-year window; a first-year does not qualify.</t>
+          <t>Geographic exclusion - excludes US-based students.</t>
         </is>
       </c>
     </row>
@@ -14755,7 +14759,7 @@
       </c>
       <c r="B97" s="3" t="inlineStr">
         <is>
-          <t>Jane Street FOCUS and IN FOCUS</t>
+          <t>IMC WiT (Women in Technology)</t>
         </is>
       </c>
       <c r="C97" s="3" t="inlineStr">
@@ -14770,14 +14774,10 @@
       </c>
       <c r="E97" s="4" t="inlineStr">
         <is>
-          <t>https://www.janestreet.com/join-jane-street/programs-and-events/</t>
-        </is>
-      </c>
-      <c r="F97" s="3" t="inlineStr">
-        <is>
-          <t>Barriers-to-access criteria (first-gen, Pell-eligible, under-resourced school). Read criteria yourself.</t>
-        </is>
-      </c>
+          <t>https://careers.imc.com/us/en/student-opportunities</t>
+        </is>
+      </c>
+      <c r="F97" s="3" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" s="3" t="inlineStr">
@@ -14787,7 +14787,7 @@
       </c>
       <c r="B98" s="3" t="inlineStr">
         <is>
-          <t>Jane Street Graduate Research Fellowship</t>
+          <t>IMC Women in Trading and Engineering</t>
         </is>
       </c>
       <c r="C98" s="3" t="inlineStr">
@@ -14802,10 +14802,14 @@
       </c>
       <c r="E98" s="4" t="inlineStr">
         <is>
-          <t>https://www.janestreet.com/join-jane-street/programs-and-events/</t>
-        </is>
-      </c>
-      <c r="F98" s="3" t="inlineStr"/>
+          <t>https://www.imc.com/ap/careers/students-graduates/programs/womens-talent</t>
+        </is>
+      </c>
+      <c r="F98" s="3" t="inlineStr">
+        <is>
+          <t>Ruled out by an identity gate: this program is for women. Christina Qi's 2026 quant competitions &amp; events list (LinkedIn Pulse), read 2026-09-06. Listed here so it is not re-researched.</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="3" t="inlineStr">
@@ -14815,12 +14819,12 @@
       </c>
       <c r="B99" s="3" t="inlineStr">
         <is>
-          <t>Jane Street INSIGHT</t>
+          <t>JPMorgan Data for Good Hackathon</t>
         </is>
       </c>
       <c r="C99" s="3" t="inlineStr">
         <is>
-          <t>Quant firm program</t>
+          <t>Conference / other</t>
         </is>
       </c>
       <c r="D99" s="8" t="inlineStr">
@@ -14830,12 +14834,12 @@
       </c>
       <c r="E99" s="4" t="inlineStr">
         <is>
-          <t>https://www.janestreet.com/join-jane-street/programs-and-events/insight/</t>
+          <t>https://careers.jpmorgan.com/</t>
         </is>
       </c>
       <c r="F99" s="3" t="inlineStr">
         <is>
-          <t>For women, transgender and gender-expansive people.</t>
+          <t>That is a junior-year window; a first-year does not qualify.</t>
         </is>
       </c>
     </row>
@@ -14847,7 +14851,7 @@
       </c>
       <c r="B100" s="3" t="inlineStr">
         <is>
-          <t>Jane Street JSIP</t>
+          <t>Jane Street FOCUS and IN FOCUS</t>
         </is>
       </c>
       <c r="C100" s="3" t="inlineStr">
@@ -14862,12 +14866,12 @@
       </c>
       <c r="E100" s="4" t="inlineStr">
         <is>
-          <t>https://www.janestreet.com/join-jane-street/programs-and-events/jsip/</t>
+          <t>https://www.janestreet.com/join-jane-street/programs-and-events/</t>
         </is>
       </c>
       <c r="F100" s="3" t="inlineStr">
         <is>
-          <t>Multi-week paid NYC program, $12,500 scholarship - but requires having experienced barriers to access in CS. | Checked 2026-09-26: now redirects to the programs-and-events index, which does not list JSIP. Kept: it may reopen for the next cycle.</t>
+          <t>Barriers-to-access criteria (first-gen, Pell-eligible, under-resourced school). Read criteria yourself.</t>
         </is>
       </c>
     </row>
@@ -14879,7 +14883,7 @@
       </c>
       <c r="B101" s="3" t="inlineStr">
         <is>
-          <t>Jane Street Visiting Researcher / Prefaculty</t>
+          <t>Jane Street Graduate Research Fellowship</t>
         </is>
       </c>
       <c r="C101" s="3" t="inlineStr">
@@ -14907,7 +14911,7 @@
       </c>
       <c r="B102" s="3" t="inlineStr">
         <is>
-          <t>Jane Street WiSE</t>
+          <t>Jane Street INSIGHT</t>
         </is>
       </c>
       <c r="C102" s="3" t="inlineStr">
@@ -14922,12 +14926,12 @@
       </c>
       <c r="E102" s="4" t="inlineStr">
         <is>
-          <t>https://www.janestreet.com/join-jane-street/programs-and-events/</t>
+          <t>https://www.janestreet.com/join-jane-street/programs-and-events/insight/</t>
         </is>
       </c>
       <c r="F102" s="3" t="inlineStr">
         <is>
-          <t>Women / trans / gender-expansive students.</t>
+          <t>For women, transgender and gender-expansive people.</t>
         </is>
       </c>
     </row>
@@ -14939,12 +14943,12 @@
       </c>
       <c r="B103" s="3" t="inlineStr">
         <is>
-          <t>KNHack 2026 Research Challenge (Mexico)</t>
+          <t>Jane Street JSIP</t>
         </is>
       </c>
       <c r="C103" s="3" t="inlineStr">
         <is>
-          <t>Competition</t>
+          <t>Quant firm program</t>
         </is>
       </c>
       <c r="D103" s="8" t="inlineStr">
@@ -14954,12 +14958,12 @@
       </c>
       <c r="E103" s="4" t="inlineStr">
         <is>
-          <t>https://kaxanuk.mx/kn-hack</t>
+          <t>https://www.janestreet.com/join-jane-street/programs-and-events/jsip/</t>
         </is>
       </c>
       <c r="F103" s="3" t="inlineStr">
         <is>
-          <t>Ruled out on geography - Mexico. Christina Qi's 2026 quant competitions &amp; events list (LinkedIn Pulse), read 2026-09-06.</t>
+          <t>Multi-week paid NYC program, $12,500 scholarship - but requires having experienced barriers to access in CS. | Checked 2026-09-26: now redirects to the programs-and-events index, which does not list JSIP. Kept: it may reopen for the next cycle.</t>
         </is>
       </c>
     </row>
@@ -14971,12 +14975,12 @@
       </c>
       <c r="B104" s="3" t="inlineStr">
         <is>
-          <t>MIT Pokerbots</t>
+          <t>Jane Street Visiting Researcher / Prefaculty</t>
         </is>
       </c>
       <c r="C104" s="3" t="inlineStr">
         <is>
-          <t>Competition</t>
+          <t>Quant firm program</t>
         </is>
       </c>
       <c r="D104" s="8" t="inlineStr">
@@ -14986,14 +14990,10 @@
       </c>
       <c r="E104" s="4" t="inlineStr">
         <is>
-          <t>https://pokerbots.org/</t>
-        </is>
-      </c>
-      <c r="F104" s="3" t="inlineStr">
-        <is>
-          <t>Must be able to register for MIT IAP classes; a team member needs MIT certificates for the competition server.</t>
-        </is>
-      </c>
+          <t>https://www.janestreet.com/join-jane-street/programs-and-events/</t>
+        </is>
+      </c>
+      <c r="F104" s="3" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" s="3" t="inlineStr">
@@ -15003,12 +15003,12 @@
       </c>
       <c r="B105" s="3" t="inlineStr">
         <is>
-          <t>Meta University</t>
+          <t>Jane Street WiSE</t>
         </is>
       </c>
       <c r="C105" s="3" t="inlineStr">
         <is>
-          <t>Tech internship</t>
+          <t>Quant firm program</t>
         </is>
       </c>
       <c r="D105" s="8" t="inlineStr">
@@ -15016,14 +15016,14 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="E105" s="3" t="inlineStr">
-        <is>
-          <t>n/a</t>
+      <c r="E105" s="4" t="inlineStr">
+        <is>
+          <t>https://www.janestreet.com/join-jane-street/programs-and-events/</t>
         </is>
       </c>
       <c r="F105" s="3" t="inlineStr">
         <is>
-          <t>Discontinued with no replacement. Ignore any list that still includes it.</t>
+          <t>Women / trans / gender-expansive students.</t>
         </is>
       </c>
     </row>
@@ -15035,12 +15035,12 @@
       </c>
       <c r="B106" s="3" t="inlineStr">
         <is>
-          <t>Optiver Career Kickstarter: Women in Tech</t>
+          <t>KNHack 2026 Research Challenge (Mexico)</t>
         </is>
       </c>
       <c r="C106" s="3" t="inlineStr">
         <is>
-          <t>Quant firm program</t>
+          <t>Competition</t>
         </is>
       </c>
       <c r="D106" s="8" t="inlineStr">
@@ -15050,12 +15050,12 @@
       </c>
       <c r="E106" s="4" t="inlineStr">
         <is>
-          <t>https://optiver.com/working-at-optiver/career-opportunities/8177160002</t>
+          <t>https://kaxanuk.mx/kn-hack</t>
         </is>
       </c>
       <c r="F106" s="3" t="inlineStr">
         <is>
-          <t>Ruled out by an identity gate: this program is for women. Christina Qi's 2026 quant competitions &amp; events list (LinkedIn Pulse), read 2026-09-06. Listed here so it is not re-researched.</t>
+          <t>Ruled out on geography - Mexico. Christina Qi's 2026 quant competitions &amp; events list (LinkedIn Pulse), read 2026-09-06.</t>
         </is>
       </c>
     </row>
@@ -15067,12 +15067,12 @@
       </c>
       <c r="B107" s="3" t="inlineStr">
         <is>
-          <t>Optiver Quantitative Intern Summer 2027</t>
+          <t>MIT Pokerbots</t>
         </is>
       </c>
       <c r="C107" s="3" t="inlineStr">
         <is>
-          <t>Quant firm program</t>
+          <t>Competition</t>
         </is>
       </c>
       <c r="D107" s="8" t="inlineStr">
@@ -15082,12 +15082,12 @@
       </c>
       <c r="E107" s="4" t="inlineStr">
         <is>
-          <t>https://optiver.com/working-at-optiver/career-opportunities/</t>
+          <t>https://pokerbots.org/</t>
         </is>
       </c>
       <c r="F107" s="3" t="inlineStr">
         <is>
-          <t>Highest pay in the industry, but a first-year is too early.</t>
+          <t>Must be able to register for MIT IAP classes; a team member needs MIT certificates for the competition server.</t>
         </is>
       </c>
     </row>
@@ -15099,12 +15099,12 @@
       </c>
       <c r="B108" s="3" t="inlineStr">
         <is>
-          <t>Optiver regional recruitment events (non-US)</t>
+          <t>Meta University</t>
         </is>
       </c>
       <c r="C108" s="3" t="inlineStr">
         <is>
-          <t>Quant firm program</t>
+          <t>Tech internship</t>
         </is>
       </c>
       <c r="D108" s="8" t="inlineStr">
@@ -15112,14 +15112,14 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="E108" s="4" t="inlineStr">
-        <is>
-          <t>https://optiver.com/recruitment-events/</t>
+      <c r="E108" s="3" t="inlineStr">
+        <is>
+          <t>n/a</t>
         </is>
       </c>
       <c r="F108" s="3" t="inlineStr">
         <is>
-          <t>Consolidated row for the ANZ, China, Singapore, India, Amsterdam and Catalunya FutureFocus / Career Kickstarter / masterclass events. Ruled out on geography; the Chicago event is tracked separately. Christina Qi's 2026 quant competitions &amp; events list (LinkedIn Pulse), read 2026-09-06.</t>
+          <t>Discontinued with no replacement. Ignore any list that still includes it.</t>
         </is>
       </c>
     </row>
@@ -15131,7 +15131,7 @@
       </c>
       <c r="B109" s="3" t="inlineStr">
         <is>
-          <t>PEAK6 Trading Bootcamp</t>
+          <t>Optiver Career Kickstarter: Women in Tech</t>
         </is>
       </c>
       <c r="C109" s="3" t="inlineStr">
@@ -15146,12 +15146,12 @@
       </c>
       <c r="E109" s="4" t="inlineStr">
         <is>
-          <t>https://peak6.com/campus/</t>
+          <t>https://optiver.com/working-at-optiver/career-opportunities/8177160002</t>
         </is>
       </c>
       <c r="F109" s="3" t="inlineStr">
         <is>
-          <t>One week, $25-31.25/hr, two sessions (May and Aug).</t>
+          <t>Ruled out by an identity gate: this program is for women. Christina Qi's 2026 quant competitions &amp; events list (LinkedIn Pulse), read 2026-09-06. Listed here so it is not re-researched.</t>
         </is>
       </c>
     </row>
@@ -15163,12 +15163,12 @@
       </c>
       <c r="B110" s="3" t="inlineStr">
         <is>
-          <t>Palantir Path</t>
+          <t>Optiver Quantitative Intern Summer 2027</t>
         </is>
       </c>
       <c r="C110" s="3" t="inlineStr">
         <is>
-          <t>Tech internship</t>
+          <t>Quant firm program</t>
         </is>
       </c>
       <c r="D110" s="8" t="inlineStr">
@@ -15176,12 +15176,16 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="E110" s="3" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="F110" s="3" t="inlineStr"/>
+      <c r="E110" s="4" t="inlineStr">
+        <is>
+          <t>https://optiver.com/working-at-optiver/career-opportunities/</t>
+        </is>
+      </c>
+      <c r="F110" s="3" t="inlineStr">
+        <is>
+          <t>Highest pay in the industry, but a first-year is too early.</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="3" t="inlineStr">
@@ -15191,7 +15195,7 @@
       </c>
       <c r="B111" s="3" t="inlineStr">
         <is>
-          <t>Point72 Academy</t>
+          <t>Optiver regional recruitment events (non-US)</t>
         </is>
       </c>
       <c r="C111" s="3" t="inlineStr">
@@ -15206,12 +15210,12 @@
       </c>
       <c r="E111" s="4" t="inlineStr">
         <is>
-          <t>https://point72.com/point72-academy/</t>
+          <t>https://optiver.com/recruitment-events/</t>
         </is>
       </c>
       <c r="F111" s="3" t="inlineStr">
         <is>
-          <t>NOT an underclassman program. 10-month paid post-grad program, $125k base. 2027 class wants Dec 2026-Jul 2027 grads.</t>
+          <t>Consolidated row for the ANZ, China, Singapore, India, Amsterdam and Catalunya FutureFocus / Career Kickstarter / masterclass events. Ruled out on geography; the Chicago event is tracked separately. Christina Qi's 2026 quant competitions &amp; events list (LinkedIn Pulse), read 2026-09-06.</t>
         </is>
       </c>
     </row>
@@ -15223,7 +15227,7 @@
       </c>
       <c r="B112" s="3" t="inlineStr">
         <is>
-          <t>SIG Sophomore Discovery Days for Women (all tracks)</t>
+          <t>PEAK6 Trading Bootcamp</t>
         </is>
       </c>
       <c r="C112" s="3" t="inlineStr">
@@ -15238,10 +15242,14 @@
       </c>
       <c r="E112" s="4" t="inlineStr">
         <is>
-          <t>https://careers.sig.com/discovery-programs/jobs</t>
-        </is>
-      </c>
-      <c r="F112" s="3" t="inlineStr"/>
+          <t>https://peak6.com/campus/</t>
+        </is>
+      </c>
+      <c r="F112" s="3" t="inlineStr">
+        <is>
+          <t>One week, $25-31.25/hr, two sessions (May and Aug).</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="3" t="inlineStr">
@@ -15251,12 +15259,12 @@
       </c>
       <c r="B113" s="3" t="inlineStr">
         <is>
-          <t>Two Sigma College Mentor Connect</t>
+          <t>Palantir Path</t>
         </is>
       </c>
       <c r="C113" s="3" t="inlineStr">
         <is>
-          <t>Quant firm program</t>
+          <t>Tech internship</t>
         </is>
       </c>
       <c r="D113" s="8" t="inlineStr">
@@ -15264,16 +15272,12 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="E113" s="4" t="inlineStr">
-        <is>
-          <t>https://www.twosigma.com/undergraduate-students/</t>
-        </is>
-      </c>
-      <c r="F113" s="3" t="inlineStr">
-        <is>
-          <t>6-week remote mentorship on open-source projects.</t>
-        </is>
-      </c>
+      <c r="E113" s="3" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F113" s="3" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" s="3" t="inlineStr">
@@ -15283,7 +15287,7 @@
       </c>
       <c r="B114" s="3" t="inlineStr">
         <is>
-          <t>Two Sigma Diversity Undergraduate Scholarship</t>
+          <t>Point72 Academy</t>
         </is>
       </c>
       <c r="C114" s="3" t="inlineStr">
@@ -15298,10 +15302,14 @@
       </c>
       <c r="E114" s="4" t="inlineStr">
         <is>
-          <t>https://www.twosigma.com/undergraduate-students/</t>
-        </is>
-      </c>
-      <c r="F114" s="3" t="inlineStr"/>
+          <t>https://point72.com/point72-academy/</t>
+        </is>
+      </c>
+      <c r="F114" s="3" t="inlineStr">
+        <is>
+          <t>NOT an underclassman program. 10-month paid post-grad program, $125k base. 2027 class wants Dec 2026-Jul 2027 grads.</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="3" t="inlineStr">
@@ -15311,7 +15319,7 @@
       </c>
       <c r="B115" s="3" t="inlineStr">
         <is>
-          <t>Two Sigma PhD Fellowship</t>
+          <t>SIG Sophomore Discovery Days for Women (all tracks)</t>
         </is>
       </c>
       <c r="C115" s="3" t="inlineStr">
@@ -15326,7 +15334,7 @@
       </c>
       <c r="E115" s="4" t="inlineStr">
         <is>
-          <t>https://www.twosigma.com/graduate-students/phd-fellowships/</t>
+          <t>https://careers.sig.com/discovery-programs/jobs</t>
         </is>
       </c>
       <c r="F115" s="3" t="inlineStr"/>
@@ -15339,7 +15347,7 @@
       </c>
       <c r="B116" s="3" t="inlineStr">
         <is>
-          <t>Virtu Financial Women's Winternship</t>
+          <t>Two Sigma College Mentor Connect</t>
         </is>
       </c>
       <c r="C116" s="3" t="inlineStr">
@@ -15354,10 +15362,14 @@
       </c>
       <c r="E116" s="4" t="inlineStr">
         <is>
-          <t>https://www.virtu.com/careers/</t>
-        </is>
-      </c>
-      <c r="F116" s="3" t="inlineStr"/>
+          <t>https://www.twosigma.com/undergraduate-students/</t>
+        </is>
+      </c>
+      <c r="F116" s="3" t="inlineStr">
+        <is>
+          <t>6-week remote mentorship on open-source projects.</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="3" t="inlineStr">
@@ -15367,12 +15379,12 @@
       </c>
       <c r="B117" s="3" t="inlineStr">
         <is>
-          <t>Wharton Global High School Investment Competition</t>
+          <t>Two Sigma Diversity Undergraduate Scholarship</t>
         </is>
       </c>
       <c r="C117" s="3" t="inlineStr">
         <is>
-          <t>Competition</t>
+          <t>Quant firm program</t>
         </is>
       </c>
       <c r="D117" s="8" t="inlineStr">
@@ -15382,14 +15394,10 @@
       </c>
       <c r="E117" s="4" t="inlineStr">
         <is>
-          <t>https://globalyouth.wharton.upenn.edu/competitions/investment-competition</t>
-        </is>
-      </c>
-      <c r="F117" s="3" t="inlineStr">
-        <is>
-          <t>Ruled out on stage - high school students only. Christina Qi's 2026 quant competitions &amp; events list (LinkedIn Pulse), read 2026-09-06.</t>
-        </is>
-      </c>
+          <t>https://www.twosigma.com/undergraduate-students/</t>
+        </is>
+      </c>
+      <c r="F117" s="3" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" s="3" t="inlineStr">
@@ -15399,12 +15407,12 @@
       </c>
       <c r="B118" s="3" t="inlineStr">
         <is>
-          <t>Women in Quantitative Finance Americas Conference</t>
+          <t>Two Sigma PhD Fellowship</t>
         </is>
       </c>
       <c r="C118" s="3" t="inlineStr">
         <is>
-          <t>Conference / other</t>
+          <t>Quant firm program</t>
         </is>
       </c>
       <c r="D118" s="8" t="inlineStr">
@@ -15414,14 +15422,10 @@
       </c>
       <c r="E118" s="4" t="inlineStr">
         <is>
-          <t>https://www.wbstraining.com/events/wqfa</t>
-        </is>
-      </c>
-      <c r="F118" s="3" t="inlineStr">
-        <is>
-          <t>Ruled out by an identity gate: this program is for women. Christina Qi's 2026 quant competitions &amp; events list (LinkedIn Pulse), read 2026-09-06. Listed here so it is not re-researched.</t>
-        </is>
-      </c>
+          <t>https://www.twosigma.com/graduate-students/phd-fellowships/</t>
+        </is>
+      </c>
+      <c r="F118" s="3" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" s="3" t="inlineStr">
@@ -15431,12 +15435,12 @@
       </c>
       <c r="B119" s="3" t="inlineStr">
         <is>
-          <t>Women in Quantitative Finance London Conference</t>
+          <t>Virtu Financial Women's Winternship</t>
         </is>
       </c>
       <c r="C119" s="3" t="inlineStr">
         <is>
-          <t>Conference / other</t>
+          <t>Quant firm program</t>
         </is>
       </c>
       <c r="D119" s="8" t="inlineStr">
@@ -15446,49 +15450,141 @@
       </c>
       <c r="E119" s="4" t="inlineStr">
         <is>
-          <t>https://www.wbstraining.com/events/london-wqf-conference</t>
-        </is>
-      </c>
-      <c r="F119" s="3" t="inlineStr">
-        <is>
-          <t>Ruled out by an identity gate: this program is for women. Christina Qi's 2026 quant competitions &amp; events list (LinkedIn Pulse), read 2026-09-06. Listed here so it is not re-researched.</t>
-        </is>
-      </c>
+          <t>https://www.virtu.com/careers/</t>
+        </is>
+      </c>
+      <c r="F119" s="3" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" s="3" t="inlineStr">
         <is>
+          <t>You cannot apply (NO)</t>
+        </is>
+      </c>
+      <c r="B120" s="3" t="inlineStr">
+        <is>
+          <t>Wharton Global High School Investment Competition</t>
+        </is>
+      </c>
+      <c r="C120" s="3" t="inlineStr">
+        <is>
+          <t>Competition</t>
+        </is>
+      </c>
+      <c r="D120" s="8" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E120" s="4" t="inlineStr">
+        <is>
+          <t>https://globalyouth.wharton.upenn.edu/competitions/investment-competition</t>
+        </is>
+      </c>
+      <c r="F120" s="3" t="inlineStr">
+        <is>
+          <t>Ruled out on stage - high school students only. Christina Qi's 2026 quant competitions &amp; events list (LinkedIn Pulse), read 2026-09-06.</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="3" t="inlineStr">
+        <is>
+          <t>You cannot apply (NO)</t>
+        </is>
+      </c>
+      <c r="B121" s="3" t="inlineStr">
+        <is>
+          <t>Women in Quantitative Finance Americas Conference</t>
+        </is>
+      </c>
+      <c r="C121" s="3" t="inlineStr">
+        <is>
+          <t>Conference / other</t>
+        </is>
+      </c>
+      <c r="D121" s="8" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E121" s="4" t="inlineStr">
+        <is>
+          <t>https://www.wbstraining.com/events/wqfa</t>
+        </is>
+      </c>
+      <c r="F121" s="3" t="inlineStr">
+        <is>
+          <t>Ruled out by an identity gate: this program is for women. Christina Qi's 2026 quant competitions &amp; events list (LinkedIn Pulse), read 2026-09-06. Listed here so it is not re-researched.</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="3" t="inlineStr">
+        <is>
+          <t>You cannot apply (NO)</t>
+        </is>
+      </c>
+      <c r="B122" s="3" t="inlineStr">
+        <is>
+          <t>Women in Quantitative Finance London Conference</t>
+        </is>
+      </c>
+      <c r="C122" s="3" t="inlineStr">
+        <is>
+          <t>Conference / other</t>
+        </is>
+      </c>
+      <c r="D122" s="8" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E122" s="4" t="inlineStr">
+        <is>
+          <t>https://www.wbstraining.com/events/london-wqf-conference</t>
+        </is>
+      </c>
+      <c r="F122" s="3" t="inlineStr">
+        <is>
+          <t>Ruled out by an identity gate: this program is for women. Christina Qi's 2026 quant competitions &amp; events list (LinkedIn Pulse), read 2026-09-06. Listed here so it is not re-researched.</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="3" t="inlineStr">
+        <is>
           <t>You cannot apply (STALE)</t>
         </is>
       </c>
-      <c r="B120" s="3" t="inlineStr">
+      <c r="B123" s="3" t="inlineStr">
         <is>
           <t>zapplyjobs underclassmen-internships</t>
         </is>
       </c>
-      <c r="C120" s="3" t="inlineStr">
+      <c r="C123" s="3" t="inlineStr">
         <is>
           <t>Tracker / resource</t>
         </is>
       </c>
-      <c r="D120" s="8" t="inlineStr">
+      <c r="D123" s="8" t="inlineStr">
         <is>
           <t>STALE</t>
         </is>
       </c>
-      <c r="E120" s="4" t="inlineStr">
+      <c r="E123" s="4" t="inlineStr">
         <is>
           <t>https://github.com/zapplyjobs/underclassmen-internships</t>
         </is>
       </c>
-      <c r="F120" s="3" t="inlineStr">
+      <c r="F123" s="3" t="inlineStr">
         <is>
           <t>Right shape, but entries and links are out of date.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F120"/>
+  <autoFilter ref="A1:F123"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId2"/>
@@ -15593,13 +15689,13 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E102" r:id="rId101"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E103" r:id="rId102"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E104" r:id="rId103"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E106" r:id="rId104"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E107" r:id="rId105"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E108" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E105" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E106" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E107" r:id="rId106"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E109" r:id="rId107"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E111" r:id="rId108"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E112" r:id="rId109"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E113" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E110" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E111" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E112" r:id="rId110"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E114" r:id="rId111"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E115" r:id="rId112"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E116" r:id="rId113"/>
@@ -15607,6 +15703,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E118" r:id="rId115"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E119" r:id="rId116"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E120" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E121" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E122" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E123" r:id="rId120"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
sources: watch eight stock pitch competitions and Weiss Asset Management
Stock pitch competitions open to undergraduates, each watched as its own
recurring page and verified under the tracker's client on 2026-10-08:
WITG x Fundamental Edge (Penn), UChicago Blue Chips, Texas Stock Pitch
(USIT), Miami University / Cleveland Research, Princeton (Tiger
Investments), the BIG Pitch Comp (SMU), and Michigan's ENGAGE UIC. HFAC x
Citadel is watched for its next edition; the 2026 one is limited to
sophomores and above.

weiss-greenhouse watches Weiss Asset Management's Greenhouse board, which
carries the 2027 Underclassmen Fellowship for current freshmen and
sophomores. Each competition and the fellowship has a programs.csv row;
WITG and Weiss are in priority.csv.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/out/programs.xlsx
+++ b/out/programs.xlsx
@@ -16,8 +16,8 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Check By Hand'!$A$1:$G$205</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Manual Watch'!$A$1:$G$37</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Priority'!$A$1:$J$37</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Left Out'!$A$1:$F$131</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Priority'!$A$1:$J$39</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Left Out'!$A$1:$F$140</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -9650,7 +9650,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J37"/>
+  <dimension ref="A1:J39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -11513,8 +11513,108 @@
         </is>
       </c>
     </row>
+    <row r="38">
+      <c r="A38" s="3" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>A - high value, do not miss</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>Weiss Asset Management 2027 Underclassmen Fellowship</t>
+        </is>
+      </c>
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>Quant firm program</t>
+        </is>
+      </c>
+      <c r="E38" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F38" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G38" s="3" t="inlineStr">
+        <is>
+          <t>Oct-Dec 2026 (event Jan 7-8, 2027)</t>
+        </is>
+      </c>
+      <c r="H38" s="3" t="inlineStr">
+        <is>
+          <t>Yes - weiss-greenhouse board</t>
+        </is>
+      </c>
+      <c r="I38" s="3" t="inlineStr">
+        <is>
+          <t>Hedge-fund programme restricted to freshmen and sophomores, travel paid, explicitly a route to internships. No deadline is stated, so the window can close without notice.</t>
+        </is>
+      </c>
+      <c r="J38" s="4" t="inlineStr">
+        <is>
+          <t>https://job-boards.greenhouse.io/weissassetmanagement</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="3" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>C - open entry, participation is the only gate</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>WITG x Fundamental Edge Stock Pitch Competition (Penn)</t>
+        </is>
+      </c>
+      <c r="D39" s="3" t="inlineStr">
+        <is>
+          <t>Competition</t>
+        </is>
+      </c>
+      <c r="E39" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F39" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G39" s="3" t="inlineStr">
+        <is>
+          <t>Sep-Oct (2026 deadline Oct 19)</t>
+        </is>
+      </c>
+      <c r="H39" s="3" t="inlineStr">
+        <is>
+          <t>Yes - witg-stock-pitch page</t>
+        </is>
+      </c>
+      <c r="I39" s="3" t="inlineStr">
+        <is>
+          <t>Open to any undergraduate, cross-school teams allowed, and the deadline is the nearest of the stock pitch competitions.</t>
+        </is>
+      </c>
+      <c r="J39" s="4" t="inlineStr">
+        <is>
+          <t>https://www.pennwitg.com/competition</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J37"/>
+  <autoFilter ref="A1:J39"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J3" r:id="rId2"/>
@@ -11551,6 +11651,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J35" r:id="rId33"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J36" r:id="rId34"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J37" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J38" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J39" r:id="rId37"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -11916,7 +12018,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F131"/>
+  <dimension ref="A1:F140"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -12090,44 +12192,44 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Already watched by bny-pre-internship</t>
+          <t>Already watched by big-pitch-comp</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>BNY Freshman Jumpstart</t>
+          <t>The BIG Pitch Comp (Boulevard Investment Group, SMU Cox)</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>Conference / other</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>YES</t>
+          <t>Competition</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>CHECK</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>https://www.bny.com/corporate/global/en/about-us/careers/students/pre-internship.html</t>
+          <t>https://www.blvdinvestmentgroup.org/thebigpitchcomp</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>Verified 2026-09-30: 'Undergraduate first-year students ... with an expected graduation date of December 2029 or May 2030.' Two virtual half-days, business &amp; corporate functions track. Low effort, low depth.</t>
+          <t>Verified 2026-10-08 on the official pages, still describing the 2026 edition: "A national stock pitch competition for collegiate undergraduates"; "Team size: 2-4 undergraduate students"; the apply page says "Undergraduate-only competition. Cross-school teams allowed." Deck plus 3-minute thesis video on one U.S.-listed equity over $1B. $20,000 prize pool ($10k / $6.5k / $3.5k); finalists must travel to Dallas and BIG pays one hotel night (Apr 10). No class-year restriction stated. The separate "2026 Freshmen Pitch Comp" on the same site is for SMU students only and is not tracked.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Already watched by bofa-campus-events</t>
+          <t>Already watched by bny-pre-internship</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Bank of America campus events (Early Insights)</t>
+          <t>BNY Freshman Jumpstart</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
@@ -12135,95 +12237,95 @@
           <t>Conference / other</t>
         </is>
       </c>
-      <c r="D7" s="5" t="inlineStr">
-        <is>
-          <t>CHECK</t>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>https://bankcampuscareers.tal.net/vx/mobile-0/candidate/jobboard/vacancy/2/feed</t>
+          <t>https://www.bny.com/corporate/global/en/about-us/careers/students/pre-internship.html</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>Verified 2026-09-26: Oleeo (tal.net) Atom feed of campus events, 18 entries, answers the honest User-Agent. Also available: vacancy/1/feed (152 entries) and a JSON API at careers.bankofamerica.com/services/campusjobssearchservlet.</t>
+          <t>Verified 2026-09-30: 'Undergraduate first-year students ... with an expected graduation date of December 2029 or May 2030.' Two virtual half-days, business &amp; corporate functions track. Low effort, low depth.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>Already watched by bridgewater-students</t>
+          <t>Already watched by bofa-campus-events</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Bridgewater Investment Immersion Program</t>
+          <t>Bank of America campus events (Early Insights)</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>Quant firm program</t>
-        </is>
-      </c>
-      <c r="D8" s="6" t="inlineStr">
-        <is>
-          <t>LATER</t>
+          <t>Conference / other</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>CHECK</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>https://www.bridgewater.com/working-at-bridgewater/students</t>
+          <t>https://bankcampuscareers.tal.net/vx/mobile-0/candidate/jobboard/vacancy/2/feed</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>3 days onsite in Westport. Explicitly 'second year of a 4-year degree'.</t>
+          <t>Verified 2026-09-26: Oleeo (tal.net) Atom feed of campus events, 18 entries, answers the honest User-Agent. Also available: vacancy/1/feed (152 entries) and a JSON API at careers.bankofamerica.com/services/campusjobssearchservlet.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Already watched by builtin-data-analytics</t>
+          <t>Already watched by bridgewater-students</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Built In data and analytics internships</t>
+          <t>Bridgewater Investment Immersion Program</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Tracker / resource</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>USE</t>
+          <t>Quant firm program</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>LATER</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>https://builtin.com/jobs/data-analytics/internship</t>
+          <t>https://www.bridgewater.com/working-at-bridgewater/students</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>Front page of Built In's data and analytics internship listings, newest first (about 14-25 cards), watched as a what's-new feed rather than a full list: the site returns HTTP 429 after roughly 70 requests at one a second, so a full crawl is not polite. Measured 2026-10-01 across a deeper crawl: most of its in-field internships were not on Simplify, but many are generic internships at large non-technology employers.</t>
+          <t>3 days onsite in Westport. Explicitly 'second year of a 4-year degree'.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>Already watched by builtin-dev-engineering</t>
+          <t>Already watched by builtin-data-analytics</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Built In software engineering internships</t>
+          <t>Built In data and analytics internships</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
@@ -12238,24 +12340,24 @@
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>https://builtin.com/jobs/dev-engineering/internship</t>
+          <t>https://builtin.com/jobs/data-analytics/internship</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>Front page of Built In's software engineering internship listings, newest first (about 14-25 cards), watched as a what's-new feed rather than a full list: the site returns HTTP 429 after roughly 70 requests at one a second, so a full crawl is not polite. Measured 2026-10-01 across a deeper crawl: most of its in-field internships were not on Simplify, but many are generic internships at large non-technology employers.</t>
+          <t>Front page of Built In's data and analytics internship listings, newest first (about 14-25 cards), watched as a what's-new feed rather than a full list: the site returns HTTP 429 after roughly 70 requests at one a second, so a full crawl is not polite. Measured 2026-10-01 across a deeper crawl: most of its in-field internships were not on Simplify, but many are generic internships at large non-technology employers.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>Already watched by builtin-finance</t>
+          <t>Already watched by builtin-dev-engineering</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Built In finance internships</t>
+          <t>Built In software engineering internships</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
@@ -12270,61 +12372,61 @@
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>https://builtin.com/jobs/finance/internship</t>
+          <t>https://builtin.com/jobs/dev-engineering/internship</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>Front page of Built In's finance internship listings, newest first (about 14-25 cards), watched as a what's-new feed rather than a full list: the site returns HTTP 429 after roughly 70 requests at one a second, so a full crawl is not polite. Measured 2026-10-01 across a deeper crawl: most of its in-field internships were not on Simplify, but many are generic internships at large non-technology employers.</t>
+          <t>Front page of Built In's software engineering internship listings, newest first (about 14-25 cards), watched as a what's-new feed rather than a full list: the site returns HTTP 429 after roughly 70 requests at one a second, so a full crawl is not polite. Measured 2026-10-01 across a deeper crawl: most of its in-field internships were not on Simplify, but many are generic internships at large non-technology employers.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>Already watched by calhacks</t>
+          <t>Already watched by builtin-finance</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Cal Hacks</t>
+          <t>Built In finance internships</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>Competition</t>
-        </is>
-      </c>
-      <c r="D12" s="5" t="inlineStr">
-        <is>
-          <t>CHECK</t>
+          <t>Tracker / resource</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>USE</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>https://www.calhacks.io/</t>
+          <t>https://builtin.com/jobs/finance/internship</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>Verified 2026-10-08: 'Cal Hacks is open to undergraduate and graduate students as well as new grads of under 1 year from all colleges and universities.' Travel: 'This year, we will be offering travel stipends to a limited number of hackers with regional caps based on the region you are coming from'; most attendees get there themselves (Caltrain, BART). Run by Hackers@Berkeley; held in San Francisco.</t>
+          <t>Front page of Built In's finance internship listings, newest first (about 14-25 cards), watched as a what's-new feed rather than a full list: the site returns HTTP 429 after roughly 70 requests at one a second, so a full crawl is not polite. Measured 2026-10-01 across a deeper crawl: most of its in-field internships were not on Simplify, but many are generic internships at large non-technology employers.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Already watched by capitalone-early-career</t>
+          <t>Already watched by calhacks</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Capital One Analyst / Tech / Product Summits</t>
+          <t>Cal Hacks</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>Tech internship</t>
+          <t>Competition</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
@@ -12334,29 +12436,29 @@
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>https://www.capitalonecareers.com/get-ahead-with-early-career-programs-for-students</t>
+          <t>https://www.calhacks.io/</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>Verified 2026-09-26: Analyst Summit 'First-year students or sophomores pursuing a quantitative/STEM major'; Tech Summit 'Sophomores with beginner coding experience'. Separate from the Capital One TEIP row.</t>
+          <t>Verified 2026-10-08: 'Cal Hacks is open to undergraduate and graduate students as well as new grads of under 1 year from all colleges and universities.' Travel: 'This year, we will be offering travel stipends to a limited number of hackers with regional caps based on the region you are coming from'; most attendees get there themselves (Caltrain, BART). Run by Hackers@Berkeley; held in San Francisco.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>Already watched by cerebralvalley-sf-events</t>
+          <t>Already watched by capitalone-early-career</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Cerebral Valley SF &amp; Bay Area AI events calendar</t>
+          <t>Capital One Analyst / Tech / Product Summits</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>Tracker / resource</t>
+          <t>Tech internship</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
@@ -12366,93 +12468,93 @@
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>https://cerebralvalley.ai/events/san-francisco</t>
+          <t>https://www.capitalonecareers.com/get-ahead-with-early-career-programs-for-students</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>Verified 2026-10-08: Cerebral Valley's SF and Bay Area AI event feed, mixing hackathons with talks and meetups, e.g. 'The Recursive Agents Hackathon' (Oct 17, Shack15 SF; 'All attendees must apply and be approved') and 'Intelligence at Work Hackathon' (Oct 23, Menlo Park). Not student-specific; check each event's own terms.</t>
+          <t>Verified 2026-09-26: Analyst Summit 'First-year students or sophomores pursuing a quantitative/STEM major'; Tech Summit 'Sophomores with beginner coding experience'. Separate from the Capital One TEIP row.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>Already watched by citi-pre-internships</t>
+          <t>Already watched by cerebralvalley-sf-events</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Citi Freshman Discovery</t>
+          <t>Cerebral Valley SF &amp; Bay Area AI events calendar</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>Conference / other</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>YES</t>
+          <t>Tracker / resource</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>CHECK</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>https://jobs.citi.com/early-career-programs-pre-internships</t>
+          <t>https://cerebralvalley.ai/events/san-francisco</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>Verified 2026-09-30: 'All first-year students in a four-year bachelor's degree program from a US accredited institution, regardless of major.' 3-day virtual introduction to financial services.</t>
+          <t>Verified 2026-10-08: Cerebral Valley's SF and Bay Area AI event feed, mixing hackathons with talks and meetups, e.g. 'The Recursive Agents Hackathon' (Oct 17, Shack15 SF; 'All attendees must apply and be approved') and 'Intelligence at Work Hackathon' (Oct 23, Menlo Park). Not student-specific; check each event's own terms.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>Already watched by cmu-riss</t>
+          <t>Already watched by citi-pre-internships</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>CMU Robotics Institute Summer Scholars (RISS)</t>
+          <t>Citi Freshman Discovery</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>Research / math</t>
-        </is>
-      </c>
-      <c r="D16" s="5" t="inlineStr">
-        <is>
-          <t>CHECK</t>
+          <t>Conference / other</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>https://riss.ri.cmu.edu/</t>
+          <t>https://jobs.citi.com/early-career-programs-pre-internships</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>11-week summer research immersion for undergraduates at CMU's Robotics Institute.</t>
+          <t>Verified 2026-09-30: 'All first-year students in a four-year bachelor's degree program from a US accredited institution, regardless of major.' 3-day virtual introduction to financial services.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>Already watched by comap-mcm</t>
+          <t>Already watched by cmu-riss</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>COMAP MCM/ICM</t>
+          <t>CMU Robotics Institute Summer Scholars (RISS)</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>Competition</t>
+          <t>Research / math</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
@@ -12462,24 +12564,24 @@
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>https://www.contest.comap.com/undergraduate/contests/</t>
+          <t>https://riss.ri.cmu.edu/</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>Verified 2026-09-26: 'high school students and college undergraduates'; 2027 contest 28 Jan - 1 Feb.</t>
+          <t>11-week summer research immersion for undergraduates at CMU's Robotics Institute.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>Already watched by cornell-trading-competition</t>
+          <t>Already watched by comap-mcm</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>Cornell Trading Competition</t>
+          <t>COMAP MCM/ICM</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
@@ -12487,95 +12589,95 @@
           <t>Competition</t>
         </is>
       </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>YES</t>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>CHECK</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>https://cornellquantfund.org/competition</t>
+          <t>https://www.contest.comap.com/undergraduate/contests/</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>Teams of 4, NO EXPERIENCE NECESSARY, $10k+ prizes, Cornell Tech NYC. Case packets released 2 weeks early.</t>
+          <t>Verified 2026-09-26: 'high school students and college undergraduates'; 2027 contest 28 Jan - 1 Feb.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>Already watched by cra-dreu</t>
+          <t>Already watched by cornell-trading-competition</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>CRA DREU</t>
+          <t>Cornell Trading Competition</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>Research / math</t>
-        </is>
-      </c>
-      <c r="D19" s="5" t="inlineStr">
-        <is>
-          <t>CHECK</t>
+          <t>Competition</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>https://cra.org/cra-wp/dreu/</t>
+          <t>https://cornellquantfund.org/competition</t>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>Verified 2026-09-26: 'High school graduates who have been accepted ... are also eligible'; priority to CS majors. Large page (94K chars).</t>
+          <t>Teams of 4, NO EXPERIENCE NECESSARY, $10k+ prizes, Cornell Tech NYC. Case packets released 2 weeks early.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>Already watched by cs-social-good-fellowships</t>
+          <t>Already watched by cra-dreu</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>CS+Social Good Summer Fellowships</t>
+          <t>CRA DREU</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>Stanford-only</t>
-        </is>
-      </c>
-      <c r="D20" s="2" t="inlineStr">
-        <is>
-          <t>YES</t>
+          <t>Research / math</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>CHECK</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>https://cardinalservice.stanford.edu/opportunities/cssocial-good-summer-fellowships</t>
+          <t>https://cra.org/cra-wp/dreu/</t>
         </is>
       </c>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t>Verified 2026-09-30 from the 2026 SOLO listing: 'enrolled as a first-year, sophomore, or junior ... must have completed CS 106B by the end of Spring Quarter.' $7,000 base stipend, full-time summer with a tech-for-good partner. Cardinal Quarter.</t>
+          <t>Verified 2026-09-26: 'High school graduates who have been accepted ... are also eligible'; priority to CS majors. Large page (94K chars).</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>Already watched by curis</t>
+          <t>Already watched by cs-social-good-fellowships</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>Stanford CURIS</t>
+          <t>CS+Social Good Summer Fellowships</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
@@ -12590,24 +12692,24 @@
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t>https://curis.stanford.edu/</t>
+          <t>https://cardinalservice.stanford.edu/opportunities/cssocial-good-summer-fellowships</t>
         </is>
       </c>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>CS dept paid summer research. Project list posted late Jan. Also lists year-round projects for units or hourly pay. | Checked 2026-09-26: now watched with render_js - the page is client-rendered and yields 1,264 chars in the browser.</t>
+          <t>Verified 2026-09-30 from the 2026 SOLO listing: 'enrolled as a first-year, sophomore, or junior ... must have completed CS 106B by the end of Spring Quarter.' $7,000 base stipend, full-time summer with a tech-for-good partner. Cardinal Quarter.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>Already watched by datasurf</t>
+          <t>Already watched by curis</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>Stanford DataSURF (formerly SURP-Stats)</t>
+          <t>Stanford CURIS</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
@@ -12622,44 +12724,44 @@
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>https://datasciencemajor.stanford.edu/research-impact/data-science-undergraduate-research-focus</t>
+          <t>https://curis.stanford.edu/</t>
         </is>
       </c>
       <c r="F22" s="3" t="inlineStr">
         <is>
-          <t>Verified 2026-09-30: 'Stanford undergraduate students from any department who meet the prerequisites are encouraged to apply' (examples: STATS 60, MATH 51-53, CS 106A/B). 10 weeks, $8,500 stipend plus need-based supplement.</t>
+          <t>CS dept paid summer research. Project list posted late Jan. Also lists year-round projects for units or hourly pay. | Checked 2026-09-26: now watched with render_js - the page is client-rendered and yields 1,264 chars in the browser.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>Already watched by deshaw-campus</t>
+          <t>Already watched by datasurf</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>D. E. Shaw Nexus Fellowship</t>
+          <t>Stanford DataSURF (formerly SURP-Stats)</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>Quant firm program</t>
-        </is>
-      </c>
-      <c r="D23" s="6" t="inlineStr">
-        <is>
-          <t>LATER</t>
+          <t>Stanford-only</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t>https://campus.deshaw.com/fellowships</t>
+          <t>https://datasciencemajor.stanford.edu/research-impact/data-science-undergraduate-research-focus</t>
         </is>
       </c>
       <c r="F23" s="3" t="inlineStr">
         <is>
-          <t>THE one for a first-year to target the following year - Nexus is the all-students track. 3 days NYC, $1,500 stipend, travel + lodging. | Checked 2026-09-26: campus.deshaw.com/fellowships now redirects to the campus root, which mentions no fellowships. Kept; the root is watched as deshaw-campus.</t>
+          <t>Verified 2026-09-30: 'Stanford undergraduate students from any department who meet the prerequisites are encouraged to apply' (examples: STATS 60, MATH 51-53, CS 106A/B). 10 weeks, $8,500 stipend plus need-based supplement.</t>
         </is>
       </c>
     </row>
@@ -12671,7 +12773,7 @@
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>D. E. Shaw campus site</t>
+          <t>D. E. Shaw Nexus Fellowship</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
@@ -12679,191 +12781,191 @@
           <t>Quant firm program</t>
         </is>
       </c>
-      <c r="D24" s="5" t="inlineStr">
-        <is>
-          <t>CHECK</t>
+      <c r="D24" s="6" t="inlineStr">
+        <is>
+          <t>LATER</t>
         </is>
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>https://campus.deshaw.com/</t>
+          <t>https://campus.deshaw.com/fellowships</t>
         </is>
       </c>
       <c r="F24" s="3" t="inlineStr">
         <is>
-          <t>Verified 2026-09-26: internships for 'undergraduate and graduate students'. The fellowship rows' campus.deshaw.com/fellowships URL now redirects here; this page is watched so a returning fellowship shows up.</t>
+          <t>THE one for a first-year to target the following year - Nexus is the all-students track. 3 days NYC, $1,500 stipend, travel + lodging. | Checked 2026-09-26: campus.deshaw.com/fellowships now redirects to the campus root, which mentions no fellowships. Kept; the root is watched as deshaw-campus.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>Already watched by dimacs-reu</t>
+          <t>Already watched by deshaw-campus</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>DIMACS REU</t>
+          <t>D. E. Shaw campus site</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>Research / math</t>
-        </is>
-      </c>
-      <c r="D25" s="6" t="inlineStr">
-        <is>
-          <t>LATER</t>
+          <t>Quant firm program</t>
+        </is>
+      </c>
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t>CHECK</t>
         </is>
       </c>
       <c r="E25" s="4" t="inlineStr">
         <is>
-          <t>https://dimacs.rutgers.edu/reu-main</t>
+          <t>https://campus.deshaw.com/</t>
         </is>
       </c>
       <c r="F25" s="3" t="inlineStr">
         <is>
-          <t>Verified 2026-09-26: 'We do not usually admit freshmen' - watch for sophomore year.</t>
+          <t>Verified 2026-09-26: internships for 'undergraduate and graduate students'. The fellowship rows' campus.deshaw.com/fellowships URL now redirects here; this page is watched so a returning fellowship shows up.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>Already watched by dukequant-competition</t>
+          <t>Already watched by dimacs-reu</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>Duke FinTech Trading Competition</t>
+          <t>DIMACS REU</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>Competition</t>
-        </is>
-      </c>
-      <c r="D26" s="2" t="inlineStr">
-        <is>
-          <t>YES</t>
+          <t>Research / math</t>
+        </is>
+      </c>
+      <c r="D26" s="6" t="inlineStr">
+        <is>
+          <t>LATER</t>
         </is>
       </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>https://www.duke.edu/</t>
+          <t>https://dimacs.rutgers.edu/reu-main</t>
         </is>
       </c>
       <c r="F26" s="3" t="inlineStr">
         <is>
-          <t>3 months, paper trading, bracket format. Sponsors include Schonfeld. Lowest time commitment. | Checked 2026-09-26: Duke Quantitative Finance's competition page is dukequant.com/general-7 (watched with render_js); not yet confirmed to be the same event this row names. The listed duke.edu is kept.</t>
+          <t>Verified 2026-09-26: 'We do not usually admit freshmen' - watch for sophomore year.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>Already watched by evercore-campus</t>
+          <t>Already watched by dukequant-competition</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>Evercore student events</t>
+          <t>Duke FinTech Trading Competition</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>Conference / other</t>
-        </is>
-      </c>
-      <c r="D27" s="5" t="inlineStr">
-        <is>
-          <t>CHECK</t>
+          <t>Competition</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
       <c r="E27" s="4" t="inlineStr">
         <is>
-          <t>https://evercore.tal.net/vx/mobile-0/candidate/jobboard/vacancy/2/feed</t>
+          <t>https://www.duke.edu/</t>
         </is>
       </c>
       <c r="F27" s="3" t="inlineStr">
         <is>
-          <t>Verified 2026-09-26: Oleeo Atom feed, 39 entries; vacancy/1/feed has 29 more. Some events are restricted-audience per the Simplify blog.</t>
+          <t>3 months, paper trading, bracket format. Sponsors include Schonfeld. Lowest time commitment. | Checked 2026-09-26: Duke Quantitative Finance's competition page is dukequant.com/general-7 (watched with render_js); not yet confirmed to be the same event this row names. The listed duke.edu is kept.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>Already watched by futureforce-launchpad</t>
+          <t>Already watched by evercore-campus</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>Salesforce Futureforce Tech Launchpad (CodePath)</t>
+          <t>Evercore student events</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>Tech internship</t>
-        </is>
-      </c>
-      <c r="D28" s="6" t="inlineStr">
-        <is>
-          <t>LATER</t>
+          <t>Conference / other</t>
+        </is>
+      </c>
+      <c r="D28" s="5" t="inlineStr">
+        <is>
+          <t>CHECK</t>
         </is>
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>https://info.codepath.org/futureforce-tech-launchpad</t>
+          <t>https://evercore.tal.net/vx/mobile-0/candidate/jobboard/vacancy/2/feed</t>
         </is>
       </c>
       <c r="F28" s="3" t="inlineStr">
         <is>
-          <t>Verified 2026-09-26: 'Students who will complete their sophomore year in Spring 2026' - so summer 2028 for a class of 2030.</t>
+          <t>Verified 2026-09-26: Oleeo Atom feed, 39 entries; vacancy/1/feed has 29 more. Some events are restricted-audience per the Simplify blog.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>Already watched by hackgt</t>
+          <t>Already watched by futureforce-launchpad</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>HackGT</t>
+          <t>Salesforce Futureforce Tech Launchpad (CodePath)</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>Competition</t>
-        </is>
-      </c>
-      <c r="D29" s="5" t="inlineStr">
-        <is>
-          <t>CHECK</t>
+          <t>Tech internship</t>
+        </is>
+      </c>
+      <c r="D29" s="6" t="inlineStr">
+        <is>
+          <t>LATER</t>
         </is>
       </c>
       <c r="E29" s="4" t="inlineStr">
         <is>
-          <t>https://hack.gt/</t>
+          <t>https://info.codepath.org/futureforce-tech-launchpad</t>
         </is>
       </c>
       <c r="F29" s="3" t="inlineStr">
         <is>
-          <t>Verified 2026-10-08 (rendered page): 'If you will be traveling from afar, we offer reimbursements to GT'; the page links a travel guide.</t>
+          <t>Verified 2026-09-26: 'Students who will complete their sophomore year in Spring 2026' - so summer 2028 for a class of 2030.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>Already watched by hackprinceton</t>
+          <t>Already watched by hackgt</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>HackPrinceton</t>
+          <t>HackGT</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
@@ -12878,24 +12980,24 @@
       </c>
       <c r="E30" s="4" t="inlineStr">
         <is>
-          <t>https://www.hackprinceton.com/</t>
+          <t>https://hack.gt/</t>
         </is>
       </c>
       <c r="F30" s="3" t="inlineStr">
         <is>
-          <t>Verified 2026-10-08: 'Applicants must be matriculated in an undergraduate or graduate program at a college or university.' Travel: 'Some admitted hackers may receive a travel stipend that covers part of their travel expenses.' No cost to apply or attend.</t>
+          <t>Verified 2026-10-08 (rendered page): 'If you will be traveling from afar, we offer reimbursements to GT'; the page links a travel guide.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>Already watched by hackumass</t>
+          <t>Already watched by hackprinceton</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>HackUMass</t>
+          <t>HackPrinceton</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
@@ -12910,24 +13012,24 @@
       </c>
       <c r="E31" s="4" t="inlineStr">
         <is>
-          <t>https://www.hackumass.com/</t>
+          <t>https://www.hackprinceton.com/</t>
         </is>
       </c>
       <c r="F31" s="3" t="inlineStr">
         <is>
-          <t>Verified 2026-10-08: 'HackUMass XIV is open to ALL college students, including graduate students, regardless of major!' Travel: 'If you apply by the early application deadline, you have the opportunity to apply for travel reimbursement.' Early applications for XIV were already closed on 2026-10-08.</t>
+          <t>Verified 2026-10-08: 'Applicants must be matriculated in an undergraduate or graduate program at a college or university.' Travel: 'Some admitted hackers may receive a travel stipend that covers part of their travel expenses.' No cost to apply or attend.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
         <is>
-          <t>Already watched by harvard-undergraduate-trading</t>
+          <t>Already watched by hackumass</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>Harvard Undergraduate Trading Competition</t>
+          <t>HackUMass</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
@@ -12942,29 +13044,29 @@
       </c>
       <c r="E32" s="4" t="inlineStr">
         <is>
-          <t>https://www.huqt.com/</t>
+          <t>https://www.hackumass.com/</t>
         </is>
       </c>
       <c r="F32" s="3" t="inlineStr">
         <is>
-          <t>Undergraduate intercollegiate trading competition run by Harvard Undergraduate Quantitative Traders. The organisation rebranded: the article's link harvarduqt.com/competition 301-redirects to www.huqt.com/competition, which 404s. The live site is huqt.com and it has an Apply link. Christina Qi's 2026 quant competitions &amp; events list (LinkedIn Pulse), read 2026-09-06. Class year and team format not published - verify before planning.</t>
+          <t>Verified 2026-10-08: 'HackUMass XIV is open to ALL college students, including graduate students, regardless of major!' Travel: 'If you apply by the early application deadline, you have the opportunity to apply for travel reimbursement.' Early applications for XIV were already closed on 2026-10-08.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>Already watched by hedgewest-sf-meetup-series</t>
+          <t>Already watched by harvard-undergraduate-trading</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>HedgeWest SF Meetup Series</t>
+          <t>Harvard Undergraduate Trading Competition</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>Conference / other</t>
+          <t>Competition</t>
         </is>
       </c>
       <c r="D33" s="5" t="inlineStr">
@@ -12974,29 +13076,29 @@
       </c>
       <c r="E33" s="4" t="inlineStr">
         <is>
-          <t>https://hedgewestsf.org/</t>
+          <t>https://www.huqt.com/</t>
         </is>
       </c>
       <c r="F33" s="3" t="inlineStr">
         <is>
-          <t>Quant/hedge-fund meetup series in San Francisco - one of the very few items in this article that is geographically local to Stanford. Christina Qi's 2026 quant competitions &amp; events list (LinkedIn Pulse), read 2026-09-06. Verify whether undergraduates may attend.</t>
+          <t>Undergraduate intercollegiate trading competition run by Harvard Undergraduate Quantitative Traders. The organisation rebranded: the article's link harvarduqt.com/competition 301-redirects to www.huqt.com/competition, which 404s. The live site is huqt.com and it has an Apply link. Christina Qi's 2026 quant competitions &amp; events list (LinkedIn Pulse), read 2026-09-06. Class year and team format not published - verify before planning.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>Already watched by hophacks</t>
+          <t>Already watched by hedgewest-sf-meetup-series</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>HopHacks</t>
+          <t>HedgeWest SF Meetup Series</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>Competition</t>
+          <t>Conference / other</t>
         </is>
       </c>
       <c r="D34" s="5" t="inlineStr">
@@ -13006,24 +13108,24 @@
       </c>
       <c r="E34" s="4" t="inlineStr">
         <is>
-          <t>https://hophacks.com/</t>
+          <t>https://hedgewestsf.org/</t>
         </is>
       </c>
       <c r="F34" s="3" t="inlineStr">
         <is>
-          <t>Verified 2026-10-08: 'We will not be offering individual travel reimbursements. However, please see the busing interest form ... If enough people from your city sign up, we may send a FREE bus.'</t>
+          <t>Quant/hedge-fund meetup series in San Francisco - one of the very few items in this article that is geographically local to Stanford. Christina Qi's 2026 quant competitions &amp; events list (LinkedIn Pulse), read 2026-09-06. Verify whether undergraduates may attend.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>Already watched by iaqf-academic-paper-competition</t>
+          <t>Already watched by hfac-citadel-pitch</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>IAQF Academic Paper Competition</t>
+          <t>HFAC x Citadel Intercollegiate Stock Pitch Competition</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
@@ -13031,36 +13133,36 @@
           <t>Competition</t>
         </is>
       </c>
-      <c r="D35" s="5" t="inlineStr">
-        <is>
-          <t>CHECK</t>
+      <c r="D35" s="6" t="inlineStr">
+        <is>
+          <t>LATER</t>
         </is>
       </c>
       <c r="E35" s="4" t="inlineStr">
         <is>
-          <t>https://www.iaqf.org/upcoming-events</t>
+          <t>https://www.harvardfac.org/hfac-citadel-pitch-comp</t>
         </is>
       </c>
       <c r="F35" s="3" t="inlineStr">
         <is>
-          <t>International Association for Quantitative Finance paper competition. Christina Qi's 2026 quant competitions &amp; events list (LinkedIn Pulse), read 2026-09-06. A paper is a slower but more durable credential than a trading competition; verify undergraduate eligibility.</t>
+          <t>Verified 2026-10-08 on the official page: HFAC with the Citadel Associate Program "is pleased to invite current sophomores, juniors, and seniors"; "*Eligibility: Teams of 2-4 undergraduate students in good standing, eighteen years of age or older, graduating between December 2026 and May 2029, attending a university located in the 50 US States, US territories, Washington, DC, or Canada". The 2026 window excludes a 2030 graduate. "Citadel will sponsor travel and lodging for all selected teams", and "all finalists in the sophomore class (Class of 2029) will receive a first round interview with the Citadel Associate Program." The page URL is not year-specific, so the 2027 edition, whose window should include the class of 2030 as sophomores, is expected here.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>Already watched by icerm-summer</t>
+          <t>Already watched by hophacks</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>Summer@ICERM</t>
+          <t>HopHacks</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>Research / math</t>
+          <t>Competition</t>
         </is>
       </c>
       <c r="D36" s="5" t="inlineStr">
@@ -13070,24 +13172,24 @@
       </c>
       <c r="E36" s="4" t="inlineStr">
         <is>
-          <t>https://icerm.brown.edu/summerug/</t>
+          <t>https://hophacks.com/</t>
         </is>
       </c>
       <c r="F36" s="3" t="inlineStr">
         <is>
-          <t>Verified 2026-09-26: 'Applicants must be matriculating undergraduate students'.</t>
+          <t>Verified 2026-10-08: 'We will not be offering individual travel reimbursements. However, please see the busing interest form ... If enough people from your city sign up, we may send a FREE bus.'</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>Already watched by icpc-pnw</t>
+          <t>Already watched by iaqf-academic-paper-competition</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>ICPC</t>
+          <t>IAQF Academic Paper Competition</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
@@ -13095,36 +13197,36 @@
           <t>Competition</t>
         </is>
       </c>
-      <c r="D37" s="2" t="inlineStr">
-        <is>
-          <t>YES</t>
+      <c r="D37" s="5" t="inlineStr">
+        <is>
+          <t>CHECK</t>
         </is>
       </c>
       <c r="E37" s="4" t="inlineStr">
         <is>
-          <t>https://icpc.global/</t>
+          <t>https://www.iaqf.org/upcoming-events</t>
         </is>
       </c>
       <c r="F37" s="3" t="inlineStr">
         <is>
-          <t>Checked 2026-09-26: icpc.global is a JavaScript shell (53 chars); Stanford's regional, pnw.na.icpc.global, is what is watched.</t>
+          <t>International Association for Quantitative Finance paper competition. Christina Qi's 2026 quant competitions &amp; events list (LinkedIn Pulse), read 2026-09-06. A paper is a slower but more durable credential than a trading competition; verify undergraduate eligibility.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
         <is>
-          <t>Already watched by imc-launchpad-us</t>
+          <t>Already watched by icerm-summer</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>IMC Launchpad (US)</t>
+          <t>Summer@ICERM</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>Quant firm program</t>
+          <t>Research / math</t>
         </is>
       </c>
       <c r="D38" s="5" t="inlineStr">
@@ -13134,29 +13236,29 @@
       </c>
       <c r="E38" s="4" t="inlineStr">
         <is>
-          <t>https://www.imc.com/us/careers/students-graduates/programs/launchpad</t>
+          <t>https://icerm.brown.edu/summerug/</t>
         </is>
       </c>
       <c r="F38" s="3" t="inlineStr">
         <is>
-          <t>IMC's US student program - distinct from the EU Business Course and UK Masterclass, which are geography-excluded. Christina Qi's 2026 quant competitions &amp; events list (LinkedIn Pulse), read 2026-09-06. Class year not published; verify.</t>
+          <t>Verified 2026-09-26: 'Applicants must be matriculating undergraduate students'.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
         <is>
-          <t>Already watched by imc-prosperity</t>
+          <t>Already watched by icpc-pnw</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>IMC Prosperity Trading Competition</t>
+          <t>ICPC</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>Quant firm program</t>
+          <t>Competition</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
@@ -13166,29 +13268,29 @@
       </c>
       <c r="E39" s="4" t="inlineStr">
         <is>
-          <t>https://prosperity.imc.com/</t>
+          <t>https://icpc.global/</t>
         </is>
       </c>
       <c r="F39" s="3" t="inlineStr">
         <is>
-          <t>Teams up to 5, $50,000 pool, fully online. Most accessible serious quant competition. Stanford won top-US in year one.</t>
+          <t>Checked 2026-09-26: icpc.global is a JavaScript shell (53 chars); Stanford's regional, pnw.na.icpc.global, is what is watched.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
         <is>
-          <t>Already watched by ipam-rips</t>
+          <t>Already watched by imc-launchpad-us</t>
         </is>
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>IPAM RIPS (UCLA)</t>
+          <t>IMC Launchpad (US)</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>Research / math</t>
+          <t>Quant firm program</t>
         </is>
       </c>
       <c r="D40" s="5" t="inlineStr">
@@ -13198,24 +13300,24 @@
       </c>
       <c r="E40" s="4" t="inlineStr">
         <is>
-          <t>https://www.ipam.ucla.edu/programs/student-research-programs/</t>
+          <t>https://www.imc.com/us/careers/students-graduates/programs/launchpad</t>
         </is>
       </c>
       <c r="F40" s="3" t="inlineStr">
         <is>
-          <t>Research in Industrial Projects for Students: teams of undergraduates on sponsored industry problems in applied mathematics.</t>
+          <t>IMC's US student program - distinct from the EU Business Course and UK Masterclass, which are geography-excluded. Christina Qi's 2026 quant competitions &amp; events list (LinkedIn Pulse), read 2026-09-06. Class year not published; verify.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>Already watched by janestreet-fttp</t>
+          <t>Already watched by imc-prosperity</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>Jane Street FTTP</t>
+          <t>IMC Prosperity Trading Competition</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
@@ -13230,29 +13332,29 @@
       </c>
       <c r="E41" s="4" t="inlineStr">
         <is>
-          <t>https://www.janestreet.com/join-jane-street/programs-and-events/fttp/</t>
+          <t>https://prosperity.imc.com/</t>
         </is>
       </c>
       <c r="F41" s="3" t="inlineStr">
         <is>
-          <t>Classes + team-based mock trading. STEM majors, no finance background needed. Rolling - apply week one.</t>
+          <t>Teams up to 5, $50,000 pool, fully online. Most accessible serious quant competition. Stanford won top-US in year one.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
         <is>
-          <t>Already watched by janestreet-preview</t>
+          <t>Already watched by ipam-rips</t>
         </is>
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>Jane Street Preview</t>
+          <t>IPAM RIPS (UCLA)</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>Quant firm program</t>
+          <t>Research / math</t>
         </is>
       </c>
       <c r="D42" s="5" t="inlineStr">
@@ -13262,24 +13364,24 @@
       </c>
       <c r="E42" s="4" t="inlineStr">
         <is>
-          <t>https://www.janestreet.com/join-jane-street/programs-and-events/preview/</t>
+          <t>https://www.ipam.ucla.edu/programs/student-research-programs/</t>
         </is>
       </c>
       <c r="F42" s="3" t="inlineStr">
         <is>
-          <t>Verified 2026-09-26 (source research): day-long programme 'for students at any point in their academic career'. One of the 12 programmes on the watched janestreet-programs index; this watches its own page.</t>
+          <t>Research in Industrial Projects for Students: teams of undergraduates on sponsored industry problems in applied mathematics.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
         <is>
-          <t>Already watched by janestreet-programs</t>
+          <t>Already watched by janestreet-fttp</t>
         </is>
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>Jane Street AMP - TA role</t>
+          <t>Jane Street FTTP</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
@@ -13287,31 +13389,31 @@
           <t>Quant firm program</t>
         </is>
       </c>
-      <c r="D43" s="6" t="inlineStr">
-        <is>
-          <t>LATER</t>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
       <c r="E43" s="4" t="inlineStr">
         <is>
-          <t>https://www.janestreet.com/join-jane-street/programs-and-events/amp/</t>
+          <t>https://www.janestreet.com/join-jane-street/programs-and-events/fttp/</t>
         </is>
       </c>
       <c r="F43" s="3" t="inlineStr">
         <is>
-          <t>Paid Jane Street summer on the teaching side. Housing, meals, travel covered. Eligible from spring 2027.</t>
+          <t>Classes + team-based mock trading. STEM majors, no finance background needed. Rolling - apply week one.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
         <is>
-          <t>Already watched by janestreet-programs</t>
+          <t>Already watched by janestreet-preview</t>
         </is>
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>Jane Street ETC</t>
+          <t>Jane Street Preview</t>
         </is>
       </c>
       <c r="C44" s="3" t="inlineStr">
@@ -13321,17 +13423,17 @@
       </c>
       <c r="D44" s="5" t="inlineStr">
         <is>
-          <t>INVITE</t>
+          <t>CHECK</t>
         </is>
       </c>
       <c r="E44" s="4" t="inlineStr">
         <is>
-          <t>https://www.janestreet.com/join-jane-street/programs-and-events/</t>
+          <t>https://www.janestreet.com/join-jane-street/programs-and-events/preview/</t>
         </is>
       </c>
       <c r="F44" s="3" t="inlineStr">
         <is>
-          <t>Electronic Trading Challenge. Entry via university, prior JS events, or the puzzle ecosystem.</t>
+          <t>Verified 2026-09-26 (source research): day-long programme 'for students at any point in their academic career'. One of the 12 programmes on the watched janestreet-programs index; this watches its own page.</t>
         </is>
       </c>
     </row>
@@ -13343,7 +13445,7 @@
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>Jane Street SEE</t>
+          <t>Jane Street AMP - TA role</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">
@@ -13351,19 +13453,19 @@
           <t>Quant firm program</t>
         </is>
       </c>
-      <c r="D45" s="2" t="inlineStr">
-        <is>
-          <t>YES</t>
+      <c r="D45" s="6" t="inlineStr">
+        <is>
+          <t>LATER</t>
         </is>
       </c>
       <c r="E45" s="4" t="inlineStr">
         <is>
-          <t>https://www.janestreet.com/join-jane-street/programs-and-events/</t>
+          <t>https://www.janestreet.com/join-jane-street/programs-and-events/amp/</t>
         </is>
       </c>
       <c r="F45" s="3" t="inlineStr">
         <is>
-          <t>Software Engineering Experience - OCaml and systems design.</t>
+          <t>Paid Jane Street summer on the teaching side. Housing, meals, travel covered. Eligible from spring 2027.</t>
         </is>
       </c>
     </row>
@@ -13375,7 +13477,7 @@
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>Jane Street Symposium</t>
+          <t>Jane Street ETC</t>
         </is>
       </c>
       <c r="C46" s="3" t="inlineStr">
@@ -13393,7 +13495,11 @@
           <t>https://www.janestreet.com/join-jane-street/programs-and-events/</t>
         </is>
       </c>
-      <c r="F46" s="3" t="inlineStr"/>
+      <c r="F46" s="3" t="inlineStr">
+        <is>
+          <t>Electronic Trading Challenge. Entry via university, prior JS events, or the puzzle ecosystem.</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
@@ -13403,7 +13509,7 @@
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>Jane Street Unboxed</t>
+          <t>Jane Street SEE</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr">
@@ -13411,9 +13517,9 @@
           <t>Quant firm program</t>
         </is>
       </c>
-      <c r="D47" s="5" t="inlineStr">
-        <is>
-          <t>CHECK</t>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
       <c r="E47" s="4" t="inlineStr">
@@ -13421,54 +13527,54 @@
           <t>https://www.janestreet.com/join-jane-street/programs-and-events/</t>
         </is>
       </c>
-      <c r="F47" s="3" t="inlineStr"/>
+      <c r="F47" s="3" t="inlineStr">
+        <is>
+          <t>Software Engineering Experience - OCaml and systems design.</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="3" t="inlineStr">
         <is>
-          <t>Already watched by jefferies-campus</t>
+          <t>Already watched by janestreet-programs</t>
         </is>
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>Jefferies campus opportunities</t>
+          <t>Jane Street Symposium</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>Conference / other</t>
+          <t>Quant firm program</t>
         </is>
       </c>
       <c r="D48" s="5" t="inlineStr">
         <is>
-          <t>CHECK</t>
+          <t>INVITE</t>
         </is>
       </c>
       <c r="E48" s="4" t="inlineStr">
         <is>
-          <t>https://jefferies.tal.net/vx/mobile-0/candidate/jobboard/vacancy/2/feed</t>
-        </is>
-      </c>
-      <c r="F48" s="3" t="inlineStr">
-        <is>
-          <t>Verified 2026-09-26: Oleeo Atom feed, 60 entries. Banking is lower priority than quant.</t>
-        </is>
-      </c>
+          <t>https://www.janestreet.com/join-jane-street/programs-and-events/</t>
+        </is>
+      </c>
+      <c r="F48" s="3" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
         <is>
-          <t>Already watched by jhuapl-internships</t>
+          <t>Already watched by janestreet-programs</t>
         </is>
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>Johns Hopkins APL internships</t>
+          <t>Jane Street Unboxed</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>Research / math</t>
+          <t>Quant firm program</t>
         </is>
       </c>
       <c r="D49" s="5" t="inlineStr">
@@ -13478,221 +13584,217 @@
       </c>
       <c r="E49" s="4" t="inlineStr">
         <is>
-          <t>https://www.jhuapl.edu/careers/internships</t>
-        </is>
-      </c>
-      <c r="F49" s="3" t="inlineStr">
-        <is>
-          <t>Page states a minimum GPA requirement. Simplify already carries some APL postings; this watches the programme page itself.</t>
-        </is>
-      </c>
+          <t>https://www.janestreet.com/join-jane-street/programs-and-events/</t>
+        </is>
+      </c>
+      <c r="F49" s="3" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="3" t="inlineStr">
         <is>
-          <t>Already watched by jpmc-career-edyou</t>
+          <t>Already watched by jefferies-campus</t>
         </is>
       </c>
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t>JPMorganChase Career.edYOU Academy</t>
+          <t>Jefferies campus opportunities</t>
         </is>
       </c>
       <c r="C50" s="3" t="inlineStr">
         <is>
-          <t>Tech internship</t>
-        </is>
-      </c>
-      <c r="D50" s="6" t="inlineStr">
-        <is>
-          <t>LATER</t>
+          <t>Conference / other</t>
+        </is>
+      </c>
+      <c r="D50" s="5" t="inlineStr">
+        <is>
+          <t>CHECK</t>
         </is>
       </c>
       <c r="E50" s="4" t="inlineStr">
         <is>
-          <t>https://www.jpmorganchase.com/careers/explore-opportunities/programs/career-edyou</t>
+          <t>https://jefferies.tal.net/vx/mobile-0/candidate/jobboard/vacancy/2/feed</t>
         </is>
       </c>
       <c r="F50" s="3" t="inlineStr">
         <is>
-          <t>Verified 2026-09-26: 'designed for college sophomores studying in the United States'.</t>
+          <t>Verified 2026-09-26: Oleeo Atom feed, 60 entries. Banking is lower priority than quant.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
         <is>
-          <t>Already watched by jpmc-fellowship</t>
+          <t>Already watched by jhuapl-internships</t>
         </is>
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>JPMC Fellowship Program</t>
+          <t>Johns Hopkins APL internships</t>
         </is>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>Tech internship</t>
-        </is>
-      </c>
-      <c r="D51" s="6" t="inlineStr">
-        <is>
-          <t>LATER</t>
+          <t>Research / math</t>
+        </is>
+      </c>
+      <c r="D51" s="5" t="inlineStr">
+        <is>
+          <t>CHECK</t>
         </is>
       </c>
       <c r="E51" s="4" t="inlineStr">
         <is>
-          <t>https://www.jpmorganchase.com/careers/explore-opportunities/programs/jpmcfellowship</t>
+          <t>https://www.jhuapl.edu/careers/internships</t>
         </is>
       </c>
       <c r="F51" s="3" t="inlineStr">
         <is>
-          <t>Verified 2026-09-26: 'sophomore students, including, without limitation, Black, Hispanic and Latino... All sophomore students... regardless of background, are welcome'.</t>
+          <t>Page states a minimum GPA requirement. Simplify already carries some APL postings; this watches the programme page itself.</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="3" t="inlineStr">
         <is>
-          <t>Already watched by jumptrading-greenhouse</t>
+          <t>Already watched by jpmc-career-edyou</t>
         </is>
       </c>
       <c r="B52" s="3" t="inlineStr">
         <is>
-          <t>Jump Trading Campus Jump Early Access</t>
+          <t>JPMorganChase Career.edYOU Academy</t>
         </is>
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>Quant firm program</t>
-        </is>
-      </c>
-      <c r="D52" s="2" t="inlineStr">
-        <is>
-          <t>YES</t>
+          <t>Tech internship</t>
+        </is>
+      </c>
+      <c r="D52" s="6" t="inlineStr">
+        <is>
+          <t>LATER</t>
         </is>
       </c>
       <c r="E52" s="4" t="inlineStr">
         <is>
-          <t>https://www.jumptrading.com/hr/students-new-grads</t>
+          <t>https://www.jpmorganchase.com/careers/explore-opportunities/programs/career-edyou</t>
         </is>
       </c>
       <c r="F52" s="3" t="inlineStr">
         <is>
-          <t>Verified 2026-09-30 from the 2026 posting: 'First-year undergraduates at US universities' in math/CS/physics/stats/engineering/econ. One-day programme in Chicago, travel/meals/lodging covered. Posts on the Greenhouse board watched by jumptrading-greenhouse; not live today.</t>
+          <t>Verified 2026-09-26: 'designed for college sophomores studying in the United States'.</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="3" t="inlineStr">
         <is>
-          <t>Already watched by kkr-greenhouse</t>
+          <t>Already watched by jpmc-fellowship</t>
         </is>
       </c>
       <c r="B53" s="3" t="inlineStr">
         <is>
-          <t>KKR Scholars Program</t>
+          <t>JPMC Fellowship Program</t>
         </is>
       </c>
       <c r="C53" s="3" t="inlineStr">
         <is>
-          <t>Quant firm program</t>
-        </is>
-      </c>
-      <c r="D53" s="2" t="inlineStr">
-        <is>
-          <t>YES</t>
+          <t>Tech internship</t>
+        </is>
+      </c>
+      <c r="D53" s="6" t="inlineStr">
+        <is>
+          <t>LATER</t>
         </is>
       </c>
       <c r="E53" s="4" t="inlineStr">
         <is>
-          <t>https://www.kkr.com/careers/student-careers/student-career-opportunities</t>
+          <t>https://www.jpmorganchase.com/careers/explore-opportunities/programs/jpmcfellowship</t>
         </is>
       </c>
       <c r="F53" s="3" t="inlineStr">
         <is>
-          <t>2025 posting: 'rising sophomores graduating with a Bachelor's degree in December 2027 – June 2028'. The 2027 edition should be Dec 2029-Jun 2030, the owner's window. Late-May dates may clash with Stanford spring quarter. Posts on KKR's Greenhouse board, slug 'staged'.</t>
+          <t>Verified 2026-09-26: 'sophomore students, including, without limitation, Black, Hispanic and Latino... All sophomore students... regardless of background, are welcome'.</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="3" t="inlineStr">
         <is>
-          <t>Already watched by kleinerperkins-fellows-ashby</t>
+          <t>Already watched by jumptrading-greenhouse</t>
         </is>
       </c>
       <c r="B54" s="3" t="inlineStr">
         <is>
-          <t>Kleiner Perkins Engineering Fellows</t>
+          <t>Jump Trading Campus Jump Early Access</t>
         </is>
       </c>
       <c r="C54" s="3" t="inlineStr">
         <is>
-          <t>Tech internship</t>
-        </is>
-      </c>
-      <c r="D54" s="5" t="inlineStr">
-        <is>
-          <t>CHECK</t>
+          <t>Quant firm program</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
       <c r="E54" s="4" t="inlineStr">
         <is>
-          <t>https://www.kleinerperkins.com/fellows/</t>
+          <t>https://www.jumptrading.com/hr/students-new-grads</t>
         </is>
       </c>
       <c r="F54" s="3" t="inlineStr">
         <is>
-          <t>Verified 2026-09-30 from the Ashby posting: no class-year gate; wants 'Degree in computer science, engineering, math, physics or other fields related to software engineering' and Bay Area availability. Summer placement at a KP portfolio startup plus speaker series. Selective, and cohorts skew upperclass.</t>
+          <t>Verified 2026-09-30 from the 2026 posting: 'First-year undergraduates at US universities' in math/CS/physics/stats/engineering/econ. One-day programme in Chicago, travel/meals/lodging covered. Posts on the Greenhouse board watched by jumptrading-greenhouse; not live today.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="3" t="inlineStr">
         <is>
-          <t>Already watched by lahacks</t>
+          <t>Already watched by kkr-greenhouse</t>
         </is>
       </c>
       <c r="B55" s="3" t="inlineStr">
         <is>
-          <t>LA Hacks</t>
+          <t>KKR Scholars Program</t>
         </is>
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>Competition</t>
-        </is>
-      </c>
-      <c r="D55" s="5" t="inlineStr">
-        <is>
-          <t>CHECK</t>
+          <t>Quant firm program</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
       <c r="E55" s="4" t="inlineStr">
         <is>
-          <t>https://www.lahacks.com/</t>
+          <t>https://www.kkr.com/careers/student-careers/student-career-opportunities</t>
         </is>
       </c>
       <c r="F55" s="3" t="inlineStr">
         <is>
-          <t>Verified 2026-10-08: 'LA Hacks is open to college students of all skill levels'; 'hosted at UCLA's Pauley Pavilion ... in Mid-April 2027'. The FAQ has a 'Travel Reimbursement' tab, but its answer is not in the served HTML, so whether travel is reimbursed for 2027 is unverified.</t>
+          <t>2025 posting: 'rising sophomores graduating with a Bachelor's degree in December 2027 – June 2028'. The 2027 edition should be Dec 2029-Jun 2030, the owner's window. Late-May dates may clash with Stanford spring quarter. Posts on KKR's Greenhouse board, slug 'staged'.</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="3" t="inlineStr">
         <is>
-          <t>Already watched by lanl-students</t>
+          <t>Already watched by kleinerperkins-fellows-ashby</t>
         </is>
       </c>
       <c r="B56" s="3" t="inlineStr">
         <is>
-          <t>LANL student internships (Los Alamos National Laboratory)</t>
+          <t>Kleiner Perkins Engineering Fellows</t>
         </is>
       </c>
       <c r="C56" s="3" t="inlineStr">
         <is>
-          <t>Research / math</t>
+          <t>Tech internship</t>
         </is>
       </c>
       <c r="D56" s="5" t="inlineStr">
@@ -13702,29 +13804,29 @@
       </c>
       <c r="E56" s="4" t="inlineStr">
         <is>
-          <t>https://www.lanl.gov/engage/collaboration/internships</t>
+          <t>https://www.kleinerperkins.com/fellows/</t>
         </is>
       </c>
       <c r="F56" s="3" t="inlineStr">
         <is>
-          <t>Lab-run undergraduate internship programme. The old /careers/career-options/student-internships URL redirects here.</t>
+          <t>Verified 2026-09-30 from the Ashby posting: no class-year gate; wants 'Degree in computer science, engineering, math, physics or other fields related to software engineering' and Bay Area availability. Summer placement at a KP portfolio startup plus speaker series. Selective, and cohorts skew upperclass.</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="3" t="inlineStr">
         <is>
-          <t>Already watched by llnl-students</t>
+          <t>Already watched by lahacks</t>
         </is>
       </c>
       <c r="B57" s="3" t="inlineStr">
         <is>
-          <t>LLNL student internships (Lawrence Livermore National Laboratory)</t>
+          <t>LA Hacks</t>
         </is>
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t>Research / math</t>
+          <t>Competition</t>
         </is>
       </c>
       <c r="D57" s="5" t="inlineStr">
@@ -13734,52 +13836,56 @@
       </c>
       <c r="E57" s="4" t="inlineStr">
         <is>
-          <t>https://www.llnl.gov/join-our-team/careers/student-internship-veteran-programs</t>
+          <t>https://www.lahacks.com/</t>
         </is>
       </c>
       <c r="F57" s="3" t="inlineStr">
         <is>
-          <t>Undergraduate summer internships plus internally and externally sponsored student programmes. Not part of DOE SULI's lab list in this file.</t>
+          <t>Verified 2026-10-08: 'LA Hacks is open to college students of all skill levels'; 'hosted at UCLA's Pauley Pavilion ... in Mid-April 2027'. The FAQ has a 'Travel Reimbursement' tab, but its answer is not in the served HTML, so whether travel is reimbursed for 2027 is unverified.</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="3" t="inlineStr">
         <is>
-          <t>Already watched by luisae</t>
+          <t>Already watched by lanl-students</t>
         </is>
       </c>
       <c r="B58" s="3" t="inlineStr">
         <is>
-          <t>LuisaE/opportunities</t>
+          <t>LANL student internships (Los Alamos National Laboratory)</t>
         </is>
       </c>
       <c r="C58" s="3" t="inlineStr">
         <is>
-          <t>Tracker / resource</t>
-        </is>
-      </c>
-      <c r="D58" s="2" t="inlineStr">
-        <is>
-          <t>USE</t>
+          <t>Research / math</t>
+        </is>
+      </c>
+      <c r="D58" s="5" t="inlineStr">
+        <is>
+          <t>CHECK</t>
         </is>
       </c>
       <c r="E58" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/LuisaE/opportunities</t>
-        </is>
-      </c>
-      <c r="F58" s="3" t="inlineStr"/>
+          <t>https://www.lanl.gov/engage/collaboration/internships</t>
+        </is>
+      </c>
+      <c r="F58" s="3" t="inlineStr">
+        <is>
+          <t>Lab-run undergraduate internship programme. The old /careers/career-options/student-internships URL redirects here.</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="3" t="inlineStr">
         <is>
-          <t>Already watched by mathprograms-listing</t>
+          <t>Already watched by llnl-students</t>
         </is>
       </c>
       <c r="B59" s="3" t="inlineStr">
         <is>
-          <t>MathPrograms.org programme listing</t>
+          <t>LLNL student internships (Lawrence Livermore National Laboratory)</t>
         </is>
       </c>
       <c r="C59" s="3" t="inlineStr">
@@ -13794,61 +13900,57 @@
       </c>
       <c r="E59" s="4" t="inlineStr">
         <is>
-          <t>https://www.mathprograms.org/db/program</t>
+          <t>https://www.llnl.gov/join-our-team/careers/student-internship-veteran-programs</t>
         </is>
       </c>
       <c r="F59" s="3" t="inlineStr">
         <is>
-          <t>Verified 2026-09-26: AMS-run application portal most math REUs use (UChicago, PCMI, Polymath Jr); already lists POLYMATHREU2027 and SLMath PROOF 2027. Substitutes for the NSF REU directory (AWS WAF challenge) and the AMS REU list (403), neither readable by this client.</t>
+          <t>Undergraduate summer internships plus internally and externally sponsored student programmes. Not part of DOE SULI's lab list in this file.</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="3" t="inlineStr">
         <is>
-          <t>Already watched by meta-hacker-cup</t>
+          <t>Already watched by luisae</t>
         </is>
       </c>
       <c r="B60" s="3" t="inlineStr">
         <is>
-          <t>Meta Hacker Cup</t>
+          <t>LuisaE/opportunities</t>
         </is>
       </c>
       <c r="C60" s="3" t="inlineStr">
         <is>
-          <t>Competition</t>
-        </is>
-      </c>
-      <c r="D60" s="5" t="inlineStr">
-        <is>
-          <t>CHECK</t>
+          <t>Tracker / resource</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>USE</t>
         </is>
       </c>
       <c r="E60" s="4" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/codingcompetitions/hacker-cup</t>
-        </is>
-      </c>
-      <c r="F60" s="3" t="inlineStr">
-        <is>
-          <t>Verified 2026-09-26: 'Open to participants around the world'. Page still shows the 2025 season. JavaScript page: 15 chars plain, 1,485 rendered.</t>
-        </is>
-      </c>
+          <t>https://github.com/LuisaE/opportunities</t>
+        </is>
+      </c>
+      <c r="F60" s="3" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="3" t="inlineStr">
         <is>
-          <t>Already watched by millennium-eightfold</t>
+          <t>Already watched by mathprograms-listing</t>
         </is>
       </c>
       <c r="B61" s="3" t="inlineStr">
         <is>
-          <t>Meet Millennium</t>
+          <t>MathPrograms.org programme listing</t>
         </is>
       </c>
       <c r="C61" s="3" t="inlineStr">
         <is>
-          <t>Quant firm program</t>
+          <t>Research / math</t>
         </is>
       </c>
       <c r="D61" s="5" t="inlineStr">
@@ -13858,24 +13960,24 @@
       </c>
       <c r="E61" s="4" t="inlineStr">
         <is>
-          <t>https://www.mlp.com/life-at-millennium/inside-meet-millennium/</t>
+          <t>https://www.mathprograms.org/db/program</t>
         </is>
       </c>
       <c r="F61" s="3" t="inlineStr">
         <is>
-          <t>Verified 2026-09-30: 'high-performing undergraduate and master's students ... Designed as an insight into Millennium's 2027 Summer Intern Program'. Travel to one of five offices; SWE/quant-engineering simulations. www.mlp.com is WP Engine, so not watched directly; the posting should surface via millennium-eightfold.</t>
+          <t>Verified 2026-09-26: AMS-run application portal most math REUs use (UChicago, PCMI, Polymath Jr); already lists POLYMATHREU2027 and SLMath PROOF 2027. Substitutes for the NSF REU directory (AWS WAF challenge) and the AMS REU list (403), neither readable by this client.</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="3" t="inlineStr">
         <is>
-          <t>Already watched by mit-battlecode-2027</t>
+          <t>Already watched by meta-hacker-cup</t>
         </is>
       </c>
       <c r="B62" s="3" t="inlineStr">
         <is>
-          <t>MIT Battlecode 2027</t>
+          <t>Meta Hacker Cup</t>
         </is>
       </c>
       <c r="C62" s="3" t="inlineStr">
@@ -13890,24 +13992,24 @@
       </c>
       <c r="E62" s="4" t="inlineStr">
         <is>
-          <t>https://battlecode.org/</t>
+          <t>https://www.facebook.com/codingcompetitions/hacker-cup</t>
         </is>
       </c>
       <c r="F62" s="3" t="inlineStr">
         <is>
-          <t>MIT's real-time strategy AI competition: you write an autonomous player that commands a robot army, then compete in scrimmages and bracketed tournaments over January. Over $20,000 in total prize money. Open beyond MIT - 'Anyone can write a bot, create a team, and participate in scrimmage matches/rankings.' Prize-tournament gates from the Full Eligibility Rules (battlecode.org/about.html): Sprint Tournaments - 'All teams are eligible.' US Qualifier - 'Teams must consist entirely of US college students studying full-time, or in a transition phase.' Final Tournament - 'Teams must have qualified via the US or International Qualifier.' MIT Newbie Tournament is MIT-only and High School Tournament is high-school-only, so neither applies. Unlike MIT Pokerbots, no MIT-affiliated teammate or MIT certificate is needed for the track you would enter. As of Sep 2026 the site still reads 'Battlecode 2026 ended on January 31st, 2026!' - no 2027 registration date posted yet, though the page already references Battlecode 2027 sponsorships. No team size limit, age limit, or citizenship rule beyond 'US college student' was stated on the pages read. Source: battlecode.org home page and about.html.</t>
+          <t>Verified 2026-09-26: 'Open to participants around the world'. Page still shows the 2025 season. JavaScript page: 15 chars plain, 1,485 rendered.</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="3" t="inlineStr">
         <is>
-          <t>Already watched by mit-trading-competition</t>
+          <t>Already watched by miami-stock-pitch</t>
         </is>
       </c>
       <c r="B63" s="3" t="inlineStr">
         <is>
-          <t>Traders@MIT Trading Competition</t>
+          <t>Miami University - Cleveland Research Intercollegiate Stock Pitch Competition</t>
         </is>
       </c>
       <c r="C63" s="3" t="inlineStr">
@@ -13915,36 +14017,36 @@
           <t>Competition</t>
         </is>
       </c>
-      <c r="D63" s="2" t="inlineStr">
-        <is>
-          <t>YES</t>
+      <c r="D63" s="5" t="inlineStr">
+        <is>
+          <t>CHECK</t>
         </is>
       </c>
       <c r="E63" s="4" t="inlineStr">
         <is>
-          <t>https://traders.mit.edu/competition</t>
+          <t>https://miamioh.edu/fsb/departments/finance/stock-pitch.html</t>
         </is>
       </c>
       <c r="F63" s="3" t="inlineStr">
         <is>
-          <t>Largest intercollegiate competition, $20,000+. NOT the same as Pokerbots - this one IS open to first-years.</t>
+          <t>Verified 2026-10-08 on the official page, which still describes the 2026 edition: "Each team of 2-4 students will assemble a slide deck to pitch a long or short equity position with a 3-12 month horizon." "interested teams must register by the end of the day on March 6"; non-Miami teams submit a written proposal (max 20 slides) by Mar 25; finalists attend a dinner Apr 9 and present in person Apr 10 in Oxford, OH, judged by Cleveland Research Company. Prizes $1,500 / $1,000 / $500. No class-year restriction stated on the page.</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="3" t="inlineStr">
         <is>
-          <t>Already watched by mitll-students</t>
+          <t>Already watched by millennium-eightfold</t>
         </is>
       </c>
       <c r="B64" s="3" t="inlineStr">
         <is>
-          <t>MIT Lincoln Laboratory student opportunities</t>
+          <t>Meet Millennium</t>
         </is>
       </c>
       <c r="C64" s="3" t="inlineStr">
         <is>
-          <t>Research / math</t>
+          <t>Quant firm program</t>
         </is>
       </c>
       <c r="D64" s="5" t="inlineStr">
@@ -13954,61 +14056,61 @@
       </c>
       <c r="E64" s="4" t="inlineStr">
         <is>
-          <t>https://www.ll.mit.edu/careers/student-opportunities</t>
+          <t>https://www.mlp.com/life-at-millennium/inside-meet-millennium/</t>
         </is>
       </c>
       <c r="F64" s="3" t="inlineStr">
         <is>
-          <t>Several tracks. The industry-mentor programme is for students in their junior year; the Summer Research Program takes undergraduate and graduate students.</t>
+          <t>Verified 2026-09-30: 'high-performing undergraduate and master's students ... Designed as an insight into Millennium's 2027 Summer Intern Program'. Travel to one of five offices; SWE/quant-engineering simulations. www.mlp.com is WP Engine, so not watched directly; the posting should surface via millennium-eightfold.</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="3" t="inlineStr">
         <is>
-          <t>Already watched by mlh-season-events</t>
+          <t>Already watched by mit-battlecode-2027</t>
         </is>
       </c>
       <c r="B65" s="3" t="inlineStr">
         <is>
-          <t>MLH hackathon season calendar</t>
+          <t>MIT Battlecode 2027</t>
         </is>
       </c>
       <c r="C65" s="3" t="inlineStr">
         <is>
-          <t>Tracker / resource</t>
-        </is>
-      </c>
-      <c r="D65" s="2" t="inlineStr">
-        <is>
-          <t>USE</t>
+          <t>Competition</t>
+        </is>
+      </c>
+      <c r="D65" s="5" t="inlineStr">
+        <is>
+          <t>CHECK</t>
         </is>
       </c>
       <c r="E65" s="4" t="inlineStr">
         <is>
-          <t>https://www.mlh.com/seasons/2027/events</t>
+          <t>https://battlecode.org/</t>
         </is>
       </c>
       <c r="F65" s="3" t="inlineStr">
         <is>
-          <t>Verified 2026-09-30: MLH's official season calendar (e.g. Gator Quant Hacks, MHacks, Oct 2026). Too high-churn for page_text; treat as a manual/calendar pointer. Correction 2026-10-08: now watched as page_text (source mlh-season-events); one Change per day at most, so the churn is bounded.</t>
+          <t>MIT's real-time strategy AI competition: you write an autonomous player that commands a robot army, then compete in scrimmages and bracketed tournaments over January. Over $20,000 in total prize money. Open beyond MIT - 'Anyone can write a bot, create a team, and participate in scrimmage matches/rankings.' Prize-tournament gates from the Full Eligibility Rules (battlecode.org/about.html): Sprint Tournaments - 'All teams are eligible.' US Qualifier - 'Teams must consist entirely of US college students studying full-time, or in a transition phase.' Final Tournament - 'Teams must have qualified via the US or International Qualifier.' MIT Newbie Tournament is MIT-only and High School Tournament is high-school-only, so neither applies. Unlike MIT Pokerbots, no MIT-affiliated teammate or MIT certificate is needed for the track you would enter. As of Sep 2026 the site still reads 'Battlecode 2026 ended on January 31st, 2026!' - no 2027 registration date posted yet, though the page already references Battlecode 2027 sponsorships. No team size limit, age limit, or citizenship rule beyond 'US college student' was stated on the pages read. Source: battlecode.org home page and about.html.</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="3" t="inlineStr">
         <is>
-          <t>Already watched by nist-surf</t>
+          <t>Already watched by mit-trading-competition</t>
         </is>
       </c>
       <c r="B66" s="3" t="inlineStr">
         <is>
-          <t>NIST SURF</t>
+          <t>Traders@MIT Trading Competition</t>
         </is>
       </c>
       <c r="C66" s="3" t="inlineStr">
         <is>
-          <t>Research / math</t>
+          <t>Competition</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
@@ -14018,24 +14120,24 @@
       </c>
       <c r="E66" s="4" t="inlineStr">
         <is>
-          <t>https://www.nist.gov/surf</t>
+          <t>https://traders.mit.edu/competition</t>
         </is>
       </c>
       <c r="F66" s="3" t="inlineStr">
         <is>
-          <t>Verified 2026-09-30: 'only open to U.S. citizens and U.S. permanent residents enrolled as undergraduate students at U.S. colleges or universities'; states no class-year minimum. 11 weeks, $710/week plus lodging/travel allowance. Information Technology Lab has math/CS/ML projects.</t>
+          <t>Largest intercollegiate competition, $20,000+. NOT the same as Pokerbots - this one IS open to first-years.</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="3" t="inlineStr">
         <is>
-          <t>Already watched by nsa-students</t>
+          <t>Already watched by mitll-students</t>
         </is>
       </c>
       <c r="B67" s="3" t="inlineStr">
         <is>
-          <t>NSA student programs</t>
+          <t>MIT Lincoln Laboratory student opportunities</t>
         </is>
       </c>
       <c r="C67" s="3" t="inlineStr">
@@ -14050,24 +14152,24 @@
       </c>
       <c r="E67" s="4" t="inlineStr">
         <is>
-          <t>https://www.intelligencecareers.gov/nsa/students</t>
+          <t>https://www.ll.mit.edu/careers/student-opportunities</t>
         </is>
       </c>
       <c r="F67" s="3" t="inlineStr">
         <is>
-          <t>NSA's student internship and co-op listings on intelligencecareers.gov. Security clearance means US citizens only.</t>
+          <t>Several tracks. The industry-mentor programme is for students in their junior year; the Summer Research Program takes undergraduate and graduate students.</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="3" t="inlineStr">
         <is>
-          <t>Already watched by nuft-2027</t>
+          <t>Already watched by mlh-season-events</t>
         </is>
       </c>
       <c r="B68" s="3" t="inlineStr">
         <is>
-          <t>NUFT 2027 Quant Internships</t>
+          <t>MLH hackathon season calendar</t>
         </is>
       </c>
       <c r="C68" s="3" t="inlineStr">
@@ -14077,66 +14179,66 @@
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>USE WEEKLY</t>
+          <t>USE</t>
         </is>
       </c>
       <c r="E68" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/northwesternfintech/2027QuantInternships</t>
+          <t>https://www.mlh.com/seasons/2027/events</t>
         </is>
       </c>
       <c r="F68" s="3" t="inlineStr">
         <is>
-          <t>47 firms. No class-year tags - use as a firm checklist and open each careers page yourself.</t>
+          <t>Verified 2026-09-30: MLH's official season calendar (e.g. Gator Quant Hacks, MHacks, Oct 2026). Too high-churn for page_text; treat as a manual/calendar pointer. Correction 2026-10-08: now watched as page_text (source mlh-season-events); one Change per day at most, so the churn is bounded.</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="3" t="inlineStr">
         <is>
-          <t>Already watched by open-source-quantitative-finance</t>
+          <t>Already watched by nist-surf</t>
         </is>
       </c>
       <c r="B69" s="3" t="inlineStr">
         <is>
-          <t>Open Source Quantitative Finance Conference</t>
+          <t>NIST SURF</t>
         </is>
       </c>
       <c r="C69" s="3" t="inlineStr">
         <is>
-          <t>Conference / other</t>
-        </is>
-      </c>
-      <c r="D69" s="5" t="inlineStr">
-        <is>
-          <t>CHECK</t>
+          <t>Research / math</t>
+        </is>
+      </c>
+      <c r="D69" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
       <c r="E69" s="4" t="inlineStr">
         <is>
-          <t>https://osqf.org/</t>
+          <t>https://www.nist.gov/surf</t>
         </is>
       </c>
       <c r="F69" s="3" t="inlineStr">
         <is>
-          <t>Open-source quant finance conference, free per the article. Christina Qi's 2026 quant competitions &amp; events list (LinkedIn Pulse), read 2026-09-06. Verify format and whether students may attend.</t>
+          <t>Verified 2026-09-30: 'only open to U.S. citizens and U.S. permanent residents enrolled as undergraduate students at U.S. colleges or universities'; states no class-year minimum. 11 weeks, $710/week plus lodging/travel allowance. Information Technology Lab has math/CS/ML projects.</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="3" t="inlineStr">
         <is>
-          <t>Already watched by optiver-futurefocus</t>
+          <t>Already watched by nsa-students</t>
         </is>
       </c>
       <c r="B70" s="3" t="inlineStr">
         <is>
-          <t>Optiver FutureFocus Chicago 2026</t>
+          <t>NSA student programs</t>
         </is>
       </c>
       <c r="C70" s="3" t="inlineStr">
         <is>
-          <t>Quant firm program</t>
+          <t>Research / math</t>
         </is>
       </c>
       <c r="D70" s="5" t="inlineStr">
@@ -14146,57 +14248,61 @@
       </c>
       <c r="E70" s="4" t="inlineStr">
         <is>
-          <t>https://optiver.com/recruitment-events/futurefocus-chicago</t>
+          <t>https://www.intelligencecareers.gov/nsa/students</t>
         </is>
       </c>
       <c r="F70" s="3" t="inlineStr">
         <is>
-          <t>Optiver's US (Chicago) student recruitment event. The other FutureFocus and Career Kickstarter events are ANZ, China, Singapore, India and Europe - see the consolidated non-US row. Christina Qi's 2026 quant competitions &amp; events list (LinkedIn Pulse), read 2026-09-06.</t>
+          <t>NSA's student internship and co-op listings on intelligencecareers.gov. Security clearance means US citizens only.</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="3" t="inlineStr">
         <is>
-          <t>Already watched by optiver-ready-trader</t>
+          <t>Already watched by nuft-2027</t>
         </is>
       </c>
       <c r="B71" s="3" t="inlineStr">
         <is>
-          <t>Optiver Ready Trader Go</t>
+          <t>NUFT 2027 Quant Internships</t>
         </is>
       </c>
       <c r="C71" s="3" t="inlineStr">
         <is>
-          <t>Quant firm program</t>
-        </is>
-      </c>
-      <c r="D71" s="5" t="inlineStr">
-        <is>
-          <t>CHECK</t>
+          <t>Tracker / resource</t>
+        </is>
+      </c>
+      <c r="D71" s="2" t="inlineStr">
+        <is>
+          <t>USE WEEKLY</t>
         </is>
       </c>
       <c r="E71" s="4" t="inlineStr">
         <is>
-          <t>https://optiver.com/working-at-optiver/career-opportunities/</t>
-        </is>
-      </c>
-      <c r="F71" s="3" t="inlineStr"/>
+          <t>https://github.com/northwesternfintech/2027QuantInternships</t>
+        </is>
+      </c>
+      <c r="F71" s="3" t="inlineStr">
+        <is>
+          <t>47 firms. No class-year tags - use as a firm checklist and open each careers page yourself.</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="3" t="inlineStr">
         <is>
-          <t>Already watched by purdue-srop</t>
+          <t>Already watched by open-source-quantitative-finance</t>
         </is>
       </c>
       <c r="B72" s="3" t="inlineStr">
         <is>
-          <t>Purdue Summer Research Opportunities Program (SROP)</t>
+          <t>Open Source Quantitative Finance Conference</t>
         </is>
       </c>
       <c r="C72" s="3" t="inlineStr">
         <is>
-          <t>Research / math</t>
+          <t>Conference / other</t>
         </is>
       </c>
       <c r="D72" s="5" t="inlineStr">
@@ -14206,71 +14312,71 @@
       </c>
       <c r="E72" s="4" t="inlineStr">
         <is>
-          <t>https://www.purdue.edu/academics/ogsps/ogrs/summer-research-opportunity-program/</t>
+          <t>https://osqf.org/</t>
         </is>
       </c>
       <c r="F72" s="3" t="inlineStr">
         <is>
-          <t>Part of the Big Ten Academic Alliance SROP. Page states eligibility includes US citizens, permanent residents, refugees and asylees enrolled at a US institution; read the full criteria on the page.</t>
+          <t>Open-source quant finance conference, free per the article. Christina Qi's 2026 quant competitions &amp; events list (LinkedIn Pulse), read 2026-09-06. Verify format and whether students may attend.</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="3" t="inlineStr">
         <is>
-          <t>Already watched by ramp-ashby</t>
+          <t>Already watched by optiver-futurefocus</t>
         </is>
       </c>
       <c r="B73" s="3" t="inlineStr">
         <is>
-          <t>Ramp Emerging Talent</t>
+          <t>Optiver FutureFocus Chicago 2026</t>
         </is>
       </c>
       <c r="C73" s="3" t="inlineStr">
         <is>
-          <t>Tech internship</t>
-        </is>
-      </c>
-      <c r="D73" s="2" t="inlineStr">
-        <is>
-          <t>YES</t>
+          <t>Quant firm program</t>
+        </is>
+      </c>
+      <c r="D73" s="5" t="inlineStr">
+        <is>
+          <t>CHECK</t>
         </is>
       </c>
       <c r="E73" s="4" t="inlineStr">
         <is>
-          <t>https://ramp.com/emerging-talent</t>
+          <t>https://optiver.com/recruitment-events/futurefocus-chicago</t>
         </is>
       </c>
       <c r="F73" s="3" t="inlineStr">
         <is>
-          <t>Verified 2026-09-30: 'For interns: anyone who will be registered in an accredited 4 year university post-internship.' Fintech SWE internships posted on Ashby 'ramp'.</t>
+          <t>Optiver's US (Chicago) student recruitment event. The other FutureFocus and Career Kickstarter events are ANZ, China, Singapore, India and Europe - see the consolidated non-US row. Christina Qi's 2026 quant competitions &amp; events list (LinkedIn Pulse), read 2026-09-06.</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="3" t="inlineStr">
         <is>
-          <t>Already watched by reufinder-freshmen</t>
+          <t>Already watched by optiver-ready-trader</t>
         </is>
       </c>
       <c r="B74" s="3" t="inlineStr">
         <is>
-          <t>REU Finder - freshman-eligible filter</t>
+          <t>Optiver Ready Trader Go</t>
         </is>
       </c>
       <c r="C74" s="3" t="inlineStr">
         <is>
-          <t>Research / math</t>
-        </is>
-      </c>
-      <c r="D74" s="2" t="inlineStr">
-        <is>
-          <t>YES</t>
+          <t>Quant firm program</t>
+        </is>
+      </c>
+      <c r="D74" s="5" t="inlineStr">
+        <is>
+          <t>CHECK</t>
         </is>
       </c>
       <c r="E74" s="4" t="inlineStr">
         <is>
-          <t>https://reufinder.com/programs-for-freshmen/</t>
+          <t>https://optiver.com/working-at-optiver/career-opportunities/</t>
         </is>
       </c>
       <c r="F74" s="3" t="inlineStr"/>
@@ -14278,76 +14384,76 @@
     <row r="75">
       <c r="A75" s="3" t="inlineStr">
         <is>
-          <t>Already watched by sandia-students</t>
+          <t>Already watched by princeton-stock-pitch</t>
         </is>
       </c>
       <c r="B75" s="3" t="inlineStr">
         <is>
-          <t>Sandia National Laboratories student internships</t>
+          <t>Princeton Stock Pitch (Tiger Investments)</t>
         </is>
       </c>
       <c r="C75" s="3" t="inlineStr">
         <is>
-          <t>Research / math</t>
+          <t>Competition</t>
         </is>
       </c>
       <c r="D75" s="5" t="inlineStr">
         <is>
-          <t>CHECK</t>
+          <t>VIA CLUB</t>
         </is>
       </c>
       <c r="E75" s="4" t="inlineStr">
         <is>
-          <t>https://www.sandia.gov/careers/careers/students-and-postdocs/</t>
+          <t>https://princetonstockpitch.vercel.app/</t>
         </is>
       </c>
       <c r="F75" s="3" t="inlineStr">
         <is>
-          <t>Undergraduate and graduate internships across Sandia's sites.</t>
+          <t>Verified 2026-10-08 on the official page: "open to student investment clubs nationwide"; "Who can enter: Open to all student investment clubs. Teams of 3-5 members." Free, virtual; 3-5 page memo, presentation and model on one long or short idea over $2B market cap. Tentative 2027 dates: submissions Mar 5, finalists Mar 12, live Zoom finals Mar 15. Prize pool ~$6,000. Entry is through a club, so a Stanford investing club team is the route in; no class-year restriction stated.</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="3" t="inlineStr">
         <is>
-          <t>Already watched by scudem</t>
+          <t>Already watched by purdue-srop</t>
         </is>
       </c>
       <c r="B76" s="3" t="inlineStr">
         <is>
-          <t>SCUDEM XI 2026</t>
+          <t>Purdue Summer Research Opportunities Program (SROP)</t>
         </is>
       </c>
       <c r="C76" s="3" t="inlineStr">
         <is>
-          <t>Competition</t>
-        </is>
-      </c>
-      <c r="D76" s="2" t="inlineStr">
-        <is>
-          <t>YES</t>
+          <t>Research / math</t>
+        </is>
+      </c>
+      <c r="D76" s="5" t="inlineStr">
+        <is>
+          <t>CHECK</t>
         </is>
       </c>
       <c r="E76" s="4" t="inlineStr">
         <is>
-          <t>https://www.contest.comap.com/scudem/index.html</t>
+          <t>https://www.purdue.edu/academics/ogsps/ogrs/summer-research-opportunity-program/</t>
         </is>
       </c>
       <c r="F76" s="3" t="inlineStr">
         <is>
-          <t>Verified 2026-09-30: COMAP's differential-equations modelling challenge. FAQ: 'open to teams of 3 undergraduate or high school students. Each team must have a coach (typically a faculty member or instructor).' Ends in a 10-minute video judged by at least 3 judges. Needs a faculty coach.</t>
+          <t>Part of the Big Ten Academic Alliance SROP. Page states eligibility includes US citizens, permanent residents, refugees and asylees enrolled at a US institution; read the full criteria on the page.</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="3" t="inlineStr">
         <is>
-          <t>Already watched by seo-tech</t>
+          <t>Already watched by ramp-ashby</t>
         </is>
       </c>
       <c r="B77" s="3" t="inlineStr">
         <is>
-          <t>SEO Tech Developer + First-Year Academy</t>
+          <t>Ramp Emerging Talent</t>
         </is>
       </c>
       <c r="C77" s="3" t="inlineStr">
@@ -14355,63 +14461,59 @@
           <t>Tech internship</t>
         </is>
       </c>
-      <c r="D77" s="5" t="inlineStr">
-        <is>
-          <t>CHECK</t>
+      <c r="D77" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
       <c r="E77" s="4" t="inlineStr">
         <is>
-          <t>https://tech.seo-usa.org/</t>
+          <t>https://ramp.com/emerging-talent</t>
         </is>
       </c>
       <c r="F77" s="3" t="inlineStr">
         <is>
-          <t>Verified 2026-09-26: 'Enrolled as a sophomore'; the Academy is for 'first-year college students'. Page says 'All are welcome to apply'; SEO is a diversity organisation, so confirm eligibility by hand.</t>
+          <t>Verified 2026-09-30: 'For interns: anyone who will be registered in an accredited 4 year university post-internship.' Fintech SWE internships posted on Ashby 'ramp'.</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="3" t="inlineStr">
         <is>
-          <t>Already watched by sfhacks</t>
+          <t>Already watched by reufinder-freshmen</t>
         </is>
       </c>
       <c r="B78" s="3" t="inlineStr">
         <is>
-          <t>SF Hacks</t>
+          <t>REU Finder - freshman-eligible filter</t>
         </is>
       </c>
       <c r="C78" s="3" t="inlineStr">
         <is>
-          <t>Competition</t>
-        </is>
-      </c>
-      <c r="D78" s="5" t="inlineStr">
-        <is>
-          <t>CHECK</t>
+          <t>Research / math</t>
+        </is>
+      </c>
+      <c r="D78" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
       <c r="E78" s="4" t="inlineStr">
         <is>
-          <t>https://www.sfhacks.io/</t>
-        </is>
-      </c>
-      <c r="F78" s="3" t="inlineStr">
-        <is>
-          <t>Verified 2026-10-08: 'All students are welcome, from high school through university.' 'We are not offering travel reimbursements this year.' San Francisco.</t>
-        </is>
-      </c>
+          <t>https://reufinder.com/programs-for-freshmen/</t>
+        </is>
+      </c>
+      <c r="F78" s="3" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" s="3" t="inlineStr">
         <is>
-          <t>Already watched by sfi-ucr</t>
+          <t>Already watched by sandia-students</t>
         </is>
       </c>
       <c r="B79" s="3" t="inlineStr">
         <is>
-          <t>SFI Undergraduate Complexity Research</t>
+          <t>Sandia National Laboratories student internships</t>
         </is>
       </c>
       <c r="C79" s="3" t="inlineStr">
@@ -14426,61 +14528,61 @@
       </c>
       <c r="E79" s="4" t="inlineStr">
         <is>
-          <t>https://www.santafe.edu/engage/learn/programs/undergraduate-complexity-research</t>
+          <t>https://www.sandia.gov/careers/careers/students-and-postdocs/</t>
         </is>
       </c>
       <c r="F79" s="3" t="inlineStr">
         <is>
-          <t>Verified 2026-09-26: 'for current undergraduate students. Prior research experience is not required'; 'return to this page in November 2026'.</t>
+          <t>Undergraduate and graduate internships across Sandia's sites.</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="3" t="inlineStr">
         <is>
-          <t>Already watched by simplify-2027</t>
+          <t>Already watched by scudem</t>
         </is>
       </c>
       <c r="B80" s="3" t="inlineStr">
         <is>
-          <t>SimplifyJobs Summer 2027 Internships</t>
+          <t>SCUDEM XI 2026</t>
         </is>
       </c>
       <c r="C80" s="3" t="inlineStr">
         <is>
-          <t>Tracker / resource</t>
-        </is>
-      </c>
-      <c r="D80" s="6" t="inlineStr">
-        <is>
-          <t>LOW VALUE</t>
+          <t>Competition</t>
+        </is>
+      </c>
+      <c r="D80" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
       <c r="E80" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/SimplifyJobs/Summer2027-Internships</t>
+          <t>https://www.contest.comap.com/scudem/index.html</t>
         </is>
       </c>
       <c r="F80" s="3" t="inlineStr">
         <is>
-          <t>613 roles, 94 quant, but no class-year tagging and almost all target penultimate-year students.</t>
+          <t>Verified 2026-09-30: COMAP's differential-equations modelling challenge. FAQ: 'open to teams of 3 undergraduate or high school students. Each team must have a coach (typically a faculty member or instructor).' Ends in a 10-minute video judged by at least 3 judges. Needs a faculty coach.</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="3" t="inlineStr">
         <is>
-          <t>Already watched by sjhacks</t>
+          <t>Already watched by seo-tech</t>
         </is>
       </c>
       <c r="B81" s="3" t="inlineStr">
         <is>
-          <t>SJHacks</t>
+          <t>SEO Tech Developer + First-Year Academy</t>
         </is>
       </c>
       <c r="C81" s="3" t="inlineStr">
         <is>
-          <t>Competition</t>
+          <t>Tech internship</t>
         </is>
       </c>
       <c r="D81" s="5" t="inlineStr">
@@ -14490,29 +14592,29 @@
       </c>
       <c r="E81" s="4" t="inlineStr">
         <is>
-          <t>https://www.sjhacks.com/</t>
+          <t>https://tech.seo-usa.org/</t>
         </is>
       </c>
       <c r="F81" s="3" t="inlineStr">
         <is>
-          <t>Verified 2026-10-08: 'SJHacks is a 24-hour in-person hackathon at San Jose State University'; 2026 edition April 25-26 at Guildhouse, San Jose. The page states no eligibility rule and nothing about travel.</t>
+          <t>Verified 2026-09-26: 'Enrolled as a sophomore'; the Academy is for 'first-year college students'. Page says 'All are welcome to apply'; SEO is a diversity organisation, so confirm eligibility by hand.</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="3" t="inlineStr">
         <is>
-          <t>Already watched by smart-scholarship</t>
+          <t>Already watched by sfhacks</t>
         </is>
       </c>
       <c r="B82" s="3" t="inlineStr">
         <is>
-          <t>SMART Scholarship</t>
+          <t>SF Hacks</t>
         </is>
       </c>
       <c r="C82" s="3" t="inlineStr">
         <is>
-          <t>Conference / other</t>
+          <t>Competition</t>
         </is>
       </c>
       <c r="D82" s="5" t="inlineStr">
@@ -14522,29 +14624,29 @@
       </c>
       <c r="E82" s="4" t="inlineStr">
         <is>
-          <t>https://www.smartscholarship.org/smart</t>
+          <t>https://www.sfhacks.io/</t>
         </is>
       </c>
       <c r="F82" s="3" t="inlineStr">
         <is>
-          <t>Verified 2026-09-26: scholarship-for-service - requires civilian employment with the Department of War after graduation. 'open annually from August 1 to the first Friday in December'.</t>
+          <t>Verified 2026-10-08: 'All students are welcome, from high school through university.' 'We are not offering travel reimbursements this year.' San Francisco.</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="3" t="inlineStr">
         <is>
-          <t>Already watched by stevens-high-frequency-trading</t>
+          <t>Already watched by sfi-ucr</t>
         </is>
       </c>
       <c r="B83" s="3" t="inlineStr">
         <is>
-          <t>Stevens High Frequency Trading Competition 2026</t>
+          <t>SFI Undergraduate Complexity Research</t>
         </is>
       </c>
       <c r="C83" s="3" t="inlineStr">
         <is>
-          <t>Competition</t>
+          <t>Research / math</t>
         </is>
       </c>
       <c r="D83" s="5" t="inlineStr">
@@ -14554,56 +14656,56 @@
       </c>
       <c r="E83" s="4" t="inlineStr">
         <is>
-          <t>https://www.stevens.edu/page-basic/2026-stevens-high-frequency-trading-competition</t>
+          <t>https://www.santafe.edu/engage/learn/programs/undergraduate-complexity-research</t>
         </is>
       </c>
       <c r="F83" s="3" t="inlineStr">
         <is>
-          <t>HFT-focused student competition at Stevens Institute (Hoboken NJ). Christina Qi's 2026 quant competitions &amp; events list (LinkedIn Pulse), read 2026-09-06. Directly relevant to quant dev; verify class-year eligibility.</t>
+          <t>Verified 2026-09-26: 'for current undergraduate students. Prior research experience is not required'; 'return to this page in November 2026'.</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="3" t="inlineStr">
         <is>
-          <t>Already watched by surim-apply</t>
+          <t>Already watched by simplify-2027</t>
         </is>
       </c>
       <c r="B84" s="3" t="inlineStr">
         <is>
-          <t>Stanford SURIM</t>
+          <t>SimplifyJobs Summer 2027 Internships</t>
         </is>
       </c>
       <c r="C84" s="3" t="inlineStr">
         <is>
-          <t>Stanford-only</t>
-        </is>
-      </c>
-      <c r="D84" s="2" t="inlineStr">
-        <is>
-          <t>YES</t>
+          <t>Tracker / resource</t>
+        </is>
+      </c>
+      <c r="D84" s="6" t="inlineStr">
+        <is>
+          <t>LOW VALUE</t>
         </is>
       </c>
       <c r="E84" s="4" t="inlineStr">
         <is>
-          <t>https://mathematics.stanford.edu/</t>
+          <t>https://github.com/SimplifyJobs/Summer2027-Internships</t>
         </is>
       </c>
       <c r="F84" s="3" t="inlineStr">
         <is>
-          <t>8 weeks, $8,500 + up to $1,500 need-based. Needs MATH 56/61CM/61DM/110/113/115 first, and 2 letters (1 from Stanford Math). | Checked 2026-09-26: SURIM has its own page at surim.stanford.edu/apply-surim, which is watched; the listed mathematics.stanford.edu is kept.</t>
+          <t>613 roles, 94 quant, but no class-year tagging and almost all target penultimate-year students.</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="3" t="inlineStr">
         <is>
-          <t>Already watched by treehacks</t>
+          <t>Already watched by sjhacks</t>
         </is>
       </c>
       <c r="B85" s="3" t="inlineStr">
         <is>
-          <t>TreeHacks</t>
+          <t>SJHacks</t>
         </is>
       </c>
       <c r="C85" s="3" t="inlineStr">
@@ -14618,56 +14720,56 @@
       </c>
       <c r="E85" s="4" t="inlineStr">
         <is>
-          <t>https://treehacks.com/</t>
+          <t>https://www.sjhacks.com/</t>
         </is>
       </c>
       <c r="F85" s="3" t="inlineStr">
         <is>
-          <t>Verified 2026-09-26: 'open to any enrolled college student'; Stanford students get priority by the priority deadline.</t>
+          <t>Verified 2026-10-08: 'SJHacks is a 24-hour in-person hackathon at San Jose State University'; 2026 edition April 25-26 at Guildhouse, San Jose. The page states no eligibility rule and nothing about travel.</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="3" t="inlineStr">
         <is>
-          <t>Already watched by twosigma-campus</t>
+          <t>Already watched by smart-scholarship</t>
         </is>
       </c>
       <c r="B86" s="3" t="inlineStr">
         <is>
-          <t>Two Sigma New Seekers Summit</t>
+          <t>SMART Scholarship</t>
         </is>
       </c>
       <c r="C86" s="3" t="inlineStr">
         <is>
-          <t>Quant firm program</t>
-        </is>
-      </c>
-      <c r="D86" s="2" t="inlineStr">
-        <is>
-          <t>YES</t>
+          <t>Conference / other</t>
+        </is>
+      </c>
+      <c r="D86" s="5" t="inlineStr">
+        <is>
+          <t>CHECK</t>
         </is>
       </c>
       <c r="E86" s="4" t="inlineStr">
         <is>
-          <t>https://www.twosigma.com/new-seekers-summit/</t>
+          <t>https://www.smartscholarship.org/smart</t>
         </is>
       </c>
       <c r="F86" s="3" t="inlineStr">
         <is>
-          <t>Verified 2026-09-30: 'gives first-and second-year undergraduates the opportunity to delve into the world of Data Scientists and Quantitative Researchers.' QR seminars, networking, interview prep. www.twosigma.com is WP Engine, which 403s the Actions runner, so it is not watched as page_text; the posting should appear on twosigma-campus (Avature).</t>
+          <t>Verified 2026-09-26: scholarship-for-service - requires civilian employment with the Department of War after graduation. 'open annually from August 1 to the first Friday in December'.</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="3" t="inlineStr">
         <is>
-          <t>Already watched by uchicago-trading-competition</t>
+          <t>Already watched by stevens-high-frequency-trading</t>
         </is>
       </c>
       <c r="B87" s="3" t="inlineStr">
         <is>
-          <t>UChicago Trading Competition</t>
+          <t>Stevens High Frequency Trading Competition 2026</t>
         </is>
       </c>
       <c r="C87" s="3" t="inlineStr">
@@ -14675,95 +14777,95 @@
           <t>Competition</t>
         </is>
       </c>
-      <c r="D87" s="2" t="inlineStr">
-        <is>
-          <t>YES</t>
+      <c r="D87" s="5" t="inlineStr">
+        <is>
+          <t>CHECK</t>
         </is>
       </c>
       <c r="E87" s="4" t="inlineStr">
         <is>
-          <t>https://tradingcompetition.uchicago.edu/</t>
+          <t>https://www.stevens.edu/page-basic/2026-stevens-high-frequency-trading-competition</t>
         </is>
       </c>
       <c r="F87" s="3" t="inlineStr">
         <is>
-          <t>PRIORITY TO TEAMS WITHOUT PRIOR TRADING WORK EXPERIENCE - structurally favors freshmen. April event, $15k+ prizes.</t>
+          <t>HFT-focused student competition at Stevens Institute (Hoboken NJ). Christina Qi's 2026 quant competitions &amp; events list (LinkedIn Pulse), read 2026-09-06. Directly relevant to quant dev; verify class-year eligibility.</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="3" t="inlineStr">
         <is>
-          <t>Already watched by underclassmen-cruz</t>
+          <t>Already watched by surim-apply</t>
         </is>
       </c>
       <c r="B88" s="3" t="inlineStr">
         <is>
-          <t>underclassmen-opportunities (Cruz-Lopez)</t>
+          <t>Stanford SURIM</t>
         </is>
       </c>
       <c r="C88" s="3" t="inlineStr">
         <is>
-          <t>Tracker / resource</t>
+          <t>Stanford-only</t>
         </is>
       </c>
       <c r="D88" s="2" t="inlineStr">
         <is>
-          <t>USE WEEKLY</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E88" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/Jose-Gael-Cruz-Lopez/underclassmen-opportunities</t>
+          <t>https://mathematics.stanford.edu/</t>
         </is>
       </c>
       <c r="F88" s="3" t="inlineStr">
         <is>
-          <t>Better maintained than zapplyjobs, with open/closing-soon flags. Heavy on ambassador programs - filter hard.</t>
+          <t>8 weeks, $8,500 + up to $1,500 need-based. Needs MATH 56/61CM/61DM/110/113/115 first, and 2 letters (1 from Stanford Math). | Checked 2026-09-26: SURIM has its own page at surim.stanford.edu/apply-surim, which is watched; the listed mathematics.stanford.edu is kept.</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="3" t="inlineStr">
         <is>
-          <t>Already watched by worldquant-iqc</t>
+          <t>Already watched by texas-usit-competitions</t>
         </is>
       </c>
       <c r="B89" s="3" t="inlineStr">
         <is>
-          <t>WorldQuant IQC / BRAIN</t>
+          <t>Texas Stock Pitch (UT Austin USIT)</t>
         </is>
       </c>
       <c r="C89" s="3" t="inlineStr">
         <is>
-          <t>Quant firm program</t>
-        </is>
-      </c>
-      <c r="D89" s="2" t="inlineStr">
-        <is>
-          <t>YES</t>
+          <t>Competition</t>
+        </is>
+      </c>
+      <c r="D89" s="5" t="inlineStr">
+        <is>
+          <t>CHECK</t>
         </is>
       </c>
       <c r="E89" s="4" t="inlineStr">
         <is>
-          <t>https://www.worldquant.com/brain/iqc/</t>
+          <t>https://www.texasusit.org/competitions-overviews</t>
         </is>
       </c>
       <c r="F89" s="3" t="inlineStr">
         <is>
-          <t>Teams of 1-4 from one university. $100k pool. Solo entry allowed. Huge field (140k+ registrations) so mid-table means little.</t>
+          <t>Verified 2026-10-08 on USIT's competitions overview: Texas Stock Pitch is "the largest stock pitch competition in the Southern United States" and "provides undergraduate students from all over the nation with the opportunity to demonstrate their proficiency in investment research, valuation, and presentation"; up to $5,000 in prizes; "This competition will be held in February 2027." Class-year rules, team size and fees are not on this page and were not verified: texasstockpitch.com does not resolve (DNS) and stockpitch.texasusit.org, linked from the page, returned 404 on 2026-10-08. The same page lists Texas Charity Pitch (Nov 2026) and the Analyst Group Stock Pitch, which is for USIT's own members only.</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="3" t="inlineStr">
         <is>
-          <t>Already watched by yhack</t>
+          <t>Already watched by treehacks</t>
         </is>
       </c>
       <c r="B90" s="3" t="inlineStr">
         <is>
-          <t>YHack</t>
+          <t>TreeHacks</t>
         </is>
       </c>
       <c r="C90" s="3" t="inlineStr">
@@ -14778,29 +14880,29 @@
       </c>
       <c r="E90" s="4" t="inlineStr">
         <is>
-          <t>https://www.yhack.org/</t>
+          <t>https://treehacks.com/</t>
         </is>
       </c>
       <c r="F90" s="3" t="inlineStr">
         <is>
-          <t>Verified 2026-10-08: 'Accepted participants will have the opportunity to apply for travel reimbursement. We expect to be able to support many participants traveling from the East Coast, with additional consideration given' beyond it. Yale.</t>
+          <t>Verified 2026-09-26: 'open to any enrolled college student'; Stanford students get priority by the priority deadline.</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="3" t="inlineStr">
         <is>
-          <t>Already watched by yutc</t>
+          <t>Already watched by twosigma-campus</t>
         </is>
       </c>
       <c r="B91" s="3" t="inlineStr">
         <is>
-          <t>Yale Undergraduate Trading Competition</t>
+          <t>Two Sigma New Seekers Summit</t>
         </is>
       </c>
       <c r="C91" s="3" t="inlineStr">
         <is>
-          <t>Competition</t>
+          <t>Quant firm program</t>
         </is>
       </c>
       <c r="D91" s="2" t="inlineStr">
@@ -14810,216 +14912,216 @@
       </c>
       <c r="E91" s="4" t="inlineStr">
         <is>
-          <t>https://www.yale.edu/</t>
+          <t>https://www.twosigma.com/new-seekers-summit/</t>
         </is>
       </c>
       <c r="F91" s="3" t="inlineStr">
         <is>
-          <t>$10,000+ in prizes, nationwide. | Checked 2026-09-26: the competition's own site is yutc.org (a JavaScript page, watched with render_js); the listed yale.edu is kept.</t>
+          <t>Verified 2026-09-30: 'gives first-and second-year undergraduates the opportunity to delve into the world of Data Scientists and Quantitative Researchers.' QR seminars, networking, interview prep. www.twosigma.com is WP Engine, which 403s the Actions runner, so it is not watched as page_text; the posting should appear on twosigma-campus (Avature).</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="3" t="inlineStr">
         <is>
-          <t>You cannot apply (NO)</t>
+          <t>Already watched by uchicago-bluechips-pitch</t>
         </is>
       </c>
       <c r="B92" s="3" t="inlineStr">
         <is>
-          <t>Bank of America APAC Quant Conference</t>
+          <t>UChicago Blue Chips Intercollegiate Stock Pitch Competition</t>
         </is>
       </c>
       <c r="C92" s="3" t="inlineStr">
         <is>
-          <t>Conference / other</t>
-        </is>
-      </c>
-      <c r="D92" s="8" t="inlineStr">
-        <is>
-          <t>NO</t>
+          <t>Competition</t>
+        </is>
+      </c>
+      <c r="D92" s="5" t="inlineStr">
+        <is>
+          <t>CHECK</t>
         </is>
       </c>
       <c r="E92" s="4" t="inlineStr">
         <is>
-          <t>https://www.bofa.com/</t>
+          <t>https://www.tbc.uchicago.edu/pitch-competition</t>
         </is>
       </c>
       <c r="F92" s="3" t="inlineStr">
         <is>
-          <t>Ruled out on geography - APAC, May 20 2026. Christina Qi's 2026 quant competitions &amp; events list (LinkedIn Pulse), read 2026-09-06.</t>
+          <t>Verified 2026-10-08 on the official page: "Our 2026 Intercollegiate Stock Pitch Competition has concluded. Please stay tuned for our 2027 Intercollegiate Stock Pitch Competition, which will be held in March 2027." Requirements: "Teams of 1-3 undergraduates (cross-school teams and international students welcome)", long-only pitch on an NYSE/Nasdaq company over $2B, 15-slide deck plus valuation model, blind submission. 2026 prizes $1,200 / $800 / $400; virtual finals. No class-year restriction stated.</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="3" t="inlineStr">
         <is>
-          <t>You cannot apply (NO)</t>
+          <t>Already watched by uchicago-trading-competition</t>
         </is>
       </c>
       <c r="B93" s="3" t="inlineStr">
         <is>
-          <t>Bridgewater Rising Fellows</t>
+          <t>UChicago Trading Competition</t>
         </is>
       </c>
       <c r="C93" s="3" t="inlineStr">
         <is>
-          <t>Quant firm program</t>
-        </is>
-      </c>
-      <c r="D93" s="8" t="inlineStr">
-        <is>
-          <t>NO</t>
+          <t>Competition</t>
+        </is>
+      </c>
+      <c r="D93" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
       <c r="E93" s="4" t="inlineStr">
         <is>
-          <t>https://www.bridgewater.com/risingfellowsprogram</t>
+          <t>https://tradingcompetition.uchicago.edu/</t>
         </is>
       </c>
       <c r="F93" s="3" t="inlineStr">
         <is>
-          <t>CORRECTED: first-year eligible BUT targets backgrounds underrepresented in the industry, recruiting via HBCUs, O4U, BLK Capital, Prep for Prep. | Checked 2026-09-26: now redirects to the generic /working-at-bridgewater page. Kept: it may reopen.</t>
+          <t>PRIORITY TO TEAMS WITHOUT PRIOR TRADING WORK EXPERIENCE - structurally favors freshmen. April event, $15k+ prizes.</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="3" t="inlineStr">
         <is>
-          <t>You cannot apply (NO)</t>
+          <t>Already watched by umich-uic</t>
         </is>
       </c>
       <c r="B94" s="3" t="inlineStr">
         <is>
-          <t>CQA Young Professionals Event</t>
+          <t>ENGAGE Undergraduate Investment Conference Stock Pitch (Michigan UIC)</t>
         </is>
       </c>
       <c r="C94" s="3" t="inlineStr">
         <is>
-          <t>Conference / other</t>
-        </is>
-      </c>
-      <c r="D94" s="8" t="inlineStr">
-        <is>
-          <t>NO</t>
+          <t>Competition</t>
+        </is>
+      </c>
+      <c r="D94" s="5" t="inlineStr">
+        <is>
+          <t>CHECK</t>
         </is>
       </c>
       <c r="E94" s="4" t="inlineStr">
         <is>
-          <t>https://cqa.org/upcoming-events-cqa-young-professional</t>
+          <t>https://www.umichuic.com/</t>
         </is>
       </c>
       <c r="F94" s="3" t="inlineStr">
         <is>
-          <t>Ruled out on stage - for working professionals, not undergraduates. Christina Qi's 2026 quant competitions &amp; events list (LinkedIn Pulse), read 2026-09-06.</t>
+          <t>Verified 2026-10-08 on the official site. Home page: the conference "will return to the University of Michigan on Saturday, November 14th 2026. Stock Pitch submissions are now live." UIC 19 page: "Each team of 2-4 members will pitch an equity, long or short"; "Each team must submit a one-pager here highlighting their idea by October 28th, 2026 at 11:59pm"; "These one-pagers will be evaluated on a rolling basis". Invited teams must each buy a conference ticket. FAQ: "groups can even be comprised of people across different organizations or different universities." Prizes $7,500 / $2,000 / $1,000. Hosted by Michigan Interactive Investments at Ross. Undergraduate conference; no class-year restriction stated.</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="3" t="inlineStr">
         <is>
-          <t>You cannot apply (NO)</t>
+          <t>Already watched by underclassmen-cruz</t>
         </is>
       </c>
       <c r="B95" s="3" t="inlineStr">
         <is>
-          <t>Citadel Securities Ignite</t>
+          <t>underclassmen-opportunities (Cruz-Lopez)</t>
         </is>
       </c>
       <c r="C95" s="3" t="inlineStr">
         <is>
-          <t>Quant firm program</t>
-        </is>
-      </c>
-      <c r="D95" s="8" t="inlineStr">
-        <is>
-          <t>NO</t>
+          <t>Tracker / resource</t>
+        </is>
+      </c>
+      <c r="D95" s="2" t="inlineStr">
+        <is>
+          <t>USE WEEKLY</t>
         </is>
       </c>
       <c r="E95" s="4" t="inlineStr">
         <is>
-          <t>https://www.citadelsecurities.com/careers/programs-and-events/</t>
+          <t>https://github.com/Jose-Gael-Cruz-Lopez/underclassmen-opportunities</t>
         </is>
       </c>
       <c r="F95" s="3" t="inlineStr">
         <is>
-          <t>Invite-only weeklong program for sophomore women.</t>
+          <t>Better maintained than zapplyjobs, with open/closing-soon flags. Heavy on ambassador programs - filter hard.</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="3" t="inlineStr">
         <is>
-          <t>You cannot apply (NO)</t>
+          <t>Already watched by weiss-greenhouse</t>
         </is>
       </c>
       <c r="B96" s="3" t="inlineStr">
         <is>
-          <t>Coding it Forward - Civic Digital Fellowship</t>
+          <t>Weiss Asset Management 2027 Underclassmen Fellowship</t>
         </is>
       </c>
       <c r="C96" s="3" t="inlineStr">
         <is>
-          <t>Tech internship</t>
-        </is>
-      </c>
-      <c r="D96" s="8" t="inlineStr">
-        <is>
-          <t>NO</t>
+          <t>Quant firm program</t>
+        </is>
+      </c>
+      <c r="D96" s="5" t="inlineStr">
+        <is>
+          <t>CHECK</t>
         </is>
       </c>
       <c r="E96" s="4" t="inlineStr">
         <is>
-          <t>https://www.codingitforward.com/fellowship</t>
+          <t>https://job-boards.greenhouse.io/weissassetmanagement</t>
         </is>
       </c>
       <c r="F96" s="3" t="inlineStr">
         <is>
-          <t>TRAP - appears on most underclassmen lists but 2026 required graduating May 2025-Dec 2027. Diary for junior year.</t>
+          <t>Verified 2026-10-08 on Weiss's Greenhouse board (posting 8831639002, updated 2026-10-02): "This program is only open to current Freshmen and Sophomores (Classes of 2029 and 2030)". Two-day in-person programme in Boston "on January 7th and 8th, 2027"; "All selected students will have their transportation and hotel costs fully covered"; "High-performing fellows may be considered for future internship opportunities." No identity gate stated. No application deadline stated in the posting, so apply early. weissasset.com/careers carries no programme text (893 chars), so the board is the watch target. Source: research notes, Freshman finance programs 2026-27.</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="3" t="inlineStr">
         <is>
-          <t>You cannot apply (NO)</t>
+          <t>Already watched by witg-stock-pitch</t>
         </is>
       </c>
       <c r="B97" s="3" t="inlineStr">
         <is>
-          <t>D. E. Shaw Discovery Fellowship</t>
+          <t>WITG x Fundamental Edge Stock Pitch Competition (Penn)</t>
         </is>
       </c>
       <c r="C97" s="3" t="inlineStr">
         <is>
-          <t>Quant firm program</t>
-        </is>
-      </c>
-      <c r="D97" s="8" t="inlineStr">
-        <is>
-          <t>NO</t>
+          <t>Competition</t>
+        </is>
+      </c>
+      <c r="D97" s="5" t="inlineStr">
+        <is>
+          <t>CHECK</t>
         </is>
       </c>
       <c r="E97" s="4" t="inlineStr">
         <is>
-          <t>https://campus.deshaw.com/fellowships</t>
+          <t>https://www.pennwitg.com/competition</t>
         </is>
       </c>
       <c r="F97" s="3" t="inlineStr">
         <is>
-          <t>Checked 2026-09-26: campus.deshaw.com/fellowships now redirects to the campus root, which mentions no fellowships. Kept; the root is watched as deshaw-campus.</t>
+          <t>Verified 2026-10-08 on the official page: "The competition is open to all university undergraduate students across the United States and internationally who wish to participate. Teams are allowed to cross-register with undergraduates from any school and are able to register in groups of 2-4." Fourth annual edition, hosted by the Wharton Investment &amp; Trading Group. Dates: registration opened Sep 21, 2026; "Registration and First Round Executive Summary Deadline ... Monday, October 19, 2026 at 11:59PM EST"; finalists Oct 22; final round Oct 28 at Huntsman Hall with a virtual option. No class-year restriction stated.</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="3" t="inlineStr">
         <is>
-          <t>You cannot apply (NO)</t>
+          <t>Already watched by worldquant-iqc</t>
         </is>
       </c>
       <c r="B98" s="3" t="inlineStr">
         <is>
-          <t>D. E. Shaw Latitude Fellowship</t>
+          <t>WorldQuant IQC / BRAIN</t>
         </is>
       </c>
       <c r="C98" s="3" t="inlineStr">
@@ -15027,83 +15129,83 @@
           <t>Quant firm program</t>
         </is>
       </c>
-      <c r="D98" s="8" t="inlineStr">
-        <is>
-          <t>NO</t>
+      <c r="D98" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
       <c r="E98" s="4" t="inlineStr">
         <is>
-          <t>https://campus.deshaw.com/fellowships</t>
+          <t>https://www.worldquant.com/brain/iqc/</t>
         </is>
       </c>
       <c r="F98" s="3" t="inlineStr">
         <is>
-          <t>Checked 2026-09-26: campus.deshaw.com/fellowships now redirects to the campus root, which mentions no fellowships. Kept; the root is watched as deshaw-campus.</t>
+          <t>Teams of 1-4 from one university. $100k pool. Solo entry allowed. Huge field (140k+ registrations) so mid-table means little.</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="3" t="inlineStr">
         <is>
-          <t>You cannot apply (NO)</t>
+          <t>Already watched by yhack</t>
         </is>
       </c>
       <c r="B99" s="3" t="inlineStr">
         <is>
-          <t>D. E. Shaw London Insight Programme</t>
+          <t>YHack</t>
         </is>
       </c>
       <c r="C99" s="3" t="inlineStr">
         <is>
-          <t>Quant firm program</t>
-        </is>
-      </c>
-      <c r="D99" s="8" t="inlineStr">
-        <is>
-          <t>NO</t>
+          <t>Competition</t>
+        </is>
+      </c>
+      <c r="D99" s="5" t="inlineStr">
+        <is>
+          <t>CHECK</t>
         </is>
       </c>
       <c r="E99" s="4" t="inlineStr">
         <is>
-          <t>https://campus.deshaw.com/additional-experiences</t>
+          <t>https://www.yhack.org/</t>
         </is>
       </c>
       <c r="F99" s="3" t="inlineStr">
         <is>
-          <t>Ruled out on geography - London. Christina Qi's 2026 quant competitions &amp; events list (LinkedIn Pulse), read 2026-09-06. | Checked 2026-09-26: campus.deshaw.com/additional-experiences now redirects to the campus root (which lists London Insight as closed). Kept.</t>
+          <t>Verified 2026-10-08: 'Accepted participants will have the opportunity to apply for travel reimbursement. We expect to be able to support many participants traveling from the East Coast, with additional consideration given' beyond it. Yale.</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="3" t="inlineStr">
         <is>
-          <t>You cannot apply (NO)</t>
+          <t>Already watched by yutc</t>
         </is>
       </c>
       <c r="B100" s="3" t="inlineStr">
         <is>
-          <t>D. E. Shaw Momentum Fellowship</t>
+          <t>Yale Undergraduate Trading Competition</t>
         </is>
       </c>
       <c r="C100" s="3" t="inlineStr">
         <is>
-          <t>Quant firm program</t>
-        </is>
-      </c>
-      <c r="D100" s="8" t="inlineStr">
-        <is>
-          <t>NO</t>
+          <t>Competition</t>
+        </is>
+      </c>
+      <c r="D100" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
       <c r="E100" s="4" t="inlineStr">
         <is>
-          <t>https://campus.deshaw.com/fellowships</t>
+          <t>https://www.yale.edu/</t>
         </is>
       </c>
       <c r="F100" s="3" t="inlineStr">
         <is>
-          <t>Checked 2026-09-26: campus.deshaw.com/fellowships now redirects to the campus root, which mentions no fellowships. Kept; the root is watched as deshaw-campus.</t>
+          <t>$10,000+ in prizes, nationwide. | Checked 2026-09-26: the competition's own site is yutc.org (a JavaScript page, watched with render_js); the listed yale.edu is kept.</t>
         </is>
       </c>
     </row>
@@ -15115,7 +15217,7 @@
       </c>
       <c r="B101" s="3" t="inlineStr">
         <is>
-          <t>Databento partner quant events (Shanghai, London)</t>
+          <t>Bank of America APAC Quant Conference</t>
         </is>
       </c>
       <c r="C101" s="3" t="inlineStr">
@@ -15130,12 +15232,12 @@
       </c>
       <c r="E101" s="4" t="inlineStr">
         <is>
-          <t>https://databento.com/</t>
+          <t>https://www.bofa.com/</t>
         </is>
       </c>
       <c r="F101" s="3" t="inlineStr">
         <is>
-          <t>Consolidated row for the Databento events with Nasdaq/Bank of America (Shanghai, May 21 2026), Google (London, June 2026) and Man Group (London, June 2026). Ruled out on geography. Christina Qi's 2026 quant competitions &amp; events list (LinkedIn Pulse), read 2026-09-06.</t>
+          <t>Ruled out on geography - APAC, May 20 2026. Christina Qi's 2026 quant competitions &amp; events list (LinkedIn Pulse), read 2026-09-06.</t>
         </is>
       </c>
     </row>
@@ -15147,12 +15249,12 @@
       </c>
       <c r="B102" s="3" t="inlineStr">
         <is>
-          <t>Global Crypto Quant Competition and Digital Asset Forum Hong Kong 2026</t>
+          <t>Bridgewater Rising Fellows</t>
         </is>
       </c>
       <c r="C102" s="3" t="inlineStr">
         <is>
-          <t>Competition</t>
+          <t>Quant firm program</t>
         </is>
       </c>
       <c r="D102" s="8" t="inlineStr">
@@ -15162,12 +15264,12 @@
       </c>
       <c r="E102" s="4" t="inlineStr">
         <is>
-          <t>https://en.tmtpost.com/post/7752441</t>
+          <t>https://www.bridgewater.com/risingfellowsprogram</t>
         </is>
       </c>
       <c r="F102" s="3" t="inlineStr">
         <is>
-          <t>Ruled out on geography - Hong Kong. Christina Qi's 2026 quant competitions &amp; events list (LinkedIn Pulse), read 2026-09-06.</t>
+          <t>CORRECTED: first-year eligible BUT targets backgrounds underrepresented in the industry, recruiting via HBCUs, O4U, BLK Capital, Prep for Prep. | Checked 2026-09-26: now redirects to the generic /working-at-bridgewater page. Kept: it may reopen.</t>
         </is>
       </c>
     </row>
@@ -15179,12 +15281,12 @@
       </c>
       <c r="B103" s="3" t="inlineStr">
         <is>
-          <t>IMC EU Business Course</t>
+          <t>CQA Young Professionals Event</t>
         </is>
       </c>
       <c r="C103" s="3" t="inlineStr">
         <is>
-          <t>Quant firm program</t>
+          <t>Conference / other</t>
         </is>
       </c>
       <c r="D103" s="8" t="inlineStr">
@@ -15194,12 +15296,12 @@
       </c>
       <c r="E103" s="4" t="inlineStr">
         <is>
-          <t>https://www.imc.com/eu/careers/students-graduates/programs/business-course</t>
+          <t>https://cqa.org/upcoming-events-cqa-young-professional</t>
         </is>
       </c>
       <c r="F103" s="3" t="inlineStr">
         <is>
-          <t>Ruled out on geography - EU. The US Launchpad program is tracked separately. Christina Qi's 2026 quant competitions &amp; events list (LinkedIn Pulse), read 2026-09-06.</t>
+          <t>Ruled out on stage - for working professionals, not undergraduates. Christina Qi's 2026 quant competitions &amp; events list (LinkedIn Pulse), read 2026-09-06.</t>
         </is>
       </c>
     </row>
@@ -15211,7 +15313,7 @@
       </c>
       <c r="B104" s="3" t="inlineStr">
         <is>
-          <t>IMC UK Masterclass</t>
+          <t>Citadel Securities Ignite</t>
         </is>
       </c>
       <c r="C104" s="3" t="inlineStr">
@@ -15226,12 +15328,12 @@
       </c>
       <c r="E104" s="4" t="inlineStr">
         <is>
-          <t>https://careers.imc.com/</t>
+          <t>https://www.citadelsecurities.com/careers/programs-and-events/</t>
         </is>
       </c>
       <c r="F104" s="3" t="inlineStr">
         <is>
-          <t>Geographic exclusion - excludes US-based students.</t>
+          <t>Invite-only weeklong program for sophomore women.</t>
         </is>
       </c>
     </row>
@@ -15243,12 +15345,12 @@
       </c>
       <c r="B105" s="3" t="inlineStr">
         <is>
-          <t>IMC WiT (Women in Technology)</t>
+          <t>Coding it Forward - Civic Digital Fellowship</t>
         </is>
       </c>
       <c r="C105" s="3" t="inlineStr">
         <is>
-          <t>Quant firm program</t>
+          <t>Tech internship</t>
         </is>
       </c>
       <c r="D105" s="8" t="inlineStr">
@@ -15258,10 +15360,14 @@
       </c>
       <c r="E105" s="4" t="inlineStr">
         <is>
-          <t>https://careers.imc.com/us/en/student-opportunities</t>
-        </is>
-      </c>
-      <c r="F105" s="3" t="inlineStr"/>
+          <t>https://www.codingitforward.com/fellowship</t>
+        </is>
+      </c>
+      <c r="F105" s="3" t="inlineStr">
+        <is>
+          <t>TRAP - appears on most underclassmen lists but 2026 required graduating May 2025-Dec 2027. Diary for junior year.</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="3" t="inlineStr">
@@ -15271,7 +15377,7 @@
       </c>
       <c r="B106" s="3" t="inlineStr">
         <is>
-          <t>IMC Women in Trading and Engineering</t>
+          <t>D. E. Shaw Discovery Fellowship</t>
         </is>
       </c>
       <c r="C106" s="3" t="inlineStr">
@@ -15286,12 +15392,12 @@
       </c>
       <c r="E106" s="4" t="inlineStr">
         <is>
-          <t>https://www.imc.com/ap/careers/students-graduates/programs/womens-talent</t>
+          <t>https://campus.deshaw.com/fellowships</t>
         </is>
       </c>
       <c r="F106" s="3" t="inlineStr">
         <is>
-          <t>Ruled out by an identity gate: this program is for women. Christina Qi's 2026 quant competitions &amp; events list (LinkedIn Pulse), read 2026-09-06. Listed here so it is not re-researched.</t>
+          <t>Checked 2026-09-26: campus.deshaw.com/fellowships now redirects to the campus root, which mentions no fellowships. Kept; the root is watched as deshaw-campus.</t>
         </is>
       </c>
     </row>
@@ -15303,12 +15409,12 @@
       </c>
       <c r="B107" s="3" t="inlineStr">
         <is>
-          <t>JPMorgan Data for Good Hackathon</t>
+          <t>D. E. Shaw Latitude Fellowship</t>
         </is>
       </c>
       <c r="C107" s="3" t="inlineStr">
         <is>
-          <t>Conference / other</t>
+          <t>Quant firm program</t>
         </is>
       </c>
       <c r="D107" s="8" t="inlineStr">
@@ -15318,12 +15424,12 @@
       </c>
       <c r="E107" s="4" t="inlineStr">
         <is>
-          <t>https://careers.jpmorgan.com/</t>
+          <t>https://campus.deshaw.com/fellowships</t>
         </is>
       </c>
       <c r="F107" s="3" t="inlineStr">
         <is>
-          <t>That is a junior-year window; a first-year does not qualify.</t>
+          <t>Checked 2026-09-26: campus.deshaw.com/fellowships now redirects to the campus root, which mentions no fellowships. Kept; the root is watched as deshaw-campus.</t>
         </is>
       </c>
     </row>
@@ -15335,7 +15441,7 @@
       </c>
       <c r="B108" s="3" t="inlineStr">
         <is>
-          <t>Jane Street FOCUS and IN FOCUS</t>
+          <t>D. E. Shaw London Insight Programme</t>
         </is>
       </c>
       <c r="C108" s="3" t="inlineStr">
@@ -15350,12 +15456,12 @@
       </c>
       <c r="E108" s="4" t="inlineStr">
         <is>
-          <t>https://www.janestreet.com/join-jane-street/programs-and-events/</t>
+          <t>https://campus.deshaw.com/additional-experiences</t>
         </is>
       </c>
       <c r="F108" s="3" t="inlineStr">
         <is>
-          <t>Barriers-to-access criteria (first-gen, Pell-eligible, under-resourced school). Read criteria yourself.</t>
+          <t>Ruled out on geography - London. Christina Qi's 2026 quant competitions &amp; events list (LinkedIn Pulse), read 2026-09-06. | Checked 2026-09-26: campus.deshaw.com/additional-experiences now redirects to the campus root (which lists London Insight as closed). Kept.</t>
         </is>
       </c>
     </row>
@@ -15367,7 +15473,7 @@
       </c>
       <c r="B109" s="3" t="inlineStr">
         <is>
-          <t>Jane Street Graduate Research Fellowship</t>
+          <t>D. E. Shaw Momentum Fellowship</t>
         </is>
       </c>
       <c r="C109" s="3" t="inlineStr">
@@ -15382,10 +15488,14 @@
       </c>
       <c r="E109" s="4" t="inlineStr">
         <is>
-          <t>https://www.janestreet.com/join-jane-street/programs-and-events/</t>
-        </is>
-      </c>
-      <c r="F109" s="3" t="inlineStr"/>
+          <t>https://campus.deshaw.com/fellowships</t>
+        </is>
+      </c>
+      <c r="F109" s="3" t="inlineStr">
+        <is>
+          <t>Checked 2026-09-26: campus.deshaw.com/fellowships now redirects to the campus root, which mentions no fellowships. Kept; the root is watched as deshaw-campus.</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="3" t="inlineStr">
@@ -15395,12 +15505,12 @@
       </c>
       <c r="B110" s="3" t="inlineStr">
         <is>
-          <t>Jane Street INSIGHT</t>
+          <t>Databento partner quant events (Shanghai, London)</t>
         </is>
       </c>
       <c r="C110" s="3" t="inlineStr">
         <is>
-          <t>Quant firm program</t>
+          <t>Conference / other</t>
         </is>
       </c>
       <c r="D110" s="8" t="inlineStr">
@@ -15410,12 +15520,12 @@
       </c>
       <c r="E110" s="4" t="inlineStr">
         <is>
-          <t>https://www.janestreet.com/join-jane-street/programs-and-events/insight/</t>
+          <t>https://databento.com/</t>
         </is>
       </c>
       <c r="F110" s="3" t="inlineStr">
         <is>
-          <t>For women, transgender and gender-expansive people.</t>
+          <t>Consolidated row for the Databento events with Nasdaq/Bank of America (Shanghai, May 21 2026), Google (London, June 2026) and Man Group (London, June 2026). Ruled out on geography. Christina Qi's 2026 quant competitions &amp; events list (LinkedIn Pulse), read 2026-09-06.</t>
         </is>
       </c>
     </row>
@@ -15427,12 +15537,12 @@
       </c>
       <c r="B111" s="3" t="inlineStr">
         <is>
-          <t>Jane Street JSIP</t>
+          <t>Global Crypto Quant Competition and Digital Asset Forum Hong Kong 2026</t>
         </is>
       </c>
       <c r="C111" s="3" t="inlineStr">
         <is>
-          <t>Quant firm program</t>
+          <t>Competition</t>
         </is>
       </c>
       <c r="D111" s="8" t="inlineStr">
@@ -15442,12 +15552,12 @@
       </c>
       <c r="E111" s="4" t="inlineStr">
         <is>
-          <t>https://www.janestreet.com/join-jane-street/programs-and-events/jsip/</t>
+          <t>https://en.tmtpost.com/post/7752441</t>
         </is>
       </c>
       <c r="F111" s="3" t="inlineStr">
         <is>
-          <t>Multi-week paid NYC program, $12,500 scholarship - but requires having experienced barriers to access in CS. | Checked 2026-09-26: now redirects to the programs-and-events index, which does not list JSIP. Kept: it may reopen for the next cycle.</t>
+          <t>Ruled out on geography - Hong Kong. Christina Qi's 2026 quant competitions &amp; events list (LinkedIn Pulse), read 2026-09-06.</t>
         </is>
       </c>
     </row>
@@ -15459,7 +15569,7 @@
       </c>
       <c r="B112" s="3" t="inlineStr">
         <is>
-          <t>Jane Street Visiting Researcher / Prefaculty</t>
+          <t>IMC EU Business Course</t>
         </is>
       </c>
       <c r="C112" s="3" t="inlineStr">
@@ -15474,10 +15584,14 @@
       </c>
       <c r="E112" s="4" t="inlineStr">
         <is>
-          <t>https://www.janestreet.com/join-jane-street/programs-and-events/</t>
-        </is>
-      </c>
-      <c r="F112" s="3" t="inlineStr"/>
+          <t>https://www.imc.com/eu/careers/students-graduates/programs/business-course</t>
+        </is>
+      </c>
+      <c r="F112" s="3" t="inlineStr">
+        <is>
+          <t>Ruled out on geography - EU. The US Launchpad program is tracked separately. Christina Qi's 2026 quant competitions &amp; events list (LinkedIn Pulse), read 2026-09-06.</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="3" t="inlineStr">
@@ -15487,7 +15601,7 @@
       </c>
       <c r="B113" s="3" t="inlineStr">
         <is>
-          <t>Jane Street WiSE</t>
+          <t>IMC UK Masterclass</t>
         </is>
       </c>
       <c r="C113" s="3" t="inlineStr">
@@ -15502,12 +15616,12 @@
       </c>
       <c r="E113" s="4" t="inlineStr">
         <is>
-          <t>https://www.janestreet.com/join-jane-street/programs-and-events/</t>
+          <t>https://careers.imc.com/</t>
         </is>
       </c>
       <c r="F113" s="3" t="inlineStr">
         <is>
-          <t>Women / trans / gender-expansive students.</t>
+          <t>Geographic exclusion - excludes US-based students.</t>
         </is>
       </c>
     </row>
@@ -15519,12 +15633,12 @@
       </c>
       <c r="B114" s="3" t="inlineStr">
         <is>
-          <t>KNHack 2026 Research Challenge (Mexico)</t>
+          <t>IMC WiT (Women in Technology)</t>
         </is>
       </c>
       <c r="C114" s="3" t="inlineStr">
         <is>
-          <t>Competition</t>
+          <t>Quant firm program</t>
         </is>
       </c>
       <c r="D114" s="8" t="inlineStr">
@@ -15534,14 +15648,10 @@
       </c>
       <c r="E114" s="4" t="inlineStr">
         <is>
-          <t>https://kaxanuk.mx/kn-hack</t>
-        </is>
-      </c>
-      <c r="F114" s="3" t="inlineStr">
-        <is>
-          <t>Ruled out on geography - Mexico. Christina Qi's 2026 quant competitions &amp; events list (LinkedIn Pulse), read 2026-09-06.</t>
-        </is>
-      </c>
+          <t>https://careers.imc.com/us/en/student-opportunities</t>
+        </is>
+      </c>
+      <c r="F114" s="3" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" s="3" t="inlineStr">
@@ -15551,12 +15661,12 @@
       </c>
       <c r="B115" s="3" t="inlineStr">
         <is>
-          <t>MIT Pokerbots</t>
+          <t>IMC Women in Trading and Engineering</t>
         </is>
       </c>
       <c r="C115" s="3" t="inlineStr">
         <is>
-          <t>Competition</t>
+          <t>Quant firm program</t>
         </is>
       </c>
       <c r="D115" s="8" t="inlineStr">
@@ -15566,12 +15676,12 @@
       </c>
       <c r="E115" s="4" t="inlineStr">
         <is>
-          <t>https://pokerbots.org/</t>
+          <t>https://www.imc.com/ap/careers/students-graduates/programs/womens-talent</t>
         </is>
       </c>
       <c r="F115" s="3" t="inlineStr">
         <is>
-          <t>Must be able to register for MIT IAP classes; a team member needs MIT certificates for the competition server.</t>
+          <t>Ruled out by an identity gate: this program is for women. Christina Qi's 2026 quant competitions &amp; events list (LinkedIn Pulse), read 2026-09-06. Listed here so it is not re-researched.</t>
         </is>
       </c>
     </row>
@@ -15583,12 +15693,12 @@
       </c>
       <c r="B116" s="3" t="inlineStr">
         <is>
-          <t>Meta University</t>
+          <t>JPMorgan Data for Good Hackathon</t>
         </is>
       </c>
       <c r="C116" s="3" t="inlineStr">
         <is>
-          <t>Tech internship</t>
+          <t>Conference / other</t>
         </is>
       </c>
       <c r="D116" s="8" t="inlineStr">
@@ -15596,14 +15706,14 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="E116" s="3" t="inlineStr">
-        <is>
-          <t>n/a</t>
+      <c r="E116" s="4" t="inlineStr">
+        <is>
+          <t>https://careers.jpmorgan.com/</t>
         </is>
       </c>
       <c r="F116" s="3" t="inlineStr">
         <is>
-          <t>Discontinued with no replacement. Ignore any list that still includes it.</t>
+          <t>That is a junior-year window; a first-year does not qualify.</t>
         </is>
       </c>
     </row>
@@ -15615,7 +15725,7 @@
       </c>
       <c r="B117" s="3" t="inlineStr">
         <is>
-          <t>Optiver Career Kickstarter: Women in Tech</t>
+          <t>Jane Street FOCUS and IN FOCUS</t>
         </is>
       </c>
       <c r="C117" s="3" t="inlineStr">
@@ -15630,12 +15740,12 @@
       </c>
       <c r="E117" s="4" t="inlineStr">
         <is>
-          <t>https://optiver.com/working-at-optiver/career-opportunities/8177160002</t>
+          <t>https://www.janestreet.com/join-jane-street/programs-and-events/</t>
         </is>
       </c>
       <c r="F117" s="3" t="inlineStr">
         <is>
-          <t>Ruled out by an identity gate: this program is for women. Christina Qi's 2026 quant competitions &amp; events list (LinkedIn Pulse), read 2026-09-06. Listed here so it is not re-researched.</t>
+          <t>Barriers-to-access criteria (first-gen, Pell-eligible, under-resourced school). Read criteria yourself.</t>
         </is>
       </c>
     </row>
@@ -15647,7 +15757,7 @@
       </c>
       <c r="B118" s="3" t="inlineStr">
         <is>
-          <t>Optiver Quantitative Intern Summer 2027</t>
+          <t>Jane Street Graduate Research Fellowship</t>
         </is>
       </c>
       <c r="C118" s="3" t="inlineStr">
@@ -15662,14 +15772,10 @@
       </c>
       <c r="E118" s="4" t="inlineStr">
         <is>
-          <t>https://optiver.com/working-at-optiver/career-opportunities/</t>
-        </is>
-      </c>
-      <c r="F118" s="3" t="inlineStr">
-        <is>
-          <t>Highest pay in the industry, but a first-year is too early.</t>
-        </is>
-      </c>
+          <t>https://www.janestreet.com/join-jane-street/programs-and-events/</t>
+        </is>
+      </c>
+      <c r="F118" s="3" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" s="3" t="inlineStr">
@@ -15679,7 +15785,7 @@
       </c>
       <c r="B119" s="3" t="inlineStr">
         <is>
-          <t>Optiver regional recruitment events (non-US)</t>
+          <t>Jane Street INSIGHT</t>
         </is>
       </c>
       <c r="C119" s="3" t="inlineStr">
@@ -15694,12 +15800,12 @@
       </c>
       <c r="E119" s="4" t="inlineStr">
         <is>
-          <t>https://optiver.com/recruitment-events/</t>
+          <t>https://www.janestreet.com/join-jane-street/programs-and-events/insight/</t>
         </is>
       </c>
       <c r="F119" s="3" t="inlineStr">
         <is>
-          <t>Consolidated row for the ANZ, China, Singapore, India, Amsterdam and Catalunya FutureFocus / Career Kickstarter / masterclass events. Ruled out on geography; the Chicago event is tracked separately. Christina Qi's 2026 quant competitions &amp; events list (LinkedIn Pulse), read 2026-09-06.</t>
+          <t>For women, transgender and gender-expansive people.</t>
         </is>
       </c>
     </row>
@@ -15711,7 +15817,7 @@
       </c>
       <c r="B120" s="3" t="inlineStr">
         <is>
-          <t>PEAK6 Trading Bootcamp</t>
+          <t>Jane Street JSIP</t>
         </is>
       </c>
       <c r="C120" s="3" t="inlineStr">
@@ -15726,12 +15832,12 @@
       </c>
       <c r="E120" s="4" t="inlineStr">
         <is>
-          <t>https://peak6.com/campus/</t>
+          <t>https://www.janestreet.com/join-jane-street/programs-and-events/jsip/</t>
         </is>
       </c>
       <c r="F120" s="3" t="inlineStr">
         <is>
-          <t>One week, $25-31.25/hr, two sessions (May and Aug).</t>
+          <t>Multi-week paid NYC program, $12,500 scholarship - but requires having experienced barriers to access in CS. | Checked 2026-09-26: now redirects to the programs-and-events index, which does not list JSIP. Kept: it may reopen for the next cycle.</t>
         </is>
       </c>
     </row>
@@ -15743,12 +15849,12 @@
       </c>
       <c r="B121" s="3" t="inlineStr">
         <is>
-          <t>Palantir Path</t>
+          <t>Jane Street Visiting Researcher / Prefaculty</t>
         </is>
       </c>
       <c r="C121" s="3" t="inlineStr">
         <is>
-          <t>Tech internship</t>
+          <t>Quant firm program</t>
         </is>
       </c>
       <c r="D121" s="8" t="inlineStr">
@@ -15756,9 +15862,9 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="E121" s="3" t="inlineStr">
-        <is>
-          <t>n/a</t>
+      <c r="E121" s="4" t="inlineStr">
+        <is>
+          <t>https://www.janestreet.com/join-jane-street/programs-and-events/</t>
         </is>
       </c>
       <c r="F121" s="3" t="inlineStr"/>
@@ -15771,7 +15877,7 @@
       </c>
       <c r="B122" s="3" t="inlineStr">
         <is>
-          <t>Point72 Academy</t>
+          <t>Jane Street WiSE</t>
         </is>
       </c>
       <c r="C122" s="3" t="inlineStr">
@@ -15786,12 +15892,12 @@
       </c>
       <c r="E122" s="4" t="inlineStr">
         <is>
-          <t>https://point72.com/point72-academy/</t>
+          <t>https://www.janestreet.com/join-jane-street/programs-and-events/</t>
         </is>
       </c>
       <c r="F122" s="3" t="inlineStr">
         <is>
-          <t>NOT an underclassman program. 10-month paid post-grad program, $125k base. 2027 class wants Dec 2026-Jul 2027 grads.</t>
+          <t>Women / trans / gender-expansive students.</t>
         </is>
       </c>
     </row>
@@ -15803,12 +15909,12 @@
       </c>
       <c r="B123" s="3" t="inlineStr">
         <is>
-          <t>SIG Sophomore Discovery Days for Women (all tracks)</t>
+          <t>KNHack 2026 Research Challenge (Mexico)</t>
         </is>
       </c>
       <c r="C123" s="3" t="inlineStr">
         <is>
-          <t>Quant firm program</t>
+          <t>Competition</t>
         </is>
       </c>
       <c r="D123" s="8" t="inlineStr">
@@ -15818,10 +15924,14 @@
       </c>
       <c r="E123" s="4" t="inlineStr">
         <is>
-          <t>https://careers.sig.com/discovery-programs/jobs</t>
-        </is>
-      </c>
-      <c r="F123" s="3" t="inlineStr"/>
+          <t>https://kaxanuk.mx/kn-hack</t>
+        </is>
+      </c>
+      <c r="F123" s="3" t="inlineStr">
+        <is>
+          <t>Ruled out on geography - Mexico. Christina Qi's 2026 quant competitions &amp; events list (LinkedIn Pulse), read 2026-09-06.</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="3" t="inlineStr">
@@ -15831,12 +15941,12 @@
       </c>
       <c r="B124" s="3" t="inlineStr">
         <is>
-          <t>Two Sigma College Mentor Connect</t>
+          <t>MIT Pokerbots</t>
         </is>
       </c>
       <c r="C124" s="3" t="inlineStr">
         <is>
-          <t>Quant firm program</t>
+          <t>Competition</t>
         </is>
       </c>
       <c r="D124" s="8" t="inlineStr">
@@ -15846,12 +15956,12 @@
       </c>
       <c r="E124" s="4" t="inlineStr">
         <is>
-          <t>https://www.twosigma.com/undergraduate-students/</t>
+          <t>https://pokerbots.org/</t>
         </is>
       </c>
       <c r="F124" s="3" t="inlineStr">
         <is>
-          <t>6-week remote mentorship on open-source projects.</t>
+          <t>Must be able to register for MIT IAP classes; a team member needs MIT certificates for the competition server.</t>
         </is>
       </c>
     </row>
@@ -15863,12 +15973,12 @@
       </c>
       <c r="B125" s="3" t="inlineStr">
         <is>
-          <t>Two Sigma Diversity Undergraduate Scholarship</t>
+          <t>Meta University</t>
         </is>
       </c>
       <c r="C125" s="3" t="inlineStr">
         <is>
-          <t>Quant firm program</t>
+          <t>Tech internship</t>
         </is>
       </c>
       <c r="D125" s="8" t="inlineStr">
@@ -15876,12 +15986,16 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="E125" s="4" t="inlineStr">
-        <is>
-          <t>https://www.twosigma.com/undergraduate-students/</t>
-        </is>
-      </c>
-      <c r="F125" s="3" t="inlineStr"/>
+      <c r="E125" s="3" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F125" s="3" t="inlineStr">
+        <is>
+          <t>Discontinued with no replacement. Ignore any list that still includes it.</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="3" t="inlineStr">
@@ -15891,7 +16005,7 @@
       </c>
       <c r="B126" s="3" t="inlineStr">
         <is>
-          <t>Two Sigma PhD Fellowship</t>
+          <t>Optiver Career Kickstarter: Women in Tech</t>
         </is>
       </c>
       <c r="C126" s="3" t="inlineStr">
@@ -15906,10 +16020,14 @@
       </c>
       <c r="E126" s="4" t="inlineStr">
         <is>
-          <t>https://www.twosigma.com/graduate-students/phd-fellowships/</t>
-        </is>
-      </c>
-      <c r="F126" s="3" t="inlineStr"/>
+          <t>https://optiver.com/working-at-optiver/career-opportunities/8177160002</t>
+        </is>
+      </c>
+      <c r="F126" s="3" t="inlineStr">
+        <is>
+          <t>Ruled out by an identity gate: this program is for women. Christina Qi's 2026 quant competitions &amp; events list (LinkedIn Pulse), read 2026-09-06. Listed here so it is not re-researched.</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="3" t="inlineStr">
@@ -15919,7 +16037,7 @@
       </c>
       <c r="B127" s="3" t="inlineStr">
         <is>
-          <t>Virtu Financial Women's Winternship</t>
+          <t>Optiver Quantitative Intern Summer 2027</t>
         </is>
       </c>
       <c r="C127" s="3" t="inlineStr">
@@ -15934,10 +16052,14 @@
       </c>
       <c r="E127" s="4" t="inlineStr">
         <is>
-          <t>https://www.virtu.com/careers/</t>
-        </is>
-      </c>
-      <c r="F127" s="3" t="inlineStr"/>
+          <t>https://optiver.com/working-at-optiver/career-opportunities/</t>
+        </is>
+      </c>
+      <c r="F127" s="3" t="inlineStr">
+        <is>
+          <t>Highest pay in the industry, but a first-year is too early.</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="3" t="inlineStr">
@@ -15947,12 +16069,12 @@
       </c>
       <c r="B128" s="3" t="inlineStr">
         <is>
-          <t>Wharton Global High School Investment Competition</t>
+          <t>Optiver regional recruitment events (non-US)</t>
         </is>
       </c>
       <c r="C128" s="3" t="inlineStr">
         <is>
-          <t>Competition</t>
+          <t>Quant firm program</t>
         </is>
       </c>
       <c r="D128" s="8" t="inlineStr">
@@ -15962,12 +16084,12 @@
       </c>
       <c r="E128" s="4" t="inlineStr">
         <is>
-          <t>https://globalyouth.wharton.upenn.edu/competitions/investment-competition</t>
+          <t>https://optiver.com/recruitment-events/</t>
         </is>
       </c>
       <c r="F128" s="3" t="inlineStr">
         <is>
-          <t>Ruled out on stage - high school students only. Christina Qi's 2026 quant competitions &amp; events list (LinkedIn Pulse), read 2026-09-06.</t>
+          <t>Consolidated row for the ANZ, China, Singapore, India, Amsterdam and Catalunya FutureFocus / Career Kickstarter / masterclass events. Ruled out on geography; the Chicago event is tracked separately. Christina Qi's 2026 quant competitions &amp; events list (LinkedIn Pulse), read 2026-09-06.</t>
         </is>
       </c>
     </row>
@@ -15979,12 +16101,12 @@
       </c>
       <c r="B129" s="3" t="inlineStr">
         <is>
-          <t>Women in Quantitative Finance Americas Conference</t>
+          <t>PEAK6 Trading Bootcamp</t>
         </is>
       </c>
       <c r="C129" s="3" t="inlineStr">
         <is>
-          <t>Conference / other</t>
+          <t>Quant firm program</t>
         </is>
       </c>
       <c r="D129" s="8" t="inlineStr">
@@ -15994,12 +16116,12 @@
       </c>
       <c r="E129" s="4" t="inlineStr">
         <is>
-          <t>https://www.wbstraining.com/events/wqfa</t>
+          <t>https://peak6.com/campus/</t>
         </is>
       </c>
       <c r="F129" s="3" t="inlineStr">
         <is>
-          <t>Ruled out by an identity gate: this program is for women. Christina Qi's 2026 quant competitions &amp; events list (LinkedIn Pulse), read 2026-09-06. Listed here so it is not re-researched.</t>
+          <t>One week, $25-31.25/hr, two sessions (May and Aug).</t>
         </is>
       </c>
     </row>
@@ -16011,12 +16133,12 @@
       </c>
       <c r="B130" s="3" t="inlineStr">
         <is>
-          <t>Women in Quantitative Finance London Conference</t>
+          <t>Palantir Path</t>
         </is>
       </c>
       <c r="C130" s="3" t="inlineStr">
         <is>
-          <t>Conference / other</t>
+          <t>Tech internship</t>
         </is>
       </c>
       <c r="D130" s="8" t="inlineStr">
@@ -16024,51 +16146,319 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="E130" s="4" t="inlineStr">
-        <is>
-          <t>https://www.wbstraining.com/events/london-wqf-conference</t>
-        </is>
-      </c>
-      <c r="F130" s="3" t="inlineStr">
-        <is>
-          <t>Ruled out by an identity gate: this program is for women. Christina Qi's 2026 quant competitions &amp; events list (LinkedIn Pulse), read 2026-09-06. Listed here so it is not re-researched.</t>
-        </is>
-      </c>
+      <c r="E130" s="3" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F130" s="3" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" s="3" t="inlineStr">
         <is>
+          <t>You cannot apply (NO)</t>
+        </is>
+      </c>
+      <c r="B131" s="3" t="inlineStr">
+        <is>
+          <t>Point72 Academy</t>
+        </is>
+      </c>
+      <c r="C131" s="3" t="inlineStr">
+        <is>
+          <t>Quant firm program</t>
+        </is>
+      </c>
+      <c r="D131" s="8" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E131" s="4" t="inlineStr">
+        <is>
+          <t>https://point72.com/point72-academy/</t>
+        </is>
+      </c>
+      <c r="F131" s="3" t="inlineStr">
+        <is>
+          <t>NOT an underclassman program. 10-month paid post-grad program, $125k base. 2027 class wants Dec 2026-Jul 2027 grads.</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="3" t="inlineStr">
+        <is>
+          <t>You cannot apply (NO)</t>
+        </is>
+      </c>
+      <c r="B132" s="3" t="inlineStr">
+        <is>
+          <t>SIG Sophomore Discovery Days for Women (all tracks)</t>
+        </is>
+      </c>
+      <c r="C132" s="3" t="inlineStr">
+        <is>
+          <t>Quant firm program</t>
+        </is>
+      </c>
+      <c r="D132" s="8" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E132" s="4" t="inlineStr">
+        <is>
+          <t>https://careers.sig.com/discovery-programs/jobs</t>
+        </is>
+      </c>
+      <c r="F132" s="3" t="inlineStr"/>
+    </row>
+    <row r="133">
+      <c r="A133" s="3" t="inlineStr">
+        <is>
+          <t>You cannot apply (NO)</t>
+        </is>
+      </c>
+      <c r="B133" s="3" t="inlineStr">
+        <is>
+          <t>Two Sigma College Mentor Connect</t>
+        </is>
+      </c>
+      <c r="C133" s="3" t="inlineStr">
+        <is>
+          <t>Quant firm program</t>
+        </is>
+      </c>
+      <c r="D133" s="8" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E133" s="4" t="inlineStr">
+        <is>
+          <t>https://www.twosigma.com/undergraduate-students/</t>
+        </is>
+      </c>
+      <c r="F133" s="3" t="inlineStr">
+        <is>
+          <t>6-week remote mentorship on open-source projects.</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="3" t="inlineStr">
+        <is>
+          <t>You cannot apply (NO)</t>
+        </is>
+      </c>
+      <c r="B134" s="3" t="inlineStr">
+        <is>
+          <t>Two Sigma Diversity Undergraduate Scholarship</t>
+        </is>
+      </c>
+      <c r="C134" s="3" t="inlineStr">
+        <is>
+          <t>Quant firm program</t>
+        </is>
+      </c>
+      <c r="D134" s="8" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E134" s="4" t="inlineStr">
+        <is>
+          <t>https://www.twosigma.com/undergraduate-students/</t>
+        </is>
+      </c>
+      <c r="F134" s="3" t="inlineStr"/>
+    </row>
+    <row r="135">
+      <c r="A135" s="3" t="inlineStr">
+        <is>
+          <t>You cannot apply (NO)</t>
+        </is>
+      </c>
+      <c r="B135" s="3" t="inlineStr">
+        <is>
+          <t>Two Sigma PhD Fellowship</t>
+        </is>
+      </c>
+      <c r="C135" s="3" t="inlineStr">
+        <is>
+          <t>Quant firm program</t>
+        </is>
+      </c>
+      <c r="D135" s="8" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E135" s="4" t="inlineStr">
+        <is>
+          <t>https://www.twosigma.com/graduate-students/phd-fellowships/</t>
+        </is>
+      </c>
+      <c r="F135" s="3" t="inlineStr"/>
+    </row>
+    <row r="136">
+      <c r="A136" s="3" t="inlineStr">
+        <is>
+          <t>You cannot apply (NO)</t>
+        </is>
+      </c>
+      <c r="B136" s="3" t="inlineStr">
+        <is>
+          <t>Virtu Financial Women's Winternship</t>
+        </is>
+      </c>
+      <c r="C136" s="3" t="inlineStr">
+        <is>
+          <t>Quant firm program</t>
+        </is>
+      </c>
+      <c r="D136" s="8" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E136" s="4" t="inlineStr">
+        <is>
+          <t>https://www.virtu.com/careers/</t>
+        </is>
+      </c>
+      <c r="F136" s="3" t="inlineStr"/>
+    </row>
+    <row r="137">
+      <c r="A137" s="3" t="inlineStr">
+        <is>
+          <t>You cannot apply (NO)</t>
+        </is>
+      </c>
+      <c r="B137" s="3" t="inlineStr">
+        <is>
+          <t>Wharton Global High School Investment Competition</t>
+        </is>
+      </c>
+      <c r="C137" s="3" t="inlineStr">
+        <is>
+          <t>Competition</t>
+        </is>
+      </c>
+      <c r="D137" s="8" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E137" s="4" t="inlineStr">
+        <is>
+          <t>https://globalyouth.wharton.upenn.edu/competitions/investment-competition</t>
+        </is>
+      </c>
+      <c r="F137" s="3" t="inlineStr">
+        <is>
+          <t>Ruled out on stage - high school students only. Christina Qi's 2026 quant competitions &amp; events list (LinkedIn Pulse), read 2026-09-06.</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="3" t="inlineStr">
+        <is>
+          <t>You cannot apply (NO)</t>
+        </is>
+      </c>
+      <c r="B138" s="3" t="inlineStr">
+        <is>
+          <t>Women in Quantitative Finance Americas Conference</t>
+        </is>
+      </c>
+      <c r="C138" s="3" t="inlineStr">
+        <is>
+          <t>Conference / other</t>
+        </is>
+      </c>
+      <c r="D138" s="8" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E138" s="4" t="inlineStr">
+        <is>
+          <t>https://www.wbstraining.com/events/wqfa</t>
+        </is>
+      </c>
+      <c r="F138" s="3" t="inlineStr">
+        <is>
+          <t>Ruled out by an identity gate: this program is for women. Christina Qi's 2026 quant competitions &amp; events list (LinkedIn Pulse), read 2026-09-06. Listed here so it is not re-researched.</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="3" t="inlineStr">
+        <is>
+          <t>You cannot apply (NO)</t>
+        </is>
+      </c>
+      <c r="B139" s="3" t="inlineStr">
+        <is>
+          <t>Women in Quantitative Finance London Conference</t>
+        </is>
+      </c>
+      <c r="C139" s="3" t="inlineStr">
+        <is>
+          <t>Conference / other</t>
+        </is>
+      </c>
+      <c r="D139" s="8" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E139" s="4" t="inlineStr">
+        <is>
+          <t>https://www.wbstraining.com/events/london-wqf-conference</t>
+        </is>
+      </c>
+      <c r="F139" s="3" t="inlineStr">
+        <is>
+          <t>Ruled out by an identity gate: this program is for women. Christina Qi's 2026 quant competitions &amp; events list (LinkedIn Pulse), read 2026-09-06. Listed here so it is not re-researched.</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="3" t="inlineStr">
+        <is>
           <t>You cannot apply (STALE)</t>
         </is>
       </c>
-      <c r="B131" s="3" t="inlineStr">
+      <c r="B140" s="3" t="inlineStr">
         <is>
           <t>zapplyjobs underclassmen-internships</t>
         </is>
       </c>
-      <c r="C131" s="3" t="inlineStr">
+      <c r="C140" s="3" t="inlineStr">
         <is>
           <t>Tracker / resource</t>
         </is>
       </c>
-      <c r="D131" s="8" t="inlineStr">
+      <c r="D140" s="8" t="inlineStr">
         <is>
           <t>STALE</t>
         </is>
       </c>
-      <c r="E131" s="4" t="inlineStr">
+      <c r="E140" s="4" t="inlineStr">
         <is>
           <t>https://github.com/zapplyjobs/underclassmen-internships</t>
         </is>
       </c>
-      <c r="F131" s="3" t="inlineStr">
+      <c r="F140" s="3" t="inlineStr">
         <is>
           <t>Right shape, but entries and links are out of date.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F131"/>
+  <autoFilter ref="A1:F140"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId2"/>
@@ -16184,20 +16574,29 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E113" r:id="rId112"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E114" r:id="rId113"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E115" r:id="rId114"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E117" r:id="rId115"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E118" r:id="rId116"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E119" r:id="rId117"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E120" r:id="rId118"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E122" r:id="rId119"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E123" r:id="rId120"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E124" r:id="rId121"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E125" r:id="rId122"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E126" r:id="rId123"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E127" r:id="rId124"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E128" r:id="rId125"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E129" r:id="rId126"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E130" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E116" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E117" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E118" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E119" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E120" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E121" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E122" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E123" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E124" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E126" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E127" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E128" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E129" r:id="rId127"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E131" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E132" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E133" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E134" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E135" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E136" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E137" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E138" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E139" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E140" r:id="rId137"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>